<commit_message>
auto: 2026-06-17 14:48 (3件)
</commit_message>
<xml_diff>
--- a/01_プロジェクト/YouTube/創作スレ下書き/2026-06-17_平将門の祟り_台本.xlsx
+++ b/01_プロジェクト/YouTube/創作スレ下書き/2026-06-17_平将門の祟り_台本.xlsx
@@ -434,7 +434,7 @@
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="70" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
     <col width="6" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
@@ -917,8 +917,9 @@
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>関東大震災のあと、首塚の跡地に建てられた
-大蔵省の仮庁舎では、</t>
+          <t>大蔵省仮庁舎の祟りとは、
+関東大震災のあと、首塚の跡地に建てられた
+大蔵省の仮庁舎で相次いだ不審な出来事を指す。</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
@@ -940,9 +941,10 @@
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>工事の関係者や省の職員が相次いで体調を崩し、
+          <t>工事の関係者や省の職員が次々と体調を崩し、
 当時の大蔵大臣・早速整爾までもが
-在任中に亡くなっている。</t>
+在任中に亡くなったことで、
+将門の祟りだと省内で噂された。</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
@@ -964,9 +966,8 @@
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>これらの不幸が将門の祟りだと省内で噂され、
-国はわざわざ建てた仮庁舎を取り壊して、
-跡地に鎮魂の碑を建てた。</t>
+          <t>国はわざわざ建てた仮庁舎を取り壊し、
+跡地に鎮魂の碑を建てている。</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
@@ -988,8 +989,7 @@
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>国家機関が一度建てた庁舎を、
-祟りを理由に解体したという、
+          <t>国家機関が一度建てた庁舎を祟りを理由に解体した、
 極めて異例の出来事として語り継がれている。</t>
         </is>
       </c>
@@ -2141,7 +2141,7 @@
       </c>
       <c r="B77" s="3" t="inlineStr">
         <is>
-          <t>新皇名乗って関東独立しようとしたやべえ奴やぞ。そこは詳しいニキ任せたわ、ワイ飯食ってくる</t>
+          <t>新皇名乗って関東独立しようとしたやべえ奴やぞ</t>
         </is>
       </c>
       <c r="C77" s="2" t="inlineStr">

</xml_diff>

<commit_message>
auto: 2026-06-17 15:08 (4件)
</commit_message>
<xml_diff>
--- a/01_プロジェクト/YouTube/創作スレ下書き/2026-06-17_平将門の祟り_台本.xlsx
+++ b/01_プロジェクト/YouTube/創作スレ下書き/2026-06-17_平将門の祟り_台本.xlsx
@@ -604,7 +604,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>スレタイ</t>
+          <t>男性A</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
@@ -626,7 +626,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>男性A</t>
+          <t>女性B下</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -648,7 +648,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>女性B</t>
+          <t>男性C</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
@@ -670,7 +670,7 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>男性C</t>
+          <t>女性D</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -692,7 +692,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>女性D</t>
+          <t>男性E</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
@@ -714,7 +714,7 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>男性E</t>
+          <t>男性A</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -736,7 +736,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>男性A</t>
+          <t>女性B</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
@@ -758,7 +758,7 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>女性B大</t>
+          <t>男性C大</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -780,7 +780,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>男性C</t>
+          <t>女性D</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
@@ -802,7 +802,7 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>女性D</t>
+          <t>男性E</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
@@ -824,7 +824,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>男性E下</t>
+          <t>男性A下</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
@@ -846,7 +846,7 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>男性A</t>
+          <t>女性B</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
@@ -868,7 +868,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>女性B下</t>
+          <t>男性C下</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
@@ -890,7 +890,7 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>男性C</t>
+          <t>女性D</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
@@ -1007,7 +1007,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>女性D</t>
+          <t>男性E</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
@@ -1029,7 +1029,7 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>男性E下</t>
+          <t>男性A下</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
@@ -1051,7 +1051,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>男性A</t>
+          <t>女性B</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
@@ -1073,7 +1073,7 @@
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>女性B大</t>
+          <t>男性C大</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
@@ -1095,7 +1095,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>男性C下</t>
+          <t>女性D下</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">
@@ -1117,7 +1117,7 @@
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>女性D</t>
+          <t>男性E</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
@@ -1139,7 +1139,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>男性E</t>
+          <t>男性A</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr">
@@ -1161,7 +1161,7 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>男性A下</t>
+          <t>女性B下</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
@@ -1183,7 +1183,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>女性B</t>
+          <t>男性C</t>
         </is>
       </c>
       <c r="B34" s="3" t="inlineStr">
@@ -1205,7 +1205,7 @@
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>男性C下</t>
+          <t>女性D下</t>
         </is>
       </c>
       <c r="B35" s="3" t="inlineStr">
@@ -1227,7 +1227,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>女性D</t>
+          <t>男性E</t>
         </is>
       </c>
       <c r="B36" s="3" t="inlineStr">
@@ -1344,7 +1344,7 @@
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>男性E大</t>
+          <t>男性A大</t>
         </is>
       </c>
       <c r="B41" s="3" t="inlineStr">
@@ -1366,7 +1366,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>男性A</t>
+          <t>女性B</t>
         </is>
       </c>
       <c r="B42" s="3" t="inlineStr">
@@ -1388,7 +1388,7 @@
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>女性B</t>
+          <t>男性C</t>
         </is>
       </c>
       <c r="B43" s="3" t="inlineStr">
@@ -1410,7 +1410,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>男性C大</t>
+          <t>女性D大</t>
         </is>
       </c>
       <c r="B44" s="3" t="inlineStr">
@@ -1432,7 +1432,7 @@
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>女性D</t>
+          <t>男性E</t>
         </is>
       </c>
       <c r="B45" s="3" t="inlineStr">
@@ -1454,7 +1454,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>男性E</t>
+          <t>男性A</t>
         </is>
       </c>
       <c r="B46" s="3" t="inlineStr">
@@ -1476,7 +1476,7 @@
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>男性A下</t>
+          <t>女性B下</t>
         </is>
       </c>
       <c r="B47" s="3" t="inlineStr">
@@ -1498,7 +1498,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>女性B大</t>
+          <t>男性C大</t>
         </is>
       </c>
       <c r="B48" s="3" t="inlineStr">
@@ -1520,7 +1520,7 @@
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>男性C</t>
+          <t>女性D</t>
         </is>
       </c>
       <c r="B49" s="3" t="inlineStr">
@@ -1542,7 +1542,7 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>女性D</t>
+          <t>男性E</t>
         </is>
       </c>
       <c r="B50" s="3" t="inlineStr">
@@ -1564,7 +1564,7 @@
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>男性E下</t>
+          <t>男性A下</t>
         </is>
       </c>
       <c r="B51" s="3" t="inlineStr">
@@ -1586,7 +1586,7 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>男性A</t>
+          <t>女性B</t>
         </is>
       </c>
       <c r="B52" s="3" t="inlineStr">
@@ -1608,7 +1608,7 @@
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>女性B</t>
+          <t>男性C</t>
         </is>
       </c>
       <c r="B53" s="3" t="inlineStr">
@@ -1630,7 +1630,7 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>男性C</t>
+          <t>女性D</t>
         </is>
       </c>
       <c r="B54" s="3" t="inlineStr">
@@ -1652,7 +1652,7 @@
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>女性D</t>
+          <t>男性E</t>
         </is>
       </c>
       <c r="B55" s="3" t="inlineStr">
@@ -1674,7 +1674,7 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>男性E大</t>
+          <t>男性A大</t>
         </is>
       </c>
       <c r="B56" s="3" t="inlineStr">
@@ -1696,7 +1696,7 @@
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>男性A</t>
+          <t>女性B</t>
         </is>
       </c>
       <c r="B57" s="3" t="inlineStr">
@@ -1718,7 +1718,7 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>女性B大</t>
+          <t>男性C大</t>
         </is>
       </c>
       <c r="B58" s="3" t="inlineStr">
@@ -1740,7 +1740,7 @@
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>男性C</t>
+          <t>女性D</t>
         </is>
       </c>
       <c r="B59" s="3" t="inlineStr">
@@ -1762,7 +1762,7 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>女性D下</t>
+          <t>男性E下</t>
         </is>
       </c>
       <c r="B60" s="3" t="inlineStr">
@@ -1784,7 +1784,7 @@
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>男性E</t>
+          <t>男性A</t>
         </is>
       </c>
       <c r="B61" s="3" t="inlineStr">
@@ -1806,7 +1806,7 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>男性A</t>
+          <t>女性B</t>
         </is>
       </c>
       <c r="B62" s="3" t="inlineStr">
@@ -1828,7 +1828,7 @@
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>女性B下</t>
+          <t>男性C下</t>
         </is>
       </c>
       <c r="B63" s="3" t="inlineStr">
@@ -1850,7 +1850,7 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>男性C</t>
+          <t>女性D</t>
         </is>
       </c>
       <c r="B64" s="3" t="inlineStr">
@@ -1872,7 +1872,7 @@
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>女性D</t>
+          <t>男性E</t>
         </is>
       </c>
       <c r="B65" s="3" t="inlineStr">
@@ -1894,7 +1894,7 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>男性E大</t>
+          <t>男性A大</t>
         </is>
       </c>
       <c r="B66" s="3" t="inlineStr">
@@ -1916,7 +1916,7 @@
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>男性A下</t>
+          <t>女性B下</t>
         </is>
       </c>
       <c r="B67" s="3" t="inlineStr">
@@ -1938,7 +1938,7 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>女性B</t>
+          <t>男性C</t>
         </is>
       </c>
       <c r="B68" s="3" t="inlineStr">
@@ -1960,7 +1960,7 @@
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>男性C</t>
+          <t>女性D</t>
         </is>
       </c>
       <c r="B69" s="3" t="inlineStr">
@@ -1982,7 +1982,7 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>女性D下</t>
+          <t>男性E下</t>
         </is>
       </c>
       <c r="B70" s="3" t="inlineStr">
@@ -2004,7 +2004,7 @@
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>男性E</t>
+          <t>男性A</t>
         </is>
       </c>
       <c r="B71" s="3" t="inlineStr">
@@ -2026,7 +2026,7 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>男性A下</t>
+          <t>女性B下</t>
         </is>
       </c>
       <c r="B72" s="3" t="inlineStr">
@@ -2048,7 +2048,7 @@
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
         <is>
-          <t>女性B</t>
+          <t>男性C</t>
         </is>
       </c>
       <c r="B73" s="3" t="inlineStr">
@@ -2070,7 +2070,7 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>男性C</t>
+          <t>女性D</t>
         </is>
       </c>
       <c r="B74" s="3" t="inlineStr">
@@ -2092,7 +2092,7 @@
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
         <is>
-          <t>女性D</t>
+          <t>男性E</t>
         </is>
       </c>
       <c r="B75" s="3" t="inlineStr">
@@ -2114,7 +2114,7 @@
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>男性E</t>
+          <t>男性A</t>
         </is>
       </c>
       <c r="B76" s="3" t="inlineStr">
@@ -2136,7 +2136,7 @@
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
         <is>
-          <t>男性A</t>
+          <t>女性B</t>
         </is>
       </c>
       <c r="B77" s="3" t="inlineStr">
@@ -2252,7 +2252,7 @@
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>スレタイ</t>
+          <t>男性A</t>
         </is>
       </c>
       <c r="B82" s="3" t="inlineStr">
@@ -2274,7 +2274,7 @@
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
         <is>
-          <t>男性A</t>
+          <t>女性B下</t>
         </is>
       </c>
       <c r="B83" s="3" t="inlineStr">
@@ -2296,7 +2296,7 @@
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>女性B</t>
+          <t>男性C</t>
         </is>
       </c>
       <c r="B84" s="3" t="inlineStr">
@@ -2318,7 +2318,7 @@
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
         <is>
-          <t>男性C</t>
+          <t>女性D</t>
         </is>
       </c>
       <c r="B85" s="3" t="inlineStr">
@@ -2340,7 +2340,7 @@
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>女性D</t>
+          <t>男性E</t>
         </is>
       </c>
       <c r="B86" s="3" t="inlineStr">
@@ -2362,7 +2362,7 @@
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
         <is>
-          <t>男性E</t>
+          <t>男性A</t>
         </is>
       </c>
       <c r="B87" s="3" t="inlineStr">
@@ -2384,7 +2384,7 @@
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>男性A</t>
+          <t>女性B</t>
         </is>
       </c>
       <c r="B88" s="3" t="inlineStr">
@@ -2406,7 +2406,7 @@
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
         <is>
-          <t>女性B大</t>
+          <t>男性C大</t>
         </is>
       </c>
       <c r="B89" s="3" t="inlineStr">
@@ -2428,7 +2428,7 @@
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>男性C</t>
+          <t>女性D</t>
         </is>
       </c>
       <c r="B90" s="3" t="inlineStr">
@@ -2450,7 +2450,7 @@
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
         <is>
-          <t>女性D</t>
+          <t>男性E</t>
         </is>
       </c>
       <c r="B91" s="3" t="inlineStr">
@@ -2472,7 +2472,7 @@
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>男性E下</t>
+          <t>男性A下</t>
         </is>
       </c>
       <c r="B92" s="3" t="inlineStr">
@@ -2494,7 +2494,7 @@
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
         <is>
-          <t>男性A大</t>
+          <t>女性B大</t>
         </is>
       </c>
       <c r="B93" s="3" t="inlineStr">
@@ -2516,7 +2516,7 @@
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>女性B</t>
+          <t>男性C</t>
         </is>
       </c>
       <c r="B94" s="3" t="inlineStr">
@@ -2538,7 +2538,7 @@
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
         <is>
-          <t>男性C下</t>
+          <t>女性D下</t>
         </is>
       </c>
       <c r="B95" s="3" t="inlineStr">
@@ -2560,7 +2560,7 @@
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>女性D大</t>
+          <t>男性E大</t>
         </is>
       </c>
       <c r="B96" s="3" t="inlineStr">
@@ -2582,7 +2582,7 @@
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
         <is>
-          <t>男性E</t>
+          <t>男性A</t>
         </is>
       </c>
       <c r="B97" s="3" t="inlineStr">
@@ -2604,7 +2604,7 @@
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>男性A下</t>
+          <t>女性B下</t>
         </is>
       </c>
       <c r="B98" s="3" t="inlineStr">
@@ -2722,7 +2722,7 @@
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
         <is>
-          <t>女性B大</t>
+          <t>男性C大</t>
         </is>
       </c>
       <c r="B103" s="3" t="inlineStr">
@@ -2744,7 +2744,7 @@
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
         <is>
-          <t>男性C下</t>
+          <t>女性D下</t>
         </is>
       </c>
       <c r="B104" s="3" t="inlineStr">
@@ -2766,7 +2766,7 @@
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
         <is>
-          <t>女性D</t>
+          <t>男性E</t>
         </is>
       </c>
       <c r="B105" s="3" t="inlineStr">
@@ -2788,7 +2788,7 @@
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
         <is>
-          <t>男性E</t>
+          <t>男性A</t>
         </is>
       </c>
       <c r="B106" s="3" t="inlineStr">
@@ -2810,7 +2810,7 @@
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
         <is>
-          <t>男性A大</t>
+          <t>女性B大</t>
         </is>
       </c>
       <c r="B107" s="3" t="inlineStr">
@@ -2832,7 +2832,7 @@
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
         <is>
-          <t>女性B</t>
+          <t>男性C</t>
         </is>
       </c>
       <c r="B108" s="3" t="inlineStr">
@@ -2854,7 +2854,7 @@
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
         <is>
-          <t>男性C</t>
+          <t>女性D</t>
         </is>
       </c>
       <c r="B109" s="3" t="inlineStr">
@@ -2876,7 +2876,7 @@
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
         <is>
-          <t>女性D</t>
+          <t>男性E</t>
         </is>
       </c>
       <c r="B110" s="3" t="inlineStr">
@@ -2898,7 +2898,7 @@
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
         <is>
-          <t>男性E下</t>
+          <t>男性A下</t>
         </is>
       </c>
       <c r="B111" s="3" t="inlineStr">
@@ -2920,7 +2920,7 @@
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
         <is>
-          <t>男性A</t>
+          <t>女性B</t>
         </is>
       </c>
       <c r="B112" s="3" t="inlineStr">
@@ -2942,7 +2942,7 @@
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
         <is>
-          <t>女性B大</t>
+          <t>男性C大</t>
         </is>
       </c>
       <c r="B113" s="3" t="inlineStr">
@@ -2964,7 +2964,7 @@
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
         <is>
-          <t>男性C下</t>
+          <t>女性D下</t>
         </is>
       </c>
       <c r="B114" s="3" t="inlineStr">
@@ -2986,7 +2986,7 @@
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
         <is>
-          <t>女性D</t>
+          <t>男性E</t>
         </is>
       </c>
       <c r="B115" s="3" t="inlineStr">
@@ -3008,7 +3008,7 @@
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
         <is>
-          <t>男性E</t>
+          <t>男性A</t>
         </is>
       </c>
       <c r="B116" s="3" t="inlineStr">
@@ -3030,7 +3030,7 @@
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
         <is>
-          <t>男性A下</t>
+          <t>女性B下</t>
         </is>
       </c>
       <c r="B117" s="3" t="inlineStr">
@@ -3052,7 +3052,7 @@
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
         <is>
-          <t>女性B</t>
+          <t>男性C</t>
         </is>
       </c>
       <c r="B118" s="3" t="inlineStr">
@@ -3074,7 +3074,7 @@
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
         <is>
-          <t>男性C大</t>
+          <t>女性D大</t>
         </is>
       </c>
       <c r="B119" s="3" t="inlineStr">
@@ -3096,7 +3096,7 @@
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
         <is>
-          <t>女性D</t>
+          <t>男性E</t>
         </is>
       </c>
       <c r="B120" s="3" t="inlineStr">
@@ -3118,7 +3118,7 @@
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
         <is>
-          <t>男性E</t>
+          <t>男性A</t>
         </is>
       </c>
       <c r="B121" s="3" t="inlineStr">
@@ -3140,7 +3140,7 @@
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
         <is>
-          <t>男性A大</t>
+          <t>女性B大</t>
         </is>
       </c>
       <c r="B122" s="3" t="inlineStr">
@@ -3162,7 +3162,7 @@
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
         <is>
-          <t>女性B下</t>
+          <t>男性C下</t>
         </is>
       </c>
       <c r="B123" s="3" t="inlineStr">
@@ -3184,7 +3184,7 @@
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
         <is>
-          <t>男性C</t>
+          <t>女性D</t>
         </is>
       </c>
       <c r="B124" s="3" t="inlineStr">
@@ -3206,7 +3206,7 @@
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
         <is>
-          <t>女性D大</t>
+          <t>男性E大</t>
         </is>
       </c>
       <c r="B125" s="3" t="inlineStr">
@@ -3228,7 +3228,7 @@
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
         <is>
-          <t>男性E</t>
+          <t>男性A</t>
         </is>
       </c>
       <c r="B126" s="3" t="inlineStr">
@@ -3250,7 +3250,7 @@
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
         <is>
-          <t>男性A</t>
+          <t>女性B</t>
         </is>
       </c>
       <c r="B127" s="3" t="inlineStr">
@@ -3272,7 +3272,7 @@
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
         <is>
-          <t>女性B</t>
+          <t>男性C</t>
         </is>
       </c>
       <c r="B128" s="3" t="inlineStr">
@@ -3294,7 +3294,7 @@
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
         <is>
-          <t>男性C</t>
+          <t>女性D</t>
         </is>
       </c>
       <c r="B129" s="3" t="inlineStr">
@@ -3316,7 +3316,7 @@
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
         <is>
-          <t>女性D</t>
+          <t>男性E</t>
         </is>
       </c>
       <c r="B130" s="3" t="inlineStr">
@@ -3338,7 +3338,7 @@
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
         <is>
-          <t>男性E大</t>
+          <t>男性A大</t>
         </is>
       </c>
       <c r="B131" s="3" t="inlineStr">
@@ -3360,7 +3360,7 @@
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
         <is>
-          <t>男性A</t>
+          <t>女性B</t>
         </is>
       </c>
       <c r="B132" s="3" t="inlineStr">
@@ -3382,7 +3382,7 @@
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
         <is>
-          <t>女性B下</t>
+          <t>男性C下</t>
         </is>
       </c>
       <c r="B133" s="3" t="inlineStr">
@@ -3404,7 +3404,7 @@
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
         <is>
-          <t>男性C</t>
+          <t>女性D</t>
         </is>
       </c>
       <c r="B134" s="3" t="inlineStr">
@@ -3426,7 +3426,7 @@
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
         <is>
-          <t>女性D下</t>
+          <t>男性E下</t>
         </is>
       </c>
       <c r="B135" s="3" t="inlineStr">
@@ -3448,7 +3448,7 @@
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
         <is>
-          <t>男性E</t>
+          <t>男性A</t>
         </is>
       </c>
       <c r="B136" s="3" t="inlineStr">
@@ -3470,7 +3470,7 @@
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
         <is>
-          <t>男性A下</t>
+          <t>女性B下</t>
         </is>
       </c>
       <c r="B137" s="3" t="inlineStr">
@@ -3587,7 +3587,7 @@
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
         <is>
-          <t>女性B</t>
+          <t>男性C</t>
         </is>
       </c>
       <c r="B142" s="3" t="inlineStr">
@@ -3609,7 +3609,7 @@
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
         <is>
-          <t>男性C大</t>
+          <t>女性D大</t>
         </is>
       </c>
       <c r="B143" s="3" t="inlineStr">
@@ -3631,7 +3631,7 @@
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
         <is>
-          <t>女性D下</t>
+          <t>男性E下</t>
         </is>
       </c>
       <c r="B144" s="3" t="inlineStr">
@@ -3653,7 +3653,7 @@
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
         <is>
-          <t>男性E</t>
+          <t>男性A</t>
         </is>
       </c>
       <c r="B145" s="3" t="inlineStr">
@@ -3675,7 +3675,7 @@
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
         <is>
-          <t>男性A</t>
+          <t>女性B</t>
         </is>
       </c>
       <c r="B146" s="3" t="inlineStr">
@@ -3697,7 +3697,7 @@
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
         <is>
-          <t>女性B</t>
+          <t>男性C</t>
         </is>
       </c>
       <c r="B147" s="3" t="inlineStr">
@@ -3719,7 +3719,7 @@
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
         <is>
-          <t>男性C下</t>
+          <t>女性D下</t>
         </is>
       </c>
       <c r="B148" s="3" t="inlineStr">
@@ -3741,7 +3741,7 @@
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
         <is>
-          <t>女性D</t>
+          <t>男性E</t>
         </is>
       </c>
       <c r="B149" s="3" t="inlineStr">

</xml_diff>

<commit_message>
auto: 2026-06-17 16:08 (5件)
</commit_message>
<xml_diff>
--- a/01_プロジェクト/YouTube/創作スレ下書き/2026-06-17_平将門の祟り_台本.xlsx
+++ b/01_プロジェクト/YouTube/創作スレ下書き/2026-06-17_平将門の祟り_台本.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D155"/>
+  <dimension ref="A1:D166"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1366,7 +1366,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>女性B</t>
+          <t>女性B下</t>
         </is>
       </c>
       <c r="B42" s="3" t="inlineStr">
@@ -1718,12 +1718,12 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>男性C大</t>
+          <t>男性C</t>
         </is>
       </c>
       <c r="B58" s="3" t="inlineStr">
         <is>
-          <t>これ豆な、将門は今や神田明神の祭神になっとって、崇徳上皇・菅原道真と並んで日本三大怨霊に数えられとる。面白いのが、徳川が江戸入りしたとき将門を江戸の守り神として篤く祀り直しとるんよ。怒らせたら祟るけど、ちゃんと祀れば街を守ってくれる、っていう道真の天神さんと同じ"祟り神の出世コース"に乗っとるわけや。その道真なんか今や学問の神様で、受験シーズンに全国の受験生が手を合わせに行くレベルやからな。恐れられた怨霊ほど後世の祀られ方が手厚なる、ってのが日本の不思議なとこやで</t>
+          <t>ワイ去年あの辺で働いとったとき、毎朝コンビニ寄る感覚で手だけ合わせて通勤しとったわ</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
@@ -1740,12 +1740,12 @@
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>女性D</t>
+          <t>女性D下</t>
         </is>
       </c>
       <c r="B59" s="3" t="inlineStr">
         <is>
-          <t>祟り神が守り神に出世しとるの草</t>
+          <t>それ完全にご近所の氏神様やん</t>
         </is>
       </c>
       <c r="C59" s="2" t="inlineStr">
@@ -1762,12 +1762,12 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>男性E下</t>
+          <t>男性E</t>
         </is>
       </c>
       <c r="B60" s="3" t="inlineStr">
         <is>
-          <t>メガテン勢からすると将門公はガチで畏れる対象や。アトラスが将門モチーフにしたら開発中トラブル続きで、表記を「マサカドこう」に直したら止んだって都市伝説あるやろ</t>
+          <t>カエルの置物いっぱい置いてあるよな、無事カエルでって。最初なんの土産物屋かと思った</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
@@ -1789,7 +1789,7 @@
       </c>
       <c r="B61" s="3" t="inlineStr">
         <is>
-          <t>ゲーム会社にまで祟るのやめたれや</t>
+          <t>で、結局三大怨霊って残り誰なん</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr">
@@ -1806,12 +1806,12 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>女性B</t>
+          <t>女性B下大</t>
         </is>
       </c>
       <c r="B62" s="3" t="inlineStr">
         <is>
-          <t>そこは祟りやのうて納期やろ</t>
+          <t>これ豆な、将門は今や神田明神の祭神になっとって、崇徳上皇・菅原道真と並んで日本三大怨霊に数えられとる。面白いのが、徳川が江戸入りしたとき将門を江戸の総鎮守として篤く祀り直しとるんよ。怒らせたら祟るけど、ちゃんと祀れば街を守ってくれる、っていう"祟り神の出世コース"に乗っとるわけや</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
@@ -1828,12 +1828,12 @@
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>男性C下</t>
+          <t>男性C</t>
         </is>
       </c>
       <c r="B63" s="3" t="inlineStr">
         <is>
-          <t>不覚にも笑った</t>
+          <t>祟り神が守り神に出世しとるの草</t>
         </is>
       </c>
       <c r="C63" s="2" t="inlineStr">
@@ -1850,12 +1850,12 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>女性D</t>
+          <t>女性D大</t>
         </is>
       </c>
       <c r="B64" s="3" t="inlineStr">
         <is>
-          <t>太田光が売れる前に首塚にドロップキックかまして、しばらく仕事来んくなったって噂もあるな</t>
+          <t>その道真なんか今や学問の神様で、受験シーズンに全国の受験生が手を合わせに行くレベルやからな。恐れられた怨霊ほど後世の祀られ方が手厚なる、っていうのが日本のおもろい癖やねん。最初は災いの元として恐れられた連中が、丁重に祀られて街や受験生を守る側に回る。将門もその王道を歩んどるわけや</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
@@ -1877,7 +1877,7 @@
       </c>
       <c r="B65" s="3" t="inlineStr">
         <is>
-          <t>それはさすがに芸人の自業自得では</t>
+          <t>落とし所が神様って発想、日本ぐらいやろ</t>
         </is>
       </c>
       <c r="C65" s="2" t="inlineStr">
@@ -1894,12 +1894,12 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>男性A大</t>
+          <t>男性A下</t>
         </is>
       </c>
       <c r="B66" s="3" t="inlineStr">
         <is>
-          <t>ここ大事なんやけど、将門はただ恐れられただけちゃうくて、もともとは関東の民にとっては英雄寄りの存在やったんよ。重い負担やら国府の横暴に苦しむ坂東の人らからしたら、中央に盾突いて「東は俺らで治める」ってやってのけた将門は反骨のシンボルやった。だからこそ討たれたあとも、祟り神として畏れられつつ土地の守り神として手厚く祀られ続けた、っていう二面性があるわけや</t>
+          <t>メガテン勢からすると将門公はガチで畏れる対象や。アトラスが将門モチーフにしたら開発中トラブル続きで、表記を「マサカドこう」に直したら止んだって都市伝説あるやろ</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr">
@@ -1916,12 +1916,12 @@
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>女性B下</t>
+          <t>女性B</t>
         </is>
       </c>
       <c r="B67" s="3" t="inlineStr">
         <is>
-          <t>ただの怨霊ちゃうくて元はヒーローなんやな</t>
+          <t>ゲーム会社にまで祟るのやめたれや</t>
         </is>
       </c>
       <c r="C67" s="2" t="inlineStr">
@@ -1943,7 +1943,7 @@
       </c>
       <c r="B68" s="3" t="inlineStr">
         <is>
-          <t>結局さ、全部"そういうことにしとこ"の後付けやろ。因果の証拠なんか無いやん</t>
+          <t>そこは祟りやのうて納期やろ</t>
         </is>
       </c>
       <c r="C68" s="2" t="inlineStr">
@@ -1960,12 +1960,12 @@
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>女性D</t>
+          <t>女性D下</t>
         </is>
       </c>
       <c r="B69" s="3" t="inlineStr">
         <is>
-          <t>信者乙、ぜんぶ偶然や</t>
+          <t>不覚にも笑った</t>
         </is>
       </c>
       <c r="C69" s="2" t="inlineStr">
@@ -1982,12 +1982,12 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>男性E下</t>
+          <t>男性E</t>
         </is>
       </c>
       <c r="B70" s="3" t="inlineStr">
         <is>
-          <t>まあ祟りに証拠もへったくれもないわな、そこは認める</t>
+          <t>太田光が売れる前に首塚にドロップキックかまして、しばらく仕事来んくなったって噂もあるな</t>
         </is>
       </c>
       <c r="C70" s="2" t="inlineStr">
@@ -2009,7 +2009,7 @@
       </c>
       <c r="B71" s="3" t="inlineStr">
         <is>
-          <t>証拠ないのに国家プロジェクトが二回もどかすのやめてる時点で、もう実質勝ちなんよ将門</t>
+          <t>それはさすがに芸人の自業自得では</t>
         </is>
       </c>
       <c r="C71" s="2" t="inlineStr">
@@ -2026,12 +2026,12 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>女性B下</t>
+          <t>女性B大</t>
         </is>
       </c>
       <c r="B72" s="3" t="inlineStr">
         <is>
-          <t>勝ち負けの話になってて草</t>
+          <t>ここ大事なんやけど、将門はただ恐れられただけちゃうくて、もともとは関東の民にとっては英雄寄りの存在やったんよ。重い負担やら国府の横暴に苦しむ坂東の人らからしたら、中央に盾突いて「東は俺らで治める」ってやってのけた将門は反骨のシンボルやった。だからこそ討たれたあとも、祟り神として畏れられつつ土地の守り神として手厚く祀られ続けた、っていう二面性があるわけや</t>
         </is>
       </c>
       <c r="C72" s="2" t="inlineStr">
@@ -2048,12 +2048,12 @@
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
         <is>
-          <t>男性C</t>
+          <t>男性C下</t>
         </is>
       </c>
       <c r="B73" s="3" t="inlineStr">
         <is>
-          <t>山手線が将門の祟りを抑える結界として作られたって都市伝説もあるよな</t>
+          <t>ただの怨霊ちゃうくて元はヒーローなんやな</t>
         </is>
       </c>
       <c r="C73" s="2" t="inlineStr">
@@ -2075,7 +2075,7 @@
       </c>
       <c r="B74" s="3" t="inlineStr">
         <is>
-          <t>それは嘘らしいで、結界説は後から誰かが言い出したやつや</t>
+          <t>結局さ、全部"そういうことにしとこ"の後付けやろ。因果の証拠なんか無いやん</t>
         </is>
       </c>
       <c r="C74" s="2" t="inlineStr">
@@ -2097,7 +2097,7 @@
       </c>
       <c r="B75" s="3" t="inlineStr">
         <is>
-          <t>なんや嘘なんか</t>
+          <t>信者乙、ぜんぶ偶然や</t>
         </is>
       </c>
       <c r="C75" s="2" t="inlineStr">
@@ -2114,12 +2114,12 @@
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>男性A</t>
+          <t>男性A下</t>
         </is>
       </c>
       <c r="B76" s="3" t="inlineStr">
         <is>
-          <t>嘘か本当か分からんのが一番こわいんよこの人。で、そもそも将門ってなんで反乱なんか起こしたん？怨霊の部分しか知らんわ</t>
+          <t>まあ祟りに証拠もへったくれもないわな、そこは認める</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
@@ -2141,7 +2141,7 @@
       </c>
       <c r="B77" s="3" t="inlineStr">
         <is>
-          <t>新皇名乗って関東独立しようとしたやべえ奴やぞ</t>
+          <t>証拠ないのに国家プロジェクトが二回もどかすのやめてる時点で、もう実質勝ちなんよ将門</t>
         </is>
       </c>
       <c r="C77" s="2" t="inlineStr">
@@ -2158,238 +2158,238 @@
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
+          <t>男性C下</t>
+        </is>
+      </c>
+      <c r="B78" s="3" t="inlineStr">
+        <is>
+          <t>勝ち負けの話になってて草</t>
+        </is>
+      </c>
+      <c r="C78" s="2" t="inlineStr">
+        <is>
+          <t>スレ①</t>
+        </is>
+      </c>
+      <c r="D78" s="2" t="inlineStr">
+        <is>
+          <t>63</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="inlineStr">
+        <is>
+          <t>女性D</t>
+        </is>
+      </c>
+      <c r="B79" s="3" t="inlineStr">
+        <is>
+          <t>山手線が将門の祟りを抑える結界として作られたって都市伝説もあるよな</t>
+        </is>
+      </c>
+      <c r="C79" s="2" t="inlineStr">
+        <is>
+          <t>スレ①</t>
+        </is>
+      </c>
+      <c r="D79" s="2" t="inlineStr">
+        <is>
+          <t>64</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="inlineStr">
+        <is>
+          <t>男性E</t>
+        </is>
+      </c>
+      <c r="B80" s="3" t="inlineStr">
+        <is>
+          <t>それは嘘らしいで、結界説は後から誰かが言い出したやつや</t>
+        </is>
+      </c>
+      <c r="C80" s="2" t="inlineStr">
+        <is>
+          <t>スレ①</t>
+        </is>
+      </c>
+      <c r="D80" s="2" t="inlineStr">
+        <is>
+          <t>65</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="inlineStr">
+        <is>
+          <t>男性A</t>
+        </is>
+      </c>
+      <c r="B81" s="3" t="inlineStr">
+        <is>
+          <t>なんや嘘なんか</t>
+        </is>
+      </c>
+      <c r="C81" s="2" t="inlineStr">
+        <is>
+          <t>スレ①</t>
+        </is>
+      </c>
+      <c r="D81" s="2" t="inlineStr">
+        <is>
+          <t>66</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="inlineStr">
+        <is>
+          <t>女性B</t>
+        </is>
+      </c>
+      <c r="B82" s="3" t="inlineStr">
+        <is>
+          <t>嘘か本当か分からんのが一番こわいんよこの人。で、そもそも将門ってなんで反乱なんか起こしたん？怨霊の部分しか知らんわ</t>
+        </is>
+      </c>
+      <c r="C82" s="2" t="inlineStr">
+        <is>
+          <t>スレ①</t>
+        </is>
+      </c>
+      <c r="D82" s="2" t="inlineStr">
+        <is>
+          <t>67</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="inlineStr">
+        <is>
+          <t>男性C</t>
+        </is>
+      </c>
+      <c r="B83" s="3" t="inlineStr">
+        <is>
+          <t>新皇名乗って関東独立しようとしたやべえ奴やぞ</t>
+        </is>
+      </c>
+      <c r="C83" s="2" t="inlineStr">
+        <is>
+          <t>スレ①</t>
+        </is>
+      </c>
+      <c r="D83" s="2" t="inlineStr">
+        <is>
+          <t>68</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="inlineStr">
+        <is>
           <t>解説者</t>
         </is>
       </c>
-      <c r="B78" s="3" t="inlineStr">
+      <c r="B84" s="3" t="inlineStr">
         <is>
           <t>ここまでは、
 平将門の首塚にまつわる祟りの噂について
 さまざまな議論を見てきたが、</t>
         </is>
       </c>
-      <c r="C78" s="2" t="inlineStr">
+      <c r="C84" s="2" t="inlineStr">
         <is>
           <t>前置き</t>
         </is>
       </c>
-      <c r="D78" s="2" t="inlineStr">
+      <c r="D84" s="2" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
     </row>
-    <row r="79">
-      <c r="A79" s="2" t="inlineStr">
+    <row r="85">
+      <c r="A85" s="2" t="inlineStr">
         <is>
           <t>解説者</t>
         </is>
       </c>
-      <c r="B79" s="3" t="inlineStr">
+      <c r="B85" s="3" t="inlineStr">
         <is>
           <t>「そもそも将門は何をして、
 ここまで恐れられる存在になったの？」
 と、肝心の生涯に疑問を持つ者も現れた。</t>
         </is>
       </c>
-      <c r="C79" s="2" t="inlineStr">
+      <c r="C85" s="2" t="inlineStr">
         <is>
           <t>前置き</t>
         </is>
       </c>
-      <c r="D79" s="2" t="inlineStr">
+      <c r="D85" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
     </row>
-    <row r="80">
-      <c r="A80" s="2" t="inlineStr">
+    <row r="86">
+      <c r="A86" s="2" t="inlineStr">
         <is>
           <t>解説者</t>
         </is>
       </c>
-      <c r="B80" s="3" t="inlineStr">
+      <c r="B86" s="3" t="inlineStr">
         <is>
           <t>たしかに、千年も祟りが語り継がれる怨霊が、
 どうやって生まれたのかは気になるところだ。</t>
         </is>
       </c>
-      <c r="C80" s="2" t="inlineStr">
+      <c r="C86" s="2" t="inlineStr">
         <is>
           <t>前置き</t>
         </is>
       </c>
-      <c r="D80" s="2" t="inlineStr">
+      <c r="D86" s="2" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
     </row>
-    <row r="81">
-      <c r="A81" s="2" t="inlineStr">
+    <row r="87">
+      <c r="A87" s="2" t="inlineStr">
         <is>
           <t>解説者</t>
         </is>
       </c>
-      <c r="B81" s="3" t="inlineStr">
+      <c r="B87" s="3" t="inlineStr">
         <is>
           <t>引き続き、2ちゃんねるの歴史オタクたちの
 議論を見ていこう。</t>
         </is>
       </c>
-      <c r="C81" s="2" t="inlineStr">
+      <c r="C87" s="2" t="inlineStr">
         <is>
           <t>前置き</t>
         </is>
       </c>
-      <c r="D81" s="2" t="inlineStr">
+      <c r="D87" s="2" t="inlineStr">
         <is>
           <t>4</t>
-        </is>
-      </c>
-    </row>
-    <row r="82">
-      <c r="A82" s="2" t="inlineStr">
-        <is>
-          <t>男性A</t>
-        </is>
-      </c>
-      <c r="B82" s="3" t="inlineStr">
-        <is>
-          <t>平将門「これからは俺が東の天皇やるわ」朝廷「は？」</t>
-        </is>
-      </c>
-      <c r="C82" s="2" t="inlineStr">
-        <is>
-          <t>スレ②</t>
-        </is>
-      </c>
-      <c r="D82" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-    </row>
-    <row r="83">
-      <c r="A83" s="2" t="inlineStr">
-        <is>
-          <t>女性B下</t>
-        </is>
-      </c>
-      <c r="B83" s="3" t="inlineStr">
-        <is>
-          <t>出た自称新皇ｗ</t>
-        </is>
-      </c>
-      <c r="C83" s="2" t="inlineStr">
-        <is>
-          <t>スレ②</t>
-        </is>
-      </c>
-      <c r="D83" s="2" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-    </row>
-    <row r="84">
-      <c r="A84" s="2" t="inlineStr">
-        <is>
-          <t>男性C</t>
-        </is>
-      </c>
-      <c r="B84" s="3" t="inlineStr">
-        <is>
-          <t>名乗ったもん勝ちかよ</t>
-        </is>
-      </c>
-      <c r="C84" s="2" t="inlineStr">
-        <is>
-          <t>スレ②</t>
-        </is>
-      </c>
-      <c r="D84" s="2" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-    </row>
-    <row r="85">
-      <c r="A85" s="2" t="inlineStr">
-        <is>
-          <t>女性D</t>
-        </is>
-      </c>
-      <c r="B85" s="3" t="inlineStr">
-        <is>
-          <t>関東の田舎で勝手に天皇名乗ったやべえ人やろ</t>
-        </is>
-      </c>
-      <c r="C85" s="2" t="inlineStr">
-        <is>
-          <t>スレ②</t>
-        </is>
-      </c>
-      <c r="D85" s="2" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-    </row>
-    <row r="86">
-      <c r="A86" s="2" t="inlineStr">
-        <is>
-          <t>男性E</t>
-        </is>
-      </c>
-      <c r="B86" s="3" t="inlineStr">
-        <is>
-          <t>怨霊の話は聞くけど何した人かは正直知らんわ</t>
-        </is>
-      </c>
-      <c r="C86" s="2" t="inlineStr">
-        <is>
-          <t>スレ②</t>
-        </is>
-      </c>
-      <c r="D86" s="2" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-    </row>
-    <row r="87">
-      <c r="A87" s="2" t="inlineStr">
-        <is>
-          <t>男性A</t>
-        </is>
-      </c>
-      <c r="B87" s="3" t="inlineStr">
-        <is>
-          <t>で、結局こいつ何がしたかったん</t>
-        </is>
-      </c>
-      <c r="C87" s="2" t="inlineStr">
-        <is>
-          <t>スレ②</t>
-        </is>
-      </c>
-      <c r="D87" s="2" t="inlineStr">
-        <is>
-          <t>6</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>女性B</t>
+          <t>男性A</t>
         </is>
       </c>
       <c r="B88" s="3" t="inlineStr">
         <is>
-          <t>中央に喧嘩売って負けた人や、それ以上でもそれ以下でもなくない？</t>
+          <t>平将門「これからは俺が東の天皇やるわ」朝廷「は？」</t>
         </is>
       </c>
       <c r="C88" s="2" t="inlineStr">
@@ -2399,19 +2399,19 @@
       </c>
       <c r="D88" s="2" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
         <is>
-          <t>男性C大</t>
+          <t>女性B下</t>
         </is>
       </c>
       <c r="B89" s="3" t="inlineStr">
         <is>
-          <t>それがな、最初っから天皇に盾突こうとしてたわけちゃうんよ。スタートはただの一族内のもめ事や。関東の平氏一門で、伯父さんらと土地や縁談がらみの私闘をやっとった、いわば身内ゲンカからの叩き上げやねん。それが勝ち続けるうちに、どんどん引くに引けん大ごとになってってもうた</t>
+          <t>出た自称新皇ｗ</t>
         </is>
       </c>
       <c r="C89" s="2" t="inlineStr">
@@ -2421,19 +2421,19 @@
       </c>
       <c r="D89" s="2" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>2</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>女性D</t>
+          <t>男性C</t>
         </is>
       </c>
       <c r="B90" s="3" t="inlineStr">
         <is>
-          <t>ファッ最初は身内ゲンカなんか</t>
+          <t>名乗ったもん勝ちかよ</t>
         </is>
       </c>
       <c r="C90" s="2" t="inlineStr">
@@ -2443,19 +2443,19 @@
       </c>
       <c r="D90" s="2" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>3</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
         <is>
-          <t>男性E</t>
+          <t>女性D</t>
         </is>
       </c>
       <c r="B91" s="3" t="inlineStr">
         <is>
-          <t>そっからどうやって天皇になんねん</t>
+          <t>関東の田舎で勝手に天皇名乗ったやべえ人やろ</t>
         </is>
       </c>
       <c r="C91" s="2" t="inlineStr">
@@ -2465,19 +2465,19 @@
       </c>
       <c r="D91" s="2" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>4</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>男性A下</t>
+          <t>男性E</t>
         </is>
       </c>
       <c r="B92" s="3" t="inlineStr">
         <is>
-          <t>ヤンキーの抗争がいつの間にか国盗りになる漫画みたいや</t>
+          <t>結局その新皇とやらも2か月で終わった負け犬やん、持ち上げる要素ある？</t>
         </is>
       </c>
       <c r="C92" s="2" t="inlineStr">
@@ -2487,19 +2487,19 @@
       </c>
       <c r="D92" s="2" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>5</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
         <is>
-          <t>女性B大</t>
+          <t>男性A</t>
         </is>
       </c>
       <c r="B93" s="3" t="inlineStr">
         <is>
-          <t>そもそも将門の出自も知っとくとええで。あいつ桓武天皇の血を引く桓武平氏で、高望王の孫にあたる名門の出やねん。若い頃は京都に上って摂関家に奉公しとった時期もあって、決して田舎のチンピラちゃう。中央の作法も権力の構造も知った上で関東に戻って、結局その中央に弓を引くことになったわけや</t>
+          <t>怨霊の話は聞くけど何した人かは正直知らんわ</t>
         </is>
       </c>
       <c r="C93" s="2" t="inlineStr">
@@ -2509,19 +2509,19 @@
       </c>
       <c r="D93" s="2" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>6</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>男性C</t>
+          <t>女性B</t>
         </is>
       </c>
       <c r="B94" s="3" t="inlineStr">
         <is>
-          <t>元エリートが地元で反乱とか厨二すぎる</t>
+          <t>で、結局こいつ何がしたかったん</t>
         </is>
       </c>
       <c r="C94" s="2" t="inlineStr">
@@ -2531,19 +2531,19 @@
       </c>
       <c r="D94" s="2" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>7</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
         <is>
-          <t>女性D下</t>
+          <t>男性C</t>
         </is>
       </c>
       <c r="B95" s="3" t="inlineStr">
         <is>
-          <t>中身を知ってる奴が反旗ひるがえすのが一番こわいやつやん</t>
+          <t>中央に喧嘩売って負けた人や、それ以上でもそれ以下でもなくない？</t>
         </is>
       </c>
       <c r="C95" s="2" t="inlineStr">
@@ -2553,19 +2553,19 @@
       </c>
       <c r="D95" s="2" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>8</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>男性E大</t>
+          <t>女性D大</t>
         </is>
       </c>
       <c r="B96" s="3" t="inlineStr">
         <is>
-          <t>で、私闘で官側の人間ともやり合ううちに、今度は朝廷の出先の国府とぶつかってまう。勢いで常陸の国府を攻め落として、国の実印にあたる印鑰まで奪ってもうた。これ当時やと完全に一線を越えた行為で、国に弓を引いた賊って扱いになる。もう後戻りでけへんとこまで行ったわけや</t>
+          <t>それがな、最初っから天皇に盾突こうとしてたわけちゃうんよ。スタートはただの一族内のもめ事や。関東の平氏一門で、伯父さんらと土地や縁談がらみの私闘をやっとった、いわば身内ゲンカからの叩き上げやねん。それが勝ち続けるうちに、どんどん引くに引けん大ごとになってってもうた</t>
         </is>
       </c>
       <c r="C96" s="2" t="inlineStr">
@@ -2575,19 +2575,19 @@
       </c>
       <c r="D96" s="2" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>9</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
         <is>
-          <t>男性A</t>
+          <t>男性E</t>
         </is>
       </c>
       <c r="B97" s="3" t="inlineStr">
         <is>
-          <t>印鑰ってなんや</t>
+          <t>ファッ最初は身内ゲンカなんか</t>
         </is>
       </c>
       <c r="C97" s="2" t="inlineStr">
@@ -2597,19 +2597,19 @@
       </c>
       <c r="D97" s="2" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>10</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>女性B下</t>
+          <t>男性A</t>
         </is>
       </c>
       <c r="B98" s="3" t="inlineStr">
         <is>
-          <t>国を動かす実印とハンコ箱みたいなもんや。それ奪うって今でいう役所まるごと乗っ取るレベルやぞ</t>
+          <t>そっからどうやって天皇になんねん</t>
         </is>
       </c>
       <c r="C98" s="2" t="inlineStr">
@@ -2619,313 +2619,313 @@
       </c>
       <c r="D98" s="2" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>11</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
         <is>
+          <t>女性B下</t>
+        </is>
+      </c>
+      <c r="B99" s="3" t="inlineStr">
+        <is>
+          <t>ヤンキーの抗争がいつの間にか国盗りになる漫画みたいや</t>
+        </is>
+      </c>
+      <c r="C99" s="2" t="inlineStr">
+        <is>
+          <t>スレ②</t>
+        </is>
+      </c>
+      <c r="D99" s="2" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="2" t="inlineStr">
+        <is>
+          <t>男性C大</t>
+        </is>
+      </c>
+      <c r="B100" s="3" t="inlineStr">
+        <is>
+          <t>そもそも将門の出自も知っとくとええで。あいつ桓武天皇の血を引く桓武平氏で、高望王の孫にあたる名門の出やねん。若い頃は京都に上って摂関家に奉公しとった時期もあって、決して田舎のチンピラちゃう。中央の作法も権力の構造も知った上で関東に戻って、結局その中央に弓を引くことになったわけや</t>
+        </is>
+      </c>
+      <c r="C100" s="2" t="inlineStr">
+        <is>
+          <t>スレ②</t>
+        </is>
+      </c>
+      <c r="D100" s="2" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="2" t="inlineStr">
+        <is>
+          <t>女性D</t>
+        </is>
+      </c>
+      <c r="B101" s="3" t="inlineStr">
+        <is>
+          <t>元エリートが地元で反乱とか厨二すぎる</t>
+        </is>
+      </c>
+      <c r="C101" s="2" t="inlineStr">
+        <is>
+          <t>スレ②</t>
+        </is>
+      </c>
+      <c r="D101" s="2" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="2" t="inlineStr">
+        <is>
+          <t>男性E下</t>
+        </is>
+      </c>
+      <c r="B102" s="3" t="inlineStr">
+        <is>
+          <t>中身を知ってる奴が反旗ひるがえすのが一番こわいやつやん</t>
+        </is>
+      </c>
+      <c r="C102" s="2" t="inlineStr">
+        <is>
+          <t>スレ②</t>
+        </is>
+      </c>
+      <c r="D102" s="2" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="2" t="inlineStr">
+        <is>
+          <t>男性A大</t>
+        </is>
+      </c>
+      <c r="B103" s="3" t="inlineStr">
+        <is>
+          <t>ちな将門の地盤は下総の猿島あたりでな、当時の坂東は朝廷の目が届きにくい辺境で、しかも良馬の産地やった。だから機動力のある騎馬の武士団を抱えやすくて、中央から来た役人よりも地元で腕の立つ将門のほうが頼りにされとった。そういう土壌があったからこそ、一介の豪族が関東一円を呑み込むなんて芸当ができたわけや</t>
+        </is>
+      </c>
+      <c r="C103" s="2" t="inlineStr">
+        <is>
+          <t>スレ②</t>
+        </is>
+      </c>
+      <c r="D103" s="2" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="2" t="inlineStr">
+        <is>
+          <t>女性B下</t>
+        </is>
+      </c>
+      <c r="B104" s="3" t="inlineStr">
+        <is>
+          <t>馬かよ、そら強いわけや</t>
+        </is>
+      </c>
+      <c r="C104" s="2" t="inlineStr">
+        <is>
+          <t>スレ②</t>
+        </is>
+      </c>
+      <c r="D104" s="2" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="2" t="inlineStr">
+        <is>
+          <t>男性C大</t>
+        </is>
+      </c>
+      <c r="B105" s="3" t="inlineStr">
+        <is>
+          <t>で、私闘で官側の人間ともやり合ううちに、今度は朝廷の出先の国府とぶつかってまう。勢いで常陸の国府を攻め落として、国の実印にあたる印鑰まで奪ってもうた。これ当時やと完全に一線を越えた行為で、国に弓を引いた賊って扱いになる。もう後戻りでけへんとこまで行ったわけや</t>
+        </is>
+      </c>
+      <c r="C105" s="2" t="inlineStr">
+        <is>
+          <t>スレ②</t>
+        </is>
+      </c>
+      <c r="D105" s="2" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="2" t="inlineStr">
+        <is>
+          <t>女性D</t>
+        </is>
+      </c>
+      <c r="B106" s="3" t="inlineStr">
+        <is>
+          <t>印鑰ってなんや</t>
+        </is>
+      </c>
+      <c r="C106" s="2" t="inlineStr">
+        <is>
+          <t>スレ②</t>
+        </is>
+      </c>
+      <c r="D106" s="2" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="2" t="inlineStr">
+        <is>
+          <t>男性E下</t>
+        </is>
+      </c>
+      <c r="B107" s="3" t="inlineStr">
+        <is>
+          <t>国を動かす実印とハンコ箱みたいなもんや。それ奪うって今でいう役所まるごと乗っ取るレベルやぞ</t>
+        </is>
+      </c>
+      <c r="C107" s="2" t="inlineStr">
+        <is>
+          <t>スレ②</t>
+        </is>
+      </c>
+      <c r="D107" s="2" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="2" t="inlineStr">
+        <is>
           <t>解説者</t>
         </is>
       </c>
-      <c r="B99" s="3" t="inlineStr">
+      <c r="B108" s="3" t="inlineStr">
         <is>
           <t>印鑰とは、
 古代から中世の役所で使われた、
 国の実印と倉の鍵を指す言葉である。</t>
         </is>
       </c>
-      <c r="C99" s="2" t="inlineStr">
+      <c r="C108" s="2" t="inlineStr">
         <is>
           <t>解説：印鑰</t>
         </is>
       </c>
-      <c r="D99" s="2" t="inlineStr">
+      <c r="D108" s="2" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
     </row>
-    <row r="100">
-      <c r="A100" s="2" t="inlineStr">
+    <row r="109">
+      <c r="A109" s="2" t="inlineStr">
         <is>
           <t>解説者</t>
         </is>
       </c>
-      <c r="B100" s="3" t="inlineStr">
+      <c r="B109" s="3" t="inlineStr">
         <is>
           <t>印は公文書に押す国家の正式な印鑑、
 鑰は税として集めた米などを納めた
 正倉の鍵を意味する。</t>
         </is>
       </c>
-      <c r="C100" s="2" t="inlineStr">
+      <c r="C109" s="2" t="inlineStr">
         <is>
           <t>解説：印鑰</t>
         </is>
       </c>
-      <c r="D100" s="2" t="inlineStr">
+      <c r="D109" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
     </row>
-    <row r="101">
-      <c r="A101" s="2" t="inlineStr">
+    <row r="110">
+      <c r="A110" s="2" t="inlineStr">
         <is>
           <t>解説者</t>
         </is>
       </c>
-      <c r="B101" s="3" t="inlineStr">
+      <c r="B110" s="3" t="inlineStr">
         <is>
           <t>つまり印鑰を押さえることは、
 その国の行政と財産をまとめて
 手中に収めることに等しかった。</t>
         </is>
       </c>
-      <c r="C101" s="2" t="inlineStr">
+      <c r="C110" s="2" t="inlineStr">
         <is>
           <t>解説：印鑰</t>
         </is>
       </c>
-      <c r="D101" s="2" t="inlineStr">
+      <c r="D110" s="2" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
     </row>
-    <row r="102">
-      <c r="A102" s="2" t="inlineStr">
+    <row r="111">
+      <c r="A111" s="2" t="inlineStr">
         <is>
           <t>解説者</t>
         </is>
       </c>
-      <c r="B102" s="3" t="inlineStr">
+      <c r="B111" s="3" t="inlineStr">
         <is>
           <t>将門が国府を襲ってこれを奪った行為は、
 朝廷の支配そのものに正面から
 弓を引いたことを意味するのである。</t>
         </is>
       </c>
-      <c r="C102" s="2" t="inlineStr">
+      <c r="C111" s="2" t="inlineStr">
         <is>
           <t>解説：印鑰</t>
         </is>
       </c>
-      <c r="D102" s="2" t="inlineStr">
+      <c r="D111" s="2" t="inlineStr">
         <is>
           <t>4</t>
-        </is>
-      </c>
-    </row>
-    <row r="103">
-      <c r="A103" s="2" t="inlineStr">
-        <is>
-          <t>男性C大</t>
-        </is>
-      </c>
-      <c r="B103" s="3" t="inlineStr">
-        <is>
-          <t>そっから勢いに乗った将門は、坂東、今でいう関東一帯の国府を次々落として、ほぼ関東全域を手中に収めてまう。各国の国司を追い出して、自前の人事で「ここからは俺が仕切る国や」ってやり始めた。地方の豪族が中央任命の役人をまとめて吹っ飛ばすって、当時前代未聞やってん</t>
-        </is>
-      </c>
-      <c r="C103" s="2" t="inlineStr">
-        <is>
-          <t>スレ②</t>
-        </is>
-      </c>
-      <c r="D103" s="2" t="inlineStr">
-        <is>
-          <t>18</t>
-        </is>
-      </c>
-    </row>
-    <row r="104">
-      <c r="A104" s="2" t="inlineStr">
-        <is>
-          <t>女性D下</t>
-        </is>
-      </c>
-      <c r="B104" s="3" t="inlineStr">
-        <is>
-          <t>関東まるごとはやりすぎやろ</t>
-        </is>
-      </c>
-      <c r="C104" s="2" t="inlineStr">
-        <is>
-          <t>スレ②</t>
-        </is>
-      </c>
-      <c r="D104" s="2" t="inlineStr">
-        <is>
-          <t>19</t>
-        </is>
-      </c>
-    </row>
-    <row r="105">
-      <c r="A105" s="2" t="inlineStr">
-        <is>
-          <t>男性E</t>
-        </is>
-      </c>
-      <c r="B105" s="3" t="inlineStr">
-        <is>
-          <t>もう完全に独立国家やん</t>
-        </is>
-      </c>
-      <c r="C105" s="2" t="inlineStr">
-        <is>
-          <t>スレ②</t>
-        </is>
-      </c>
-      <c r="D105" s="2" t="inlineStr">
-        <is>
-          <t>20</t>
-        </is>
-      </c>
-    </row>
-    <row r="106">
-      <c r="A106" s="2" t="inlineStr">
-        <is>
-          <t>男性A</t>
-        </is>
-      </c>
-      <c r="B106" s="3" t="inlineStr">
-        <is>
-          <t>で、調子乗って新皇宣言と</t>
-        </is>
-      </c>
-      <c r="C106" s="2" t="inlineStr">
-        <is>
-          <t>スレ②</t>
-        </is>
-      </c>
-      <c r="D106" s="2" t="inlineStr">
-        <is>
-          <t>21</t>
-        </is>
-      </c>
-    </row>
-    <row r="107">
-      <c r="A107" s="2" t="inlineStr">
-        <is>
-          <t>女性B大</t>
-        </is>
-      </c>
-      <c r="B107" s="3" t="inlineStr">
-        <is>
-          <t>そう、ここで「新皇」、つまり新しい天皇を名乗る。伝説やと八幡神のお告げで位を授かったってことになっとるけど、要は京都の天皇とは別に、東国に自分を頂点とした朝廷を立てようとしたわけや。関東に独立政権を作るっていう、日本史でもなかなかおらんスケールの反逆やねん</t>
-        </is>
-      </c>
-      <c r="C107" s="2" t="inlineStr">
-        <is>
-          <t>スレ②</t>
-        </is>
-      </c>
-      <c r="D107" s="2" t="inlineStr">
-        <is>
-          <t>22</t>
-        </is>
-      </c>
-    </row>
-    <row r="108">
-      <c r="A108" s="2" t="inlineStr">
-        <is>
-          <t>男性C</t>
-        </is>
-      </c>
-      <c r="B108" s="3" t="inlineStr">
-        <is>
-          <t>八幡のお告げは草、自分で言うてるだけやろ知らんけど</t>
-        </is>
-      </c>
-      <c r="C108" s="2" t="inlineStr">
-        <is>
-          <t>スレ②</t>
-        </is>
-      </c>
-      <c r="D108" s="2" t="inlineStr">
-        <is>
-          <t>23</t>
-        </is>
-      </c>
-    </row>
-    <row r="109">
-      <c r="A109" s="2" t="inlineStr">
-        <is>
-          <t>女性D</t>
-        </is>
-      </c>
-      <c r="B109" s="3" t="inlineStr">
-        <is>
-          <t>神様持ち出すの強気すぎる</t>
-        </is>
-      </c>
-      <c r="C109" s="2" t="inlineStr">
-        <is>
-          <t>スレ②</t>
-        </is>
-      </c>
-      <c r="D109" s="2" t="inlineStr">
-        <is>
-          <t>24</t>
-        </is>
-      </c>
-    </row>
-    <row r="110">
-      <c r="A110" s="2" t="inlineStr">
-        <is>
-          <t>男性E</t>
-        </is>
-      </c>
-      <c r="B110" s="3" t="inlineStr">
-        <is>
-          <t>正直そこは盛りやろ、神託とか後付けくさいわ</t>
-        </is>
-      </c>
-      <c r="C110" s="2" t="inlineStr">
-        <is>
-          <t>スレ②</t>
-        </is>
-      </c>
-      <c r="D110" s="2" t="inlineStr">
-        <is>
-          <t>25</t>
-        </is>
-      </c>
-    </row>
-    <row r="111">
-      <c r="A111" s="2" t="inlineStr">
-        <is>
-          <t>男性A下</t>
-        </is>
-      </c>
-      <c r="B111" s="3" t="inlineStr">
-        <is>
-          <t>まあ伝説部分はな。ただ実際に独立政権を作ろうとしたのは確からしいで</t>
-        </is>
-      </c>
-      <c r="C111" s="2" t="inlineStr">
-        <is>
-          <t>スレ②</t>
-        </is>
-      </c>
-      <c r="D111" s="2" t="inlineStr">
-        <is>
-          <t>26</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
         <is>
-          <t>女性B</t>
+          <t>男性A大</t>
         </is>
       </c>
       <c r="B112" s="3" t="inlineStr">
         <is>
-          <t>でもこんなん中央がブチギレて終わりやん</t>
+          <t>そっから勢いに乗った将門は、坂東、今でいう関東一帯の国府を次々落として、ほぼ関東全域を手中に収めてまう。各国の国司を追い出して、自前の人事で「ここからは俺が仕切る国や」ってやり始めた。地方の豪族が中央任命の役人をまとめて吹っ飛ばすって、当時前代未聞やってん</t>
         </is>
       </c>
       <c r="C112" s="2" t="inlineStr">
@@ -2935,19 +2935,19 @@
       </c>
       <c r="D112" s="2" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>21</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
         <is>
-          <t>男性C大</t>
+          <t>女性B下</t>
         </is>
       </c>
       <c r="B113" s="3" t="inlineStr">
         <is>
-          <t>そうなる。京都は将門を朝敵認定して追討令を出す。で、ここで動いたのが同じ関東の平貞盛と、下野の豪族やった藤原秀郷や。身内や近隣やった連中が討伐側に回って、将門包囲網が出来てまうわけや</t>
+          <t>関東まるごとはやりすぎやろ</t>
         </is>
       </c>
       <c r="C113" s="2" t="inlineStr">
@@ -2957,19 +2957,19 @@
       </c>
       <c r="D113" s="2" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>22</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
         <is>
-          <t>女性D下</t>
+          <t>男性C</t>
         </is>
       </c>
       <c r="B114" s="3" t="inlineStr">
         <is>
-          <t>結局身内に討たれるんかい</t>
+          <t>もう完全に独立国家やん</t>
         </is>
       </c>
       <c r="C114" s="2" t="inlineStr">
@@ -2979,19 +2979,19 @@
       </c>
       <c r="D114" s="2" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>23</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
         <is>
-          <t>男性E</t>
+          <t>女性D</t>
         </is>
       </c>
       <c r="B115" s="3" t="inlineStr">
         <is>
-          <t>関東の独立より自分の家のほうが大事って奴がおったわけやな</t>
+          <t>で、調子乗って新皇宣言と</t>
         </is>
       </c>
       <c r="C115" s="2" t="inlineStr">
@@ -3001,19 +3001,19 @@
       </c>
       <c r="D115" s="2" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>24</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
         <is>
-          <t>男性A</t>
+          <t>男性E大</t>
         </is>
       </c>
       <c r="B116" s="3" t="inlineStr">
         <is>
-          <t>将門を討ったのって源氏の先祖やっけ？</t>
+          <t>そう、ここで「新皇」、つまり新しい天皇を名乗る。伝説やと八幡神のお告げで位を授かったってことになっとるけど、要は京都の天皇とは別に、東国に自分を頂点とした朝廷を立てようとしたわけや。関東に独立政権を作るっていう、日本史でもなかなかおらんスケールの反逆やねん</t>
         </is>
       </c>
       <c r="C116" s="2" t="inlineStr">
@@ -3023,19 +3023,19 @@
       </c>
       <c r="D116" s="2" t="inlineStr">
         <is>
-          <t>31</t>
+          <t>25</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
         <is>
-          <t>女性B下</t>
+          <t>男性A</t>
         </is>
       </c>
       <c r="B117" s="3" t="inlineStr">
         <is>
-          <t>ちゃう、討ったのは平貞盛と藤原秀郷や。源氏ちゃうから、そこ混同したらあかんで</t>
+          <t>八幡のお告げは草、自分で言うてるだけやろ知らんけど</t>
         </is>
       </c>
       <c r="C117" s="2" t="inlineStr">
@@ -3045,19 +3045,19 @@
       </c>
       <c r="D117" s="2" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>26</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
         <is>
-          <t>男性C</t>
+          <t>女性B</t>
         </is>
       </c>
       <c r="B118" s="3" t="inlineStr">
         <is>
-          <t>あっそうやったか、すまんね</t>
+          <t>神様持ち出すの強気すぎる</t>
         </is>
       </c>
       <c r="C118" s="2" t="inlineStr">
@@ -3067,19 +3067,19 @@
       </c>
       <c r="D118" s="2" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>27</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
         <is>
-          <t>女性D大</t>
+          <t>男性C</t>
         </is>
       </c>
       <c r="B119" s="3" t="inlineStr">
         <is>
-          <t>で、天慶3年、西暦940年に討伐軍とぶつかって、将門は敗れる。伝承やと、戦いの最中に飛んできた流れ矢が額に当たって、それが致命傷になって命を落としたって言われとる。新皇を名乗ってからわずか2か月ほどでの最期や。あれだけ関東を席巻したのに、終わりはほんま一瞬やった</t>
+          <t>正直そこは盛りやろ、神託とか後付けくさいわ</t>
         </is>
       </c>
       <c r="C119" s="2" t="inlineStr">
@@ -3089,19 +3089,19 @@
       </c>
       <c r="D119" s="2" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>28</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
         <is>
-          <t>男性E</t>
+          <t>女性D</t>
         </is>
       </c>
       <c r="B120" s="3" t="inlineStr">
         <is>
-          <t>2か月て短すぎやろ</t>
+          <t>で？神名乗ろうがすぐ討たれたんやから、結局ただの勘違いした田舎の暴れん坊やん</t>
         </is>
       </c>
       <c r="C120" s="2" t="inlineStr">
@@ -3111,19 +3111,19 @@
       </c>
       <c r="D120" s="2" t="inlineStr">
         <is>
-          <t>35</t>
+          <t>29</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
         <is>
-          <t>男性A</t>
+          <t>男性E下</t>
         </is>
       </c>
       <c r="B121" s="3" t="inlineStr">
         <is>
-          <t>天下取り損ねたというか、名乗っただけで終わったやんｗ</t>
+          <t>勘違いで関東一国まとめられたら誰も苦労せんわ、そこは認めたれや</t>
         </is>
       </c>
       <c r="C121" s="2" t="inlineStr">
@@ -3133,19 +3133,19 @@
       </c>
       <c r="D121" s="2" t="inlineStr">
         <is>
-          <t>36</t>
+          <t>30</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
         <is>
-          <t>女性B大</t>
+          <t>男性A</t>
         </is>
       </c>
       <c r="B122" s="3" t="inlineStr">
         <is>
-          <t>その最期にも伝説があってな。将門は矢も通さんと評判の無敵の体で討伐軍が苦戦しとったけど、戦いの最中に陣の風向きが急に変わって、その隙に放たれた矢が額に当たったって話が残っとる。神がかった強さやのに、最後は風っていう運否天賦みたいなもんで決着した、っていうのがまた伝説を盛り上げとるんや</t>
+          <t>でもこんなん中央がブチギレて終わりやん</t>
         </is>
       </c>
       <c r="C122" s="2" t="inlineStr">
@@ -3155,19 +3155,19 @@
       </c>
       <c r="D122" s="2" t="inlineStr">
         <is>
-          <t>37</t>
+          <t>31</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
         <is>
-          <t>男性C下</t>
+          <t>女性B大</t>
         </is>
       </c>
       <c r="B123" s="3" t="inlineStr">
         <is>
-          <t>急に弱点が出てくるの少年漫画やん</t>
+          <t>そうなる。京都は将門を朝敵認定して追討令を出す。で、ここで動いたのが同じ関東の平貞盛と、下野の豪族やった藤原秀郷や。身内や近隣やった連中が討伐側に回って、将門包囲網が出来てまうわけや</t>
         </is>
       </c>
       <c r="C123" s="2" t="inlineStr">
@@ -3177,19 +3177,19 @@
       </c>
       <c r="D123" s="2" t="inlineStr">
         <is>
-          <t>38</t>
+          <t>32</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
         <is>
-          <t>女性D</t>
+          <t>男性C下</t>
         </is>
       </c>
       <c r="B124" s="3" t="inlineStr">
         <is>
-          <t>風で負けるラスボスすこｗ</t>
+          <t>結局身内に討たれるんかい</t>
         </is>
       </c>
       <c r="C124" s="2" t="inlineStr">
@@ -3199,19 +3199,19 @@
       </c>
       <c r="D124" s="2" t="inlineStr">
         <is>
-          <t>39</t>
+          <t>33</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
         <is>
-          <t>男性E大</t>
+          <t>女性D</t>
         </is>
       </c>
       <c r="B125" s="3" t="inlineStr">
         <is>
-          <t>もういっこ有名なんが影武者伝説や。将門にはそっくりの影武者が何人もおって、本物を見分けられんかったけど、こめかみのあたりに本物だけ影が無かった、みたいな尾ひれが後世に付いとる。要は強すぎて普通には討てんかったっていう"負けたのが信じられん"空気が、こういう伝説を生んだわけやな</t>
+          <t>関東の独立より自分の家のほうが大事って奴がおったわけやな</t>
         </is>
       </c>
       <c r="C125" s="2" t="inlineStr">
@@ -3221,19 +3221,19 @@
       </c>
       <c r="D125" s="2" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>34</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
         <is>
-          <t>男性A</t>
+          <t>男性E</t>
         </is>
       </c>
       <c r="B126" s="3" t="inlineStr">
         <is>
-          <t>影武者まで盛られるの大物の証や</t>
+          <t>将門を討ったのって源氏の先祖やっけ？</t>
         </is>
       </c>
       <c r="C126" s="2" t="inlineStr">
@@ -3243,19 +3243,19 @@
       </c>
       <c r="D126" s="2" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>35</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
         <is>
-          <t>女性B</t>
+          <t>男性A下</t>
         </is>
       </c>
       <c r="B127" s="3" t="inlineStr">
         <is>
-          <t>そこからの首が飛ぶ伝説に繋がるわけやな</t>
+          <t>ちゃう、討ったのは平貞盛と藤原秀郷や。源氏ちゃうから、そこ混同したらあかんで</t>
         </is>
       </c>
       <c r="C127" s="2" t="inlineStr">
@@ -3265,19 +3265,19 @@
       </c>
       <c r="D127" s="2" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>36</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
         <is>
-          <t>男性C</t>
+          <t>女性B</t>
         </is>
       </c>
       <c r="B128" s="3" t="inlineStr">
         <is>
-          <t>そう、討たれた首は京都に送られて晒される。で、その首が夜に飛んで関東に戻った、っていうのが前半の祟りの話に繋がるんや</t>
+          <t>あっそうやったか、すまんね</t>
         </is>
       </c>
       <c r="C128" s="2" t="inlineStr">
@@ -3287,19 +3287,19 @@
       </c>
       <c r="D128" s="2" t="inlineStr">
         <is>
-          <t>43</t>
+          <t>37</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
         <is>
-          <t>女性D</t>
+          <t>男性C大</t>
         </is>
       </c>
       <c r="B129" s="3" t="inlineStr">
         <is>
-          <t>きれいに一周してて草</t>
+          <t>で、天慶3年、西暦940年に討伐軍とぶつかって、将門は敗れる。伝承やと、戦いの最中に飛んできた流れ矢が額に当たって、それが致命傷になって命を落としたって言われとる。新皇を名乗ってからわずか2か月ほどでの最期や。あれだけ関東を席巻したのに、終わりはほんま一瞬やった</t>
         </is>
       </c>
       <c r="C129" s="2" t="inlineStr">
@@ -3309,19 +3309,19 @@
       </c>
       <c r="D129" s="2" t="inlineStr">
         <is>
-          <t>44</t>
+          <t>38</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
         <is>
-          <t>男性E</t>
+          <t>女性D</t>
         </is>
       </c>
       <c r="B130" s="3" t="inlineStr">
         <is>
-          <t>でもさ、結局こいつただの調子乗った反乱者やん。評価する要素ある？</t>
+          <t>2か月て短すぎやろ</t>
         </is>
       </c>
       <c r="C130" s="2" t="inlineStr">
@@ -3331,19 +3331,19 @@
       </c>
       <c r="D130" s="2" t="inlineStr">
         <is>
-          <t>45</t>
+          <t>39</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
         <is>
-          <t>男性A大</t>
+          <t>男性E</t>
         </is>
       </c>
       <c r="B131" s="3" t="inlineStr">
         <is>
-          <t>それがそうとも言い切れんのよ。中央の貴族が地方を搾取する仕組みに、地方の武装勢力が真っ向から「ノー」を突きつけた最初級の例なんや。後の武士が自分らの力で土地を治める時代の、いわば走りやねん。だから単なる謀反人やのうて、関東武士の精神的な元祖として評価する見方も根強いんや</t>
+          <t>天下取り損ねたというか、名乗っただけで終わったやんｗ</t>
         </is>
       </c>
       <c r="C131" s="2" t="inlineStr">
@@ -3353,19 +3353,19 @@
       </c>
       <c r="D131" s="2" t="inlineStr">
         <is>
-          <t>46</t>
+          <t>40</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
         <is>
-          <t>女性B</t>
+          <t>男性A大</t>
         </is>
       </c>
       <c r="B132" s="3" t="inlineStr">
         <is>
-          <t>はい武士オタの過大評価、盛りすぎて引くわ</t>
+          <t>その最期にも伝説があってな。将門は矢も通さんと評判の無敵の体で討伐軍が苦戦しとったけど、戦いの最中に陣の風向きが急に変わって、その隙に放たれた矢が額に当たったって話が残っとる。神がかった強さやのに、最後は風っていう運否天賦みたいなもんで決着した、っていうのがまた伝説を盛り上げとるんや</t>
         </is>
       </c>
       <c r="C132" s="2" t="inlineStr">
@@ -3375,19 +3375,19 @@
       </c>
       <c r="D132" s="2" t="inlineStr">
         <is>
-          <t>47</t>
+          <t>41</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
         <is>
-          <t>男性C下</t>
+          <t>女性B下</t>
         </is>
       </c>
       <c r="B133" s="3" t="inlineStr">
         <is>
-          <t>過大評価ってだけで片付けるのも雑やろ、現に怨霊で千年語り継がれとるんやから</t>
+          <t>急に弱点が出てくるの少年漫画やん</t>
         </is>
       </c>
       <c r="C133" s="2" t="inlineStr">
@@ -3397,19 +3397,19 @@
       </c>
       <c r="D133" s="2" t="inlineStr">
         <is>
-          <t>48</t>
+          <t>42</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
         <is>
-          <t>女性D</t>
+          <t>男性C</t>
         </is>
       </c>
       <c r="B134" s="3" t="inlineStr">
         <is>
-          <t>で？千年語り継がれようが負けは負けやろ、はい解散</t>
+          <t>風で負けるラスボスすこｗ</t>
         </is>
       </c>
       <c r="C134" s="2" t="inlineStr">
@@ -3419,19 +3419,19 @@
       </c>
       <c r="D134" s="2" t="inlineStr">
         <is>
-          <t>49</t>
+          <t>43</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
         <is>
-          <t>男性E下</t>
+          <t>女性D大</t>
         </is>
       </c>
       <c r="B135" s="3" t="inlineStr">
         <is>
-          <t>その負けっぷりで神様にまでなっとるんやから世話ないわ</t>
+          <t>もういっこ有名なんが影武者伝説や。将門にはそっくりの影武者が何人もおって、本物を見分けられんかったけど、こめかみのあたりに本物だけ影が無かった、みたいな尾ひれが後世に付いとる。要は強すぎて普通には討てんかったっていう"負けたのが信じられん"空気が、こういう伝説を生んだわけやな</t>
         </is>
       </c>
       <c r="C135" s="2" t="inlineStr">
@@ -3441,19 +3441,19 @@
       </c>
       <c r="D135" s="2" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>44</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
         <is>
-          <t>男性A</t>
+          <t>男性E</t>
         </is>
       </c>
       <c r="B136" s="3" t="inlineStr">
         <is>
-          <t>あと同じ時期に西で藤原純友も暴れとって、東西で同時に乱が起きとったんよな</t>
+          <t>影武者まで盛られるの大物の証や</t>
         </is>
       </c>
       <c r="C136" s="2" t="inlineStr">
@@ -3463,19 +3463,19 @@
       </c>
       <c r="D136" s="2" t="inlineStr">
         <is>
-          <t>51</t>
+          <t>45</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
         <is>
-          <t>女性B下</t>
+          <t>男性A</t>
         </is>
       </c>
       <c r="B137" s="3" t="inlineStr">
         <is>
-          <t>それや、承平天慶の乱でセット扱いされるやつ。朝廷からしたら東西挟み撃ちで生きた心地せんかったやろな</t>
+          <t>そういや将門を祀っとる国王神社が茨城にあって、将門の三女が建てたって伝わっとるな。ワイ一回行ったけど、めっちゃ静かでええとこやった</t>
         </is>
       </c>
       <c r="C137" s="2" t="inlineStr">
@@ -3485,357 +3485,599 @@
       </c>
       <c r="D137" s="2" t="inlineStr">
         <is>
-          <t>52</t>
+          <t>46</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
         <is>
+          <t>女性B</t>
+        </is>
+      </c>
+      <c r="B138" s="3" t="inlineStr">
+        <is>
+          <t>大河で将門やらんのかな、昔の風と雲と虹と以来やろ</t>
+        </is>
+      </c>
+      <c r="C138" s="2" t="inlineStr">
+        <is>
+          <t>スレ②</t>
+        </is>
+      </c>
+      <c r="D138" s="2" t="inlineStr">
+        <is>
+          <t>47</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="2" t="inlineStr">
+        <is>
+          <t>男性C</t>
+        </is>
+      </c>
+      <c r="B139" s="3" t="inlineStr">
+        <is>
+          <t>主役が朝敵やと今のNHKはやりにくいやろなあ</t>
+        </is>
+      </c>
+      <c r="C139" s="2" t="inlineStr">
+        <is>
+          <t>スレ②</t>
+        </is>
+      </c>
+      <c r="D139" s="2" t="inlineStr">
+        <is>
+          <t>48</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="2" t="inlineStr">
+        <is>
+          <t>女性D</t>
+        </is>
+      </c>
+      <c r="B140" s="3" t="inlineStr">
+        <is>
+          <t>で、その首が飛ぶ伝説に繋がるわけやな</t>
+        </is>
+      </c>
+      <c r="C140" s="2" t="inlineStr">
+        <is>
+          <t>スレ②</t>
+        </is>
+      </c>
+      <c r="D140" s="2" t="inlineStr">
+        <is>
+          <t>49</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="2" t="inlineStr">
+        <is>
+          <t>男性E</t>
+        </is>
+      </c>
+      <c r="B141" s="3" t="inlineStr">
+        <is>
+          <t>そう、討たれた首は京都に送られて晒される。で、その首が夜に飛んで関東に戻った、っていうのが前半の祟りの話に繋がるんや</t>
+        </is>
+      </c>
+      <c r="C141" s="2" t="inlineStr">
+        <is>
+          <t>スレ②</t>
+        </is>
+      </c>
+      <c r="D141" s="2" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="2" t="inlineStr">
+        <is>
+          <t>男性A下</t>
+        </is>
+      </c>
+      <c r="B142" s="3" t="inlineStr">
+        <is>
+          <t>きれいに一周してて草</t>
+        </is>
+      </c>
+      <c r="C142" s="2" t="inlineStr">
+        <is>
+          <t>スレ②</t>
+        </is>
+      </c>
+      <c r="D142" s="2" t="inlineStr">
+        <is>
+          <t>51</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="2" t="inlineStr">
+        <is>
+          <t>女性B</t>
+        </is>
+      </c>
+      <c r="B143" s="3" t="inlineStr">
+        <is>
+          <t>でもさ、結局こいつただの調子乗った反乱者やん。評価する要素ある？</t>
+        </is>
+      </c>
+      <c r="C143" s="2" t="inlineStr">
+        <is>
+          <t>スレ②</t>
+        </is>
+      </c>
+      <c r="D143" s="2" t="inlineStr">
+        <is>
+          <t>52</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="2" t="inlineStr">
+        <is>
+          <t>男性C大</t>
+        </is>
+      </c>
+      <c r="B144" s="3" t="inlineStr">
+        <is>
+          <t>それがそうとも言い切れんのよ。中央の貴族が地方を搾取する仕組みに、地方の武装勢力が真っ向から「ノー」を突きつけた最初級の例なんや。後の武士が自分らの力で土地を治める時代の、いわば走りやねん。だから単なる謀反人やのうて、関東武士の精神的な元祖として評価する見方も根強いんや</t>
+        </is>
+      </c>
+      <c r="C144" s="2" t="inlineStr">
+        <is>
+          <t>スレ②</t>
+        </is>
+      </c>
+      <c r="D144" s="2" t="inlineStr">
+        <is>
+          <t>53</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="2" t="inlineStr">
+        <is>
+          <t>女性D</t>
+        </is>
+      </c>
+      <c r="B145" s="3" t="inlineStr">
+        <is>
+          <t>はい武士オタの過大評価、盛りすぎて引くわ</t>
+        </is>
+      </c>
+      <c r="C145" s="2" t="inlineStr">
+        <is>
+          <t>スレ②</t>
+        </is>
+      </c>
+      <c r="D145" s="2" t="inlineStr">
+        <is>
+          <t>54</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="2" t="inlineStr">
+        <is>
+          <t>男性E下</t>
+        </is>
+      </c>
+      <c r="B146" s="3" t="inlineStr">
+        <is>
+          <t>過大評価ってだけで片付けるのも雑やろ、現に怨霊で千年語り継がれとるんやから</t>
+        </is>
+      </c>
+      <c r="C146" s="2" t="inlineStr">
+        <is>
+          <t>スレ②</t>
+        </is>
+      </c>
+      <c r="D146" s="2" t="inlineStr">
+        <is>
+          <t>55</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="2" t="inlineStr">
+        <is>
+          <t>男性A</t>
+        </is>
+      </c>
+      <c r="B147" s="3" t="inlineStr">
+        <is>
+          <t>あと同じ時期に西で藤原純友も暴れとって、東西で同時に乱が起きとったんよな</t>
+        </is>
+      </c>
+      <c r="C147" s="2" t="inlineStr">
+        <is>
+          <t>スレ②</t>
+        </is>
+      </c>
+      <c r="D147" s="2" t="inlineStr">
+        <is>
+          <t>56</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="2" t="inlineStr">
+        <is>
+          <t>女性B下</t>
+        </is>
+      </c>
+      <c r="B148" s="3" t="inlineStr">
+        <is>
+          <t>それや、承平天慶の乱でセット扱いされるやつ。朝廷からしたら東西挟み撃ちで生きた心地せんかったやろな</t>
+        </is>
+      </c>
+      <c r="C148" s="2" t="inlineStr">
+        <is>
+          <t>スレ②</t>
+        </is>
+      </c>
+      <c r="D148" s="2" t="inlineStr">
+        <is>
+          <t>57</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="2" t="inlineStr">
+        <is>
           <t>解説者</t>
         </is>
       </c>
-      <c r="B138" s="3" t="inlineStr">
+      <c r="B149" s="3" t="inlineStr">
         <is>
           <t>承平天慶の乱とは、
 平安時代中期に東西で同時に起きた
 二つの大きな反乱の総称である。</t>
         </is>
       </c>
-      <c r="C138" s="2" t="inlineStr">
+      <c r="C149" s="2" t="inlineStr">
         <is>
           <t>解説：承平天慶の乱</t>
         </is>
       </c>
-      <c r="D138" s="2" t="inlineStr">
+      <c r="D149" s="2" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
     </row>
-    <row r="139">
-      <c r="A139" s="2" t="inlineStr">
+    <row r="150">
+      <c r="A150" s="2" t="inlineStr">
         <is>
           <t>解説者</t>
         </is>
       </c>
-      <c r="B139" s="3" t="inlineStr">
+      <c r="B150" s="3" t="inlineStr">
         <is>
           <t>東国では平将門が新皇を名乗って関東を制圧し、
 西国では瀬戸内で藤原純友が
 海賊を率いて朝廷に反旗をひるがえした。</t>
         </is>
       </c>
-      <c r="C139" s="2" t="inlineStr">
+      <c r="C150" s="2" t="inlineStr">
         <is>
           <t>解説：承平天慶の乱</t>
         </is>
       </c>
-      <c r="D139" s="2" t="inlineStr">
+      <c r="D150" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
     </row>
-    <row r="140">
-      <c r="A140" s="2" t="inlineStr">
+    <row r="151">
+      <c r="A151" s="2" t="inlineStr">
         <is>
           <t>解説者</t>
         </is>
       </c>
-      <c r="B140" s="3" t="inlineStr">
+      <c r="B151" s="3" t="inlineStr">
         <is>
           <t>朝廷にとっては東西から同時に
 挑戦を突きつけられた前代未聞の事態であり、</t>
         </is>
       </c>
-      <c r="C140" s="2" t="inlineStr">
+      <c r="C151" s="2" t="inlineStr">
         <is>
           <t>解説：承平天慶の乱</t>
         </is>
       </c>
-      <c r="D140" s="2" t="inlineStr">
+      <c r="D151" s="2" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
     </row>
-    <row r="141">
-      <c r="A141" s="2" t="inlineStr">
+    <row r="152">
+      <c r="A152" s="2" t="inlineStr">
         <is>
           <t>解説者</t>
         </is>
       </c>
-      <c r="B141" s="3" t="inlineStr">
+      <c r="B152" s="3" t="inlineStr">
         <is>
           <t>地方の武士の力を
 中央が無視できなくなっていく
 大きな転機となった出来事である。</t>
         </is>
       </c>
-      <c r="C141" s="2" t="inlineStr">
+      <c r="C152" s="2" t="inlineStr">
         <is>
           <t>解説：承平天慶の乱</t>
         </is>
       </c>
-      <c r="D141" s="2" t="inlineStr">
+      <c r="D152" s="2" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
     </row>
-    <row r="142">
-      <c r="A142" s="2" t="inlineStr">
+    <row r="153">
+      <c r="A153" s="2" t="inlineStr">
         <is>
           <t>男性C</t>
         </is>
       </c>
-      <c r="B142" s="3" t="inlineStr">
+      <c r="B153" s="3" t="inlineStr">
         <is>
           <t>もし将門が勝っとったら関東に別の国できてたんかな</t>
         </is>
       </c>
-      <c r="C142" s="2" t="inlineStr">
-        <is>
-          <t>スレ②</t>
-        </is>
-      </c>
-      <c r="D142" s="2" t="inlineStr">
-        <is>
-          <t>53</t>
-        </is>
-      </c>
-    </row>
-    <row r="143">
-      <c r="A143" s="2" t="inlineStr">
+      <c r="C153" s="2" t="inlineStr">
+        <is>
+          <t>スレ②</t>
+        </is>
+      </c>
+      <c r="D153" s="2" t="inlineStr">
+        <is>
+          <t>58</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="2" t="inlineStr">
         <is>
           <t>女性D大</t>
         </is>
       </c>
-      <c r="B143" s="3" t="inlineStr">
+      <c r="B154" s="3" t="inlineStr">
         <is>
           <t>そこはロマンあるよな。もし討伐をしのいで東国政権が定着しとったら、関東拠点の独立勢力が早い段階で出来て、武士の世が何百年か前倒しになってたかもしれん。まあ補給も人望もまだ足りんかったから現実は厳しかったやろけど。知らんけど、たらればとしては最高に面白い人物やわ</t>
         </is>
       </c>
-      <c r="C143" s="2" t="inlineStr">
-        <is>
-          <t>スレ②</t>
-        </is>
-      </c>
-      <c r="D143" s="2" t="inlineStr">
-        <is>
-          <t>54</t>
-        </is>
-      </c>
-    </row>
-    <row r="144">
-      <c r="A144" s="2" t="inlineStr">
+      <c r="C154" s="2" t="inlineStr">
+        <is>
+          <t>スレ②</t>
+        </is>
+      </c>
+      <c r="D154" s="2" t="inlineStr">
+        <is>
+          <t>59</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="2" t="inlineStr">
         <is>
           <t>男性E下</t>
         </is>
       </c>
-      <c r="B144" s="3" t="inlineStr">
+      <c r="B155" s="3" t="inlineStr">
         <is>
           <t>関東人としてはちょっと応援したくなる</t>
         </is>
       </c>
-      <c r="C144" s="2" t="inlineStr">
-        <is>
-          <t>スレ②</t>
-        </is>
-      </c>
-      <c r="D144" s="2" t="inlineStr">
-        <is>
-          <t>55</t>
-        </is>
-      </c>
-    </row>
-    <row r="145">
-      <c r="A145" s="2" t="inlineStr">
+      <c r="C155" s="2" t="inlineStr">
+        <is>
+          <t>スレ②</t>
+        </is>
+      </c>
+      <c r="D155" s="2" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="2" t="inlineStr">
         <is>
           <t>男性A</t>
         </is>
       </c>
-      <c r="B145" s="3" t="inlineStr">
+      <c r="B156" s="3" t="inlineStr">
         <is>
           <t>ワイ千葉県民、地味に将門ゆかりの地に住んどる</t>
         </is>
       </c>
-      <c r="C145" s="2" t="inlineStr">
-        <is>
-          <t>スレ②</t>
-        </is>
-      </c>
-      <c r="D145" s="2" t="inlineStr">
-        <is>
-          <t>56</t>
-        </is>
-      </c>
-    </row>
-    <row r="146">
-      <c r="A146" s="2" t="inlineStr">
+      <c r="C156" s="2" t="inlineStr">
+        <is>
+          <t>スレ②</t>
+        </is>
+      </c>
+      <c r="D156" s="2" t="inlineStr">
+        <is>
+          <t>61</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="2" t="inlineStr">
         <is>
           <t>女性B</t>
         </is>
       </c>
-      <c r="B146" s="3" t="inlineStr">
+      <c r="B157" s="3" t="inlineStr">
         <is>
           <t>で、結局その首が今も大手町でブチギレてるわけやな</t>
         </is>
       </c>
-      <c r="C146" s="2" t="inlineStr">
-        <is>
-          <t>スレ②</t>
-        </is>
-      </c>
-      <c r="D146" s="2" t="inlineStr">
-        <is>
-          <t>57</t>
-        </is>
-      </c>
-    </row>
-    <row r="147">
-      <c r="A147" s="2" t="inlineStr">
-        <is>
-          <t>男性C</t>
-        </is>
-      </c>
-      <c r="B147" s="3" t="inlineStr">
+      <c r="C157" s="2" t="inlineStr">
+        <is>
+          <t>スレ②</t>
+        </is>
+      </c>
+      <c r="D157" s="2" t="inlineStr">
+        <is>
+          <t>62</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="2" t="inlineStr">
+        <is>
+          <t>男性C下</t>
+        </is>
+      </c>
+      <c r="B158" s="3" t="inlineStr">
         <is>
           <t>千年たっても一等地から動かんあたり、ある意味いまだに関東の主やってるとも言えるわ</t>
         </is>
       </c>
-      <c r="C147" s="2" t="inlineStr">
-        <is>
-          <t>スレ②</t>
-        </is>
-      </c>
-      <c r="D147" s="2" t="inlineStr">
-        <is>
-          <t>58</t>
-        </is>
-      </c>
-    </row>
-    <row r="148">
-      <c r="A148" s="2" t="inlineStr">
-        <is>
-          <t>女性D下</t>
-        </is>
-      </c>
-      <c r="B148" s="3" t="inlineStr">
+      <c r="C158" s="2" t="inlineStr">
+        <is>
+          <t>スレ②</t>
+        </is>
+      </c>
+      <c r="D158" s="2" t="inlineStr">
+        <is>
+          <t>63</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="2" t="inlineStr">
+        <is>
+          <t>女性D</t>
+        </is>
+      </c>
+      <c r="B159" s="3" t="inlineStr">
         <is>
           <t>うまいこと言うやん</t>
         </is>
       </c>
-      <c r="C148" s="2" t="inlineStr">
-        <is>
-          <t>スレ②</t>
-        </is>
-      </c>
-      <c r="D148" s="2" t="inlineStr">
-        <is>
-          <t>59</t>
-        </is>
-      </c>
-    </row>
-    <row r="149">
-      <c r="A149" s="2" t="inlineStr">
+      <c r="C159" s="2" t="inlineStr">
+        <is>
+          <t>スレ②</t>
+        </is>
+      </c>
+      <c r="D159" s="2" t="inlineStr">
+        <is>
+          <t>64</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="2" t="inlineStr">
         <is>
           <t>男性E</t>
         </is>
       </c>
-      <c r="B149" s="3" t="inlineStr">
+      <c r="B160" s="3" t="inlineStr">
         <is>
           <t>ワイ明日大手町で乗り換えあるし、ちゃんと拝んどくわ。将門さん祟らんといてな</t>
         </is>
       </c>
-      <c r="C149" s="2" t="inlineStr">
-        <is>
-          <t>スレ②</t>
-        </is>
-      </c>
-      <c r="D149" s="2" t="inlineStr">
-        <is>
-          <t>60</t>
-        </is>
-      </c>
-    </row>
-    <row r="150">
-      <c r="A150" s="2" t="inlineStr">
+      <c r="C160" s="2" t="inlineStr">
+        <is>
+          <t>スレ②</t>
+        </is>
+      </c>
+      <c r="D160" s="2" t="inlineStr">
+        <is>
+          <t>65</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="2" t="inlineStr">
         <is>
           <t>解説者</t>
         </is>
       </c>
-      <c r="B150" s="3" t="inlineStr">
+      <c r="B161" s="3" t="inlineStr">
         <is>
           <t>本日はここまで。</t>
         </is>
       </c>
-      <c r="C150" s="2" t="inlineStr">
+      <c r="C161" s="2" t="inlineStr">
         <is>
           <t>締め</t>
         </is>
       </c>
-      <c r="D150" s="2" t="inlineStr">
+      <c r="D161" s="2" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
     </row>
-    <row r="151">
-      <c r="A151" s="2" t="inlineStr">
+    <row r="162">
+      <c r="A162" s="2" t="inlineStr">
         <is>
           <t>解説者</t>
         </is>
       </c>
-      <c r="B151" s="3" t="inlineStr">
+      <c r="B162" s="3" t="inlineStr">
         <is>
           <t>今回は、平将門の祟りについての
 さまざまな議論を見てきたが、
 いかがだっただろうか？</t>
         </is>
       </c>
-      <c r="C151" s="2" t="inlineStr">
+      <c r="C162" s="2" t="inlineStr">
         <is>
           <t>締め</t>
         </is>
       </c>
-      <c r="D151" s="2" t="inlineStr">
+      <c r="D162" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
     </row>
-    <row r="152">
-      <c r="A152" s="2" t="inlineStr">
+    <row r="163">
+      <c r="A163" s="2" t="inlineStr">
         <is>
           <t>解説者</t>
         </is>
       </c>
-      <c r="B152" s="3" t="inlineStr">
+      <c r="B163" s="3" t="inlineStr">
         <is>
           <t>2ちゃんねるの歴史オタクたちの
 議論を見ていると、</t>
         </is>
       </c>
-      <c r="C152" s="2" t="inlineStr">
+      <c r="C163" s="2" t="inlineStr">
         <is>
           <t>締め</t>
         </is>
       </c>
-      <c r="D152" s="2" t="inlineStr">
+      <c r="D163" s="2" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
     </row>
-    <row r="153">
-      <c r="A153" s="2" t="inlineStr">
+    <row r="164">
+      <c r="A164" s="2" t="inlineStr">
         <is>
           <t>解説者</t>
         </is>
       </c>
-      <c r="B153" s="3" t="inlineStr">
+      <c r="B164" s="3" t="inlineStr">
         <is>
           <t>将門は単なる祟り神ではなく、
 時代に真っ向から立ち向かって果てた反骨の武将であり、
@@ -3843,59 +4085,59 @@
 畏れと敬いを同時に集め続けているのだと思えた。</t>
         </is>
       </c>
-      <c r="C153" s="2" t="inlineStr">
+      <c r="C164" s="2" t="inlineStr">
         <is>
           <t>締め</t>
         </is>
       </c>
-      <c r="D153" s="2" t="inlineStr">
+      <c r="D164" s="2" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
     </row>
-    <row r="154">
-      <c r="A154" s="2" t="inlineStr">
+    <row r="165">
+      <c r="A165" s="2" t="inlineStr">
         <is>
           <t>解説者</t>
         </is>
       </c>
-      <c r="B154" s="3" t="inlineStr">
+      <c r="B165" s="3" t="inlineStr">
         <is>
           <t>今回の動画について他の意見や
 感想があったらぜひコメントで教えてね！</t>
         </is>
       </c>
-      <c r="C154" s="2" t="inlineStr">
+      <c r="C165" s="2" t="inlineStr">
         <is>
           <t>締め</t>
         </is>
       </c>
-      <c r="D154" s="2" t="inlineStr">
+      <c r="D165" s="2" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
     </row>
-    <row r="155">
-      <c r="A155" s="2" t="inlineStr">
+    <row r="166">
+      <c r="A166" s="2" t="inlineStr">
         <is>
           <t>解説者</t>
         </is>
       </c>
-      <c r="B155" s="3" t="inlineStr">
+      <c r="B166" s="3" t="inlineStr">
         <is>
           <t>他にも歴史にまつわる情報をまとめた
 動画が満載なので、ぜひ見てみてくださいね。
 ご視聴ありがとうございました！</t>
         </is>
       </c>
-      <c r="C155" s="2" t="inlineStr">
+      <c r="C166" s="2" t="inlineStr">
         <is>
           <t>締め</t>
         </is>
       </c>
-      <c r="D155" s="2" t="inlineStr">
+      <c r="D166" s="2" t="inlineStr">
         <is>
           <t>6</t>
         </is>

</xml_diff>

<commit_message>
auto: 2026-06-17 16:18 (4件)
</commit_message>
<xml_diff>
--- a/01_プロジェクト/YouTube/創作スレ下書き/2026-06-17_平将門の祟り_台本.xlsx
+++ b/01_プロジェクト/YouTube/創作スレ下書き/2026-06-17_平将門の祟り_台本.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D166"/>
+  <dimension ref="A1:D169"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2031,7 +2031,7 @@
       </c>
       <c r="B72" s="3" t="inlineStr">
         <is>
-          <t>ここ大事なんやけど、将門はただ恐れられただけちゃうくて、もともとは関東の民にとっては英雄寄りの存在やったんよ。重い負担やら国府の横暴に苦しむ坂東の人らからしたら、中央に盾突いて「東は俺らで治める」ってやってのけた将門は反骨のシンボルやった。だからこそ討たれたあとも、祟り神として畏れられつつ土地の守り神として手厚く祀られ続けた、っていう二面性があるわけや</t>
+          <t>ついでに言うと、将門を祀る神田明神の神田祭は、今も山王祭と並ぶ江戸三大祭のひとつでな。将門は江戸の総鎮守として庶民にめちゃくちゃ愛されてきたんよ。怨霊として恐れられた男が、江戸っ子の誇りの祭の主役になっとるんやから、畏れと信仰なんて紙一重やなって思うわ</t>
         </is>
       </c>
       <c r="C72" s="2" t="inlineStr">
@@ -2048,12 +2048,12 @@
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
         <is>
-          <t>男性C下</t>
+          <t>男性C大</t>
         </is>
       </c>
       <c r="B73" s="3" t="inlineStr">
         <is>
-          <t>ただの怨霊ちゃうくて元はヒーローなんやな</t>
+          <t>ここ大事なんやけど、将門はただ恐れられただけちゃうくて、もともとは関東の民にとっては英雄寄りの存在やったんよ。重い負担やら国府の横暴に苦しむ坂東の人らからしたら、中央に盾突いて「東は俺らで治める」ってやってのけた将門は反骨のシンボルやった。だからこそ討たれたあとも、祟り神として畏れられつつ土地の守り神として手厚く祀られ続けた、っていう二面性があるわけや</t>
         </is>
       </c>
       <c r="C73" s="2" t="inlineStr">
@@ -2070,12 +2070,12 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>女性D</t>
+          <t>女性D下</t>
         </is>
       </c>
       <c r="B74" s="3" t="inlineStr">
         <is>
-          <t>結局さ、全部"そういうことにしとこ"の後付けやろ。因果の証拠なんか無いやん</t>
+          <t>ただの怨霊ちゃうくて元はヒーローなんやな</t>
         </is>
       </c>
       <c r="C74" s="2" t="inlineStr">
@@ -2097,7 +2097,7 @@
       </c>
       <c r="B75" s="3" t="inlineStr">
         <is>
-          <t>信者乙、ぜんぶ偶然や</t>
+          <t>怨霊を祀る祭で江戸三大祭って、考えたら相当パンチ効いとるな</t>
         </is>
       </c>
       <c r="C75" s="2" t="inlineStr">
@@ -2114,12 +2114,12 @@
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>男性A下</t>
+          <t>男性A</t>
         </is>
       </c>
       <c r="B76" s="3" t="inlineStr">
         <is>
-          <t>まあ祟りに証拠もへったくれもないわな、そこは認める</t>
+          <t>結局さ、全部"そういうことにしとこ"の後付けやろ。因果の証拠なんか無いやん</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
@@ -2141,7 +2141,7 @@
       </c>
       <c r="B77" s="3" t="inlineStr">
         <is>
-          <t>証拠ないのに国家プロジェクトが二回もどかすのやめてる時点で、もう実質勝ちなんよ将門</t>
+          <t>信者乙、ぜんぶ偶然や</t>
         </is>
       </c>
       <c r="C77" s="2" t="inlineStr">
@@ -2163,7 +2163,7 @@
       </c>
       <c r="B78" s="3" t="inlineStr">
         <is>
-          <t>勝ち負けの話になってて草</t>
+          <t>まあ祟りに証拠もへったくれもないわな、そこは認める</t>
         </is>
       </c>
       <c r="C78" s="2" t="inlineStr">
@@ -2185,7 +2185,7 @@
       </c>
       <c r="B79" s="3" t="inlineStr">
         <is>
-          <t>山手線が将門の祟りを抑える結界として作られたって都市伝説もあるよな</t>
+          <t>証拠ないのに国家プロジェクトが二回もどかすのやめてる時点で、もう実質勝ちなんよ将門</t>
         </is>
       </c>
       <c r="C79" s="2" t="inlineStr">
@@ -2202,12 +2202,12 @@
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>男性E</t>
+          <t>男性E下</t>
         </is>
       </c>
       <c r="B80" s="3" t="inlineStr">
         <is>
-          <t>それは嘘らしいで、結界説は後から誰かが言い出したやつや</t>
+          <t>勝ち負けの話になってて草</t>
         </is>
       </c>
       <c r="C80" s="2" t="inlineStr">
@@ -2229,7 +2229,7 @@
       </c>
       <c r="B81" s="3" t="inlineStr">
         <is>
-          <t>なんや嘘なんか</t>
+          <t>山手線が将門の祟りを抑える結界として作られたって都市伝説もあるよな</t>
         </is>
       </c>
       <c r="C81" s="2" t="inlineStr">
@@ -2251,7 +2251,7 @@
       </c>
       <c r="B82" s="3" t="inlineStr">
         <is>
-          <t>嘘か本当か分からんのが一番こわいんよこの人。で、そもそも将門ってなんで反乱なんか起こしたん？怨霊の部分しか知らんわ</t>
+          <t>それは嘘らしいで、結界説は後から誰かが言い出したやつや</t>
         </is>
       </c>
       <c r="C82" s="2" t="inlineStr">
@@ -2273,7 +2273,7 @@
       </c>
       <c r="B83" s="3" t="inlineStr">
         <is>
-          <t>新皇名乗って関東独立しようとしたやべえ奴やぞ</t>
+          <t>なんや嘘なんか</t>
         </is>
       </c>
       <c r="C83" s="2" t="inlineStr">
@@ -2290,150 +2290,150 @@
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
+          <t>女性D</t>
+        </is>
+      </c>
+      <c r="B84" s="3" t="inlineStr">
+        <is>
+          <t>嘘か本当か分からんのが一番こわいんよこの人。で、そもそも将門ってなんで反乱なんか起こしたん？怨霊の部分しか知らんわ</t>
+        </is>
+      </c>
+      <c r="C84" s="2" t="inlineStr">
+        <is>
+          <t>スレ①</t>
+        </is>
+      </c>
+      <c r="D84" s="2" t="inlineStr">
+        <is>
+          <t>69</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="inlineStr">
+        <is>
+          <t>男性E</t>
+        </is>
+      </c>
+      <c r="B85" s="3" t="inlineStr">
+        <is>
+          <t>新皇名乗って関東独立しようとしたやべえ奴やぞ</t>
+        </is>
+      </c>
+      <c r="C85" s="2" t="inlineStr">
+        <is>
+          <t>スレ①</t>
+        </is>
+      </c>
+      <c r="D85" s="2" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="inlineStr">
+        <is>
           <t>解説者</t>
         </is>
       </c>
-      <c r="B84" s="3" t="inlineStr">
+      <c r="B86" s="3" t="inlineStr">
         <is>
           <t>ここまでは、
 平将門の首塚にまつわる祟りの噂について
 さまざまな議論を見てきたが、</t>
         </is>
       </c>
-      <c r="C84" s="2" t="inlineStr">
+      <c r="C86" s="2" t="inlineStr">
         <is>
           <t>前置き</t>
         </is>
       </c>
-      <c r="D84" s="2" t="inlineStr">
+      <c r="D86" s="2" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
     </row>
-    <row r="85">
-      <c r="A85" s="2" t="inlineStr">
+    <row r="87">
+      <c r="A87" s="2" t="inlineStr">
         <is>
           <t>解説者</t>
         </is>
       </c>
-      <c r="B85" s="3" t="inlineStr">
+      <c r="B87" s="3" t="inlineStr">
         <is>
           <t>「そもそも将門は何をして、
 ここまで恐れられる存在になったの？」
 と、肝心の生涯に疑問を持つ者も現れた。</t>
         </is>
       </c>
-      <c r="C85" s="2" t="inlineStr">
+      <c r="C87" s="2" t="inlineStr">
         <is>
           <t>前置き</t>
         </is>
       </c>
-      <c r="D85" s="2" t="inlineStr">
+      <c r="D87" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
     </row>
-    <row r="86">
-      <c r="A86" s="2" t="inlineStr">
+    <row r="88">
+      <c r="A88" s="2" t="inlineStr">
         <is>
           <t>解説者</t>
         </is>
       </c>
-      <c r="B86" s="3" t="inlineStr">
+      <c r="B88" s="3" t="inlineStr">
         <is>
           <t>たしかに、千年も祟りが語り継がれる怨霊が、
 どうやって生まれたのかは気になるところだ。</t>
         </is>
       </c>
-      <c r="C86" s="2" t="inlineStr">
+      <c r="C88" s="2" t="inlineStr">
         <is>
           <t>前置き</t>
         </is>
       </c>
-      <c r="D86" s="2" t="inlineStr">
+      <c r="D88" s="2" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
     </row>
-    <row r="87">
-      <c r="A87" s="2" t="inlineStr">
+    <row r="89">
+      <c r="A89" s="2" t="inlineStr">
         <is>
           <t>解説者</t>
         </is>
       </c>
-      <c r="B87" s="3" t="inlineStr">
+      <c r="B89" s="3" t="inlineStr">
         <is>
           <t>引き続き、2ちゃんねるの歴史オタクたちの
 議論を見ていこう。</t>
         </is>
       </c>
-      <c r="C87" s="2" t="inlineStr">
+      <c r="C89" s="2" t="inlineStr">
         <is>
           <t>前置き</t>
         </is>
       </c>
-      <c r="D87" s="2" t="inlineStr">
+      <c r="D89" s="2" t="inlineStr">
         <is>
           <t>4</t>
-        </is>
-      </c>
-    </row>
-    <row r="88">
-      <c r="A88" s="2" t="inlineStr">
-        <is>
-          <t>男性A</t>
-        </is>
-      </c>
-      <c r="B88" s="3" t="inlineStr">
-        <is>
-          <t>平将門「これからは俺が東の天皇やるわ」朝廷「は？」</t>
-        </is>
-      </c>
-      <c r="C88" s="2" t="inlineStr">
-        <is>
-          <t>スレ②</t>
-        </is>
-      </c>
-      <c r="D88" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-    </row>
-    <row r="89">
-      <c r="A89" s="2" t="inlineStr">
-        <is>
-          <t>女性B下</t>
-        </is>
-      </c>
-      <c r="B89" s="3" t="inlineStr">
-        <is>
-          <t>出た自称新皇ｗ</t>
-        </is>
-      </c>
-      <c r="C89" s="2" t="inlineStr">
-        <is>
-          <t>スレ②</t>
-        </is>
-      </c>
-      <c r="D89" s="2" t="inlineStr">
-        <is>
-          <t>2</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>男性C</t>
+          <t>男性A</t>
         </is>
       </c>
       <c r="B90" s="3" t="inlineStr">
         <is>
-          <t>名乗ったもん勝ちかよ</t>
+          <t>平将門「これからは俺が東の天皇やるわ」朝廷「は？」</t>
         </is>
       </c>
       <c r="C90" s="2" t="inlineStr">
@@ -2443,19 +2443,19 @@
       </c>
       <c r="D90" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
         <is>
-          <t>女性D</t>
+          <t>女性B下</t>
         </is>
       </c>
       <c r="B91" s="3" t="inlineStr">
         <is>
-          <t>関東の田舎で勝手に天皇名乗ったやべえ人やろ</t>
+          <t>出た自称新皇ｗ</t>
         </is>
       </c>
       <c r="C91" s="2" t="inlineStr">
@@ -2465,19 +2465,19 @@
       </c>
       <c r="D91" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>男性E</t>
+          <t>男性C</t>
         </is>
       </c>
       <c r="B92" s="3" t="inlineStr">
         <is>
-          <t>結局その新皇とやらも2か月で終わった負け犬やん、持ち上げる要素ある？</t>
+          <t>名乗ったもん勝ちかよ</t>
         </is>
       </c>
       <c r="C92" s="2" t="inlineStr">
@@ -2487,19 +2487,19 @@
       </c>
       <c r="D92" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
         <is>
-          <t>男性A</t>
+          <t>女性D</t>
         </is>
       </c>
       <c r="B93" s="3" t="inlineStr">
         <is>
-          <t>怨霊の話は聞くけど何した人かは正直知らんわ</t>
+          <t>関東の田舎で勝手に天皇名乗ったやべえ人やろ</t>
         </is>
       </c>
       <c r="C93" s="2" t="inlineStr">
@@ -2509,19 +2509,19 @@
       </c>
       <c r="D93" s="2" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>4</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>女性B</t>
+          <t>男性E</t>
         </is>
       </c>
       <c r="B94" s="3" t="inlineStr">
         <is>
-          <t>で、結局こいつ何がしたかったん</t>
+          <t>結局その新皇とやらも2か月で終わった負け犬やん、持ち上げる要素ある？</t>
         </is>
       </c>
       <c r="C94" s="2" t="inlineStr">
@@ -2531,19 +2531,19 @@
       </c>
       <c r="D94" s="2" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
         <is>
-          <t>男性C</t>
+          <t>男性A</t>
         </is>
       </c>
       <c r="B95" s="3" t="inlineStr">
         <is>
-          <t>中央に喧嘩売って負けた人や、それ以上でもそれ以下でもなくない？</t>
+          <t>怨霊の話は聞くけど何した人かは正直知らんわ</t>
         </is>
       </c>
       <c r="C95" s="2" t="inlineStr">
@@ -2553,19 +2553,19 @@
       </c>
       <c r="D95" s="2" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>6</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>女性D大</t>
+          <t>女性B</t>
         </is>
       </c>
       <c r="B96" s="3" t="inlineStr">
         <is>
-          <t>それがな、最初っから天皇に盾突こうとしてたわけちゃうんよ。スタートはただの一族内のもめ事や。関東の平氏一門で、伯父さんらと土地や縁談がらみの私闘をやっとった、いわば身内ゲンカからの叩き上げやねん。それが勝ち続けるうちに、どんどん引くに引けん大ごとになってってもうた</t>
+          <t>で、結局こいつ何がしたかったん</t>
         </is>
       </c>
       <c r="C96" s="2" t="inlineStr">
@@ -2575,19 +2575,19 @@
       </c>
       <c r="D96" s="2" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>7</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
         <is>
-          <t>男性E</t>
+          <t>男性C</t>
         </is>
       </c>
       <c r="B97" s="3" t="inlineStr">
         <is>
-          <t>ファッ最初は身内ゲンカなんか</t>
+          <t>中央に喧嘩売って負けた人や、それ以上でもそれ以下でもなくない？</t>
         </is>
       </c>
       <c r="C97" s="2" t="inlineStr">
@@ -2597,19 +2597,19 @@
       </c>
       <c r="D97" s="2" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>8</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>男性A</t>
+          <t>女性D大</t>
         </is>
       </c>
       <c r="B98" s="3" t="inlineStr">
         <is>
-          <t>そっからどうやって天皇になんねん</t>
+          <t>それがな、最初っから天皇に盾突こうとしてたわけちゃうんよ。スタートはただの一族内のもめ事や。関東の平氏一門で、伯父さんらと土地や縁談がらみの私闘をやっとった、いわば身内ゲンカからの叩き上げやねん。それが勝ち続けるうちに、どんどん引くに引けん大ごとになってってもうた</t>
         </is>
       </c>
       <c r="C98" s="2" t="inlineStr">
@@ -2619,19 +2619,19 @@
       </c>
       <c r="D98" s="2" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>9</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
         <is>
-          <t>女性B下</t>
+          <t>男性E</t>
         </is>
       </c>
       <c r="B99" s="3" t="inlineStr">
         <is>
-          <t>ヤンキーの抗争がいつの間にか国盗りになる漫画みたいや</t>
+          <t>ファッ最初は身内ゲンカなんか</t>
         </is>
       </c>
       <c r="C99" s="2" t="inlineStr">
@@ -2641,19 +2641,19 @@
       </c>
       <c r="D99" s="2" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>男性C大</t>
+          <t>男性A</t>
         </is>
       </c>
       <c r="B100" s="3" t="inlineStr">
         <is>
-          <t>そもそも将門の出自も知っとくとええで。あいつ桓武天皇の血を引く桓武平氏で、高望王の孫にあたる名門の出やねん。若い頃は京都に上って摂関家に奉公しとった時期もあって、決して田舎のチンピラちゃう。中央の作法も権力の構造も知った上で関東に戻って、結局その中央に弓を引くことになったわけや</t>
+          <t>そっからどうやって天皇になんねん</t>
         </is>
       </c>
       <c r="C100" s="2" t="inlineStr">
@@ -2663,19 +2663,19 @@
       </c>
       <c r="D100" s="2" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>11</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
         <is>
-          <t>女性D</t>
+          <t>女性B下</t>
         </is>
       </c>
       <c r="B101" s="3" t="inlineStr">
         <is>
-          <t>元エリートが地元で反乱とか厨二すぎる</t>
+          <t>ヤンキーの抗争がいつの間にか国盗りになる漫画みたいや</t>
         </is>
       </c>
       <c r="C101" s="2" t="inlineStr">
@@ -2685,19 +2685,19 @@
       </c>
       <c r="D101" s="2" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>12</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
         <is>
-          <t>男性E下</t>
+          <t>男性C大</t>
         </is>
       </c>
       <c r="B102" s="3" t="inlineStr">
         <is>
-          <t>中身を知ってる奴が反旗ひるがえすのが一番こわいやつやん</t>
+          <t>そもそも将門の出自も知っとくとええで。あいつ桓武天皇の血を引く桓武平氏で、高望王の孫にあたる名門の出やねん。若い頃は京都に上って摂関家に奉公しとった時期もあって、決して田舎のチンピラちゃう。中央の作法も権力の構造も知った上で関東に戻って、結局その中央に弓を引くことになったわけや</t>
         </is>
       </c>
       <c r="C102" s="2" t="inlineStr">
@@ -2707,19 +2707,19 @@
       </c>
       <c r="D102" s="2" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>13</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
         <is>
-          <t>男性A大</t>
+          <t>女性D</t>
         </is>
       </c>
       <c r="B103" s="3" t="inlineStr">
         <is>
-          <t>ちな将門の地盤は下総の猿島あたりでな、当時の坂東は朝廷の目が届きにくい辺境で、しかも良馬の産地やった。だから機動力のある騎馬の武士団を抱えやすくて、中央から来た役人よりも地元で腕の立つ将門のほうが頼りにされとった。そういう土壌があったからこそ、一介の豪族が関東一円を呑み込むなんて芸当ができたわけや</t>
+          <t>元エリートが地元で反乱とか厨二すぎる</t>
         </is>
       </c>
       <c r="C103" s="2" t="inlineStr">
@@ -2729,19 +2729,19 @@
       </c>
       <c r="D103" s="2" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>14</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
         <is>
-          <t>女性B下</t>
+          <t>男性E下</t>
         </is>
       </c>
       <c r="B104" s="3" t="inlineStr">
         <is>
-          <t>馬かよ、そら強いわけや</t>
+          <t>中身を知ってる奴が反旗ひるがえすのが一番こわいやつやん</t>
         </is>
       </c>
       <c r="C104" s="2" t="inlineStr">
@@ -2751,19 +2751,19 @@
       </c>
       <c r="D104" s="2" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>15</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
         <is>
-          <t>男性C大</t>
+          <t>男性A大</t>
         </is>
       </c>
       <c r="B105" s="3" t="inlineStr">
         <is>
-          <t>で、私闘で官側の人間ともやり合ううちに、今度は朝廷の出先の国府とぶつかってまう。勢いで常陸の国府を攻め落として、国の実印にあたる印鑰まで奪ってもうた。これ当時やと完全に一線を越えた行為で、国に弓を引いた賊って扱いになる。もう後戻りでけへんとこまで行ったわけや</t>
+          <t>ちな将門の地盤は下総の猿島あたりでな、当時の坂東は朝廷の目が届きにくい辺境で、しかも良馬の産地やった。だから機動力のある騎馬の武士団を抱えやすくて、中央から来た役人よりも地元で腕の立つ将門のほうが頼りにされとった。そういう土壌があったからこそ、一介の豪族が関東一円を呑み込むなんて芸当ができたわけや</t>
         </is>
       </c>
       <c r="C105" s="2" t="inlineStr">
@@ -2773,19 +2773,19 @@
       </c>
       <c r="D105" s="2" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>16</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
         <is>
-          <t>女性D</t>
+          <t>女性B下</t>
         </is>
       </c>
       <c r="B106" s="3" t="inlineStr">
         <is>
-          <t>印鑰ってなんや</t>
+          <t>馬かよ、そら強いわけや</t>
         </is>
       </c>
       <c r="C106" s="2" t="inlineStr">
@@ -2795,19 +2795,19 @@
       </c>
       <c r="D106" s="2" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>17</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
         <is>
-          <t>男性E下</t>
+          <t>男性C大</t>
         </is>
       </c>
       <c r="B107" s="3" t="inlineStr">
         <is>
-          <t>国を動かす実印とハンコ箱みたいなもんや。それ奪うって今でいう役所まるごと乗っ取るレベルやぞ</t>
+          <t>で、私闘で官側の人間ともやり合ううちに、今度は朝廷の出先の国府とぶつかってまう。勢いで常陸の国府を攻め落として、国の実印にあたる印鑰まで奪ってもうた。これ当時やと完全に一線を越えた行為で、国に弓を引いた賊って扱いになる。もう後戻りでけへんとこまで行ったわけや</t>
         </is>
       </c>
       <c r="C107" s="2" t="inlineStr">
@@ -2817,159 +2817,159 @@
       </c>
       <c r="D107" s="2" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>18</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
         <is>
+          <t>女性D</t>
+        </is>
+      </c>
+      <c r="B108" s="3" t="inlineStr">
+        <is>
+          <t>印鑰ってなんや</t>
+        </is>
+      </c>
+      <c r="C108" s="2" t="inlineStr">
+        <is>
+          <t>スレ②</t>
+        </is>
+      </c>
+      <c r="D108" s="2" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="2" t="inlineStr">
+        <is>
+          <t>男性E下</t>
+        </is>
+      </c>
+      <c r="B109" s="3" t="inlineStr">
+        <is>
+          <t>国を動かす実印とハンコ箱みたいなもんや。それ奪うって今でいう役所まるごと乗っ取るレベルやぞ</t>
+        </is>
+      </c>
+      <c r="C109" s="2" t="inlineStr">
+        <is>
+          <t>スレ②</t>
+        </is>
+      </c>
+      <c r="D109" s="2" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="2" t="inlineStr">
+        <is>
           <t>解説者</t>
         </is>
       </c>
-      <c r="B108" s="3" t="inlineStr">
+      <c r="B110" s="3" t="inlineStr">
         <is>
           <t>印鑰とは、
 古代から中世の役所で使われた、
 国の実印と倉の鍵を指す言葉である。</t>
         </is>
       </c>
-      <c r="C108" s="2" t="inlineStr">
+      <c r="C110" s="2" t="inlineStr">
         <is>
           <t>解説：印鑰</t>
         </is>
       </c>
-      <c r="D108" s="2" t="inlineStr">
+      <c r="D110" s="2" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
     </row>
-    <row r="109">
-      <c r="A109" s="2" t="inlineStr">
+    <row r="111">
+      <c r="A111" s="2" t="inlineStr">
         <is>
           <t>解説者</t>
         </is>
       </c>
-      <c r="B109" s="3" t="inlineStr">
+      <c r="B111" s="3" t="inlineStr">
         <is>
           <t>印は公文書に押す国家の正式な印鑑、
 鑰は税として集めた米などを納めた
 正倉の鍵を意味する。</t>
         </is>
       </c>
-      <c r="C109" s="2" t="inlineStr">
+      <c r="C111" s="2" t="inlineStr">
         <is>
           <t>解説：印鑰</t>
         </is>
       </c>
-      <c r="D109" s="2" t="inlineStr">
+      <c r="D111" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
     </row>
-    <row r="110">
-      <c r="A110" s="2" t="inlineStr">
+    <row r="112">
+      <c r="A112" s="2" t="inlineStr">
         <is>
           <t>解説者</t>
         </is>
       </c>
-      <c r="B110" s="3" t="inlineStr">
+      <c r="B112" s="3" t="inlineStr">
         <is>
           <t>つまり印鑰を押さえることは、
 その国の行政と財産をまとめて
 手中に収めることに等しかった。</t>
         </is>
       </c>
-      <c r="C110" s="2" t="inlineStr">
+      <c r="C112" s="2" t="inlineStr">
         <is>
           <t>解説：印鑰</t>
         </is>
       </c>
-      <c r="D110" s="2" t="inlineStr">
+      <c r="D112" s="2" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
     </row>
-    <row r="111">
-      <c r="A111" s="2" t="inlineStr">
+    <row r="113">
+      <c r="A113" s="2" t="inlineStr">
         <is>
           <t>解説者</t>
         </is>
       </c>
-      <c r="B111" s="3" t="inlineStr">
+      <c r="B113" s="3" t="inlineStr">
         <is>
           <t>将門が国府を襲ってこれを奪った行為は、
 朝廷の支配そのものに正面から
 弓を引いたことを意味するのである。</t>
         </is>
       </c>
-      <c r="C111" s="2" t="inlineStr">
+      <c r="C113" s="2" t="inlineStr">
         <is>
           <t>解説：印鑰</t>
         </is>
       </c>
-      <c r="D111" s="2" t="inlineStr">
+      <c r="D113" s="2" t="inlineStr">
         <is>
           <t>4</t>
-        </is>
-      </c>
-    </row>
-    <row r="112">
-      <c r="A112" s="2" t="inlineStr">
-        <is>
-          <t>男性A大</t>
-        </is>
-      </c>
-      <c r="B112" s="3" t="inlineStr">
-        <is>
-          <t>そっから勢いに乗った将門は、坂東、今でいう関東一帯の国府を次々落として、ほぼ関東全域を手中に収めてまう。各国の国司を追い出して、自前の人事で「ここからは俺が仕切る国や」ってやり始めた。地方の豪族が中央任命の役人をまとめて吹っ飛ばすって、当時前代未聞やってん</t>
-        </is>
-      </c>
-      <c r="C112" s="2" t="inlineStr">
-        <is>
-          <t>スレ②</t>
-        </is>
-      </c>
-      <c r="D112" s="2" t="inlineStr">
-        <is>
-          <t>21</t>
-        </is>
-      </c>
-    </row>
-    <row r="113">
-      <c r="A113" s="2" t="inlineStr">
-        <is>
-          <t>女性B下</t>
-        </is>
-      </c>
-      <c r="B113" s="3" t="inlineStr">
-        <is>
-          <t>関東まるごとはやりすぎやろ</t>
-        </is>
-      </c>
-      <c r="C113" s="2" t="inlineStr">
-        <is>
-          <t>スレ②</t>
-        </is>
-      </c>
-      <c r="D113" s="2" t="inlineStr">
-        <is>
-          <t>22</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
         <is>
-          <t>男性C</t>
+          <t>男性A大</t>
         </is>
       </c>
       <c r="B114" s="3" t="inlineStr">
         <is>
-          <t>もう完全に独立国家やん</t>
+          <t>そっから勢いに乗った将門は、坂東、今でいう関東一帯の国府を次々落として、ほぼ関東全域を手中に収めてまう。各国の国司を追い出して、自前の人事で「ここからは俺が仕切る国や」ってやり始めた。地方の豪族が中央任命の役人をまとめて吹っ飛ばすって、当時前代未聞やってん</t>
         </is>
       </c>
       <c r="C114" s="2" t="inlineStr">
@@ -2979,19 +2979,19 @@
       </c>
       <c r="D114" s="2" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>21</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
         <is>
-          <t>女性D</t>
+          <t>女性B下</t>
         </is>
       </c>
       <c r="B115" s="3" t="inlineStr">
         <is>
-          <t>で、調子乗って新皇宣言と</t>
+          <t>関東まるごとはやりすぎやろ</t>
         </is>
       </c>
       <c r="C115" s="2" t="inlineStr">
@@ -3001,19 +3001,19 @@
       </c>
       <c r="D115" s="2" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>22</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
         <is>
-          <t>男性E大</t>
+          <t>男性C</t>
         </is>
       </c>
       <c r="B116" s="3" t="inlineStr">
         <is>
-          <t>そう、ここで「新皇」、つまり新しい天皇を名乗る。伝説やと八幡神のお告げで位を授かったってことになっとるけど、要は京都の天皇とは別に、東国に自分を頂点とした朝廷を立てようとしたわけや。関東に独立政権を作るっていう、日本史でもなかなかおらんスケールの反逆やねん</t>
+          <t>もう完全に独立国家やん</t>
         </is>
       </c>
       <c r="C116" s="2" t="inlineStr">
@@ -3023,19 +3023,19 @@
       </c>
       <c r="D116" s="2" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>23</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
         <is>
-          <t>男性A</t>
+          <t>女性D</t>
         </is>
       </c>
       <c r="B117" s="3" t="inlineStr">
         <is>
-          <t>八幡のお告げは草、自分で言うてるだけやろ知らんけど</t>
+          <t>で、調子乗って新皇宣言と</t>
         </is>
       </c>
       <c r="C117" s="2" t="inlineStr">
@@ -3045,19 +3045,19 @@
       </c>
       <c r="D117" s="2" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>24</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
         <is>
-          <t>女性B</t>
+          <t>男性E大</t>
         </is>
       </c>
       <c r="B118" s="3" t="inlineStr">
         <is>
-          <t>神様持ち出すの強気すぎる</t>
+          <t>そう、ここで「新皇」、つまり新しい天皇を名乗る。伝説やと八幡神のお告げで位を授かったってことになっとるけど、要は京都の天皇とは別に、東国に自分を頂点とした朝廷を立てようとしたわけや。関東に独立政権を作るっていう、日本史でもなかなかおらんスケールの反逆やねん</t>
         </is>
       </c>
       <c r="C118" s="2" t="inlineStr">
@@ -3067,19 +3067,19 @@
       </c>
       <c r="D118" s="2" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>25</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
         <is>
-          <t>男性C</t>
+          <t>男性A</t>
         </is>
       </c>
       <c r="B119" s="3" t="inlineStr">
         <is>
-          <t>正直そこは盛りやろ、神託とか後付けくさいわ</t>
+          <t>八幡のお告げは草、自分で言うてるだけやろ知らんけど</t>
         </is>
       </c>
       <c r="C119" s="2" t="inlineStr">
@@ -3089,19 +3089,19 @@
       </c>
       <c r="D119" s="2" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>26</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
         <is>
-          <t>女性D</t>
+          <t>女性B</t>
         </is>
       </c>
       <c r="B120" s="3" t="inlineStr">
         <is>
-          <t>で？神名乗ろうがすぐ討たれたんやから、結局ただの勘違いした田舎の暴れん坊やん</t>
+          <t>神様持ち出すの強気すぎる</t>
         </is>
       </c>
       <c r="C120" s="2" t="inlineStr">
@@ -3111,19 +3111,19 @@
       </c>
       <c r="D120" s="2" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>27</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
         <is>
-          <t>男性E下</t>
+          <t>男性C</t>
         </is>
       </c>
       <c r="B121" s="3" t="inlineStr">
         <is>
-          <t>勘違いで関東一国まとめられたら誰も苦労せんわ、そこは認めたれや</t>
+          <t>正直そこは盛りやろ、神託とか後付けくさいわ</t>
         </is>
       </c>
       <c r="C121" s="2" t="inlineStr">
@@ -3133,19 +3133,19 @@
       </c>
       <c r="D121" s="2" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>28</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
         <is>
-          <t>男性A</t>
+          <t>女性D</t>
         </is>
       </c>
       <c r="B122" s="3" t="inlineStr">
         <is>
-          <t>でもこんなん中央がブチギレて終わりやん</t>
+          <t>で？神名乗ろうがすぐ討たれたんやから、結局ただの勘違いした田舎の暴れん坊やん</t>
         </is>
       </c>
       <c r="C122" s="2" t="inlineStr">
@@ -3155,19 +3155,19 @@
       </c>
       <c r="D122" s="2" t="inlineStr">
         <is>
-          <t>31</t>
+          <t>29</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
         <is>
-          <t>女性B大</t>
+          <t>男性E下</t>
         </is>
       </c>
       <c r="B123" s="3" t="inlineStr">
         <is>
-          <t>そうなる。京都は将門を朝敵認定して追討令を出す。で、ここで動いたのが同じ関東の平貞盛と、下野の豪族やった藤原秀郷や。身内や近隣やった連中が討伐側に回って、将門包囲網が出来てまうわけや</t>
+          <t>勘違いで関東一国まとめられたら誰も苦労せんわ、そこは認めたれや</t>
         </is>
       </c>
       <c r="C123" s="2" t="inlineStr">
@@ -3177,19 +3177,19 @@
       </c>
       <c r="D123" s="2" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>30</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
         <is>
-          <t>男性C下</t>
+          <t>男性A</t>
         </is>
       </c>
       <c r="B124" s="3" t="inlineStr">
         <is>
-          <t>結局身内に討たれるんかい</t>
+          <t>でもこんなん中央がブチギレて終わりやん</t>
         </is>
       </c>
       <c r="C124" s="2" t="inlineStr">
@@ -3199,19 +3199,19 @@
       </c>
       <c r="D124" s="2" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>31</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
         <is>
-          <t>女性D</t>
+          <t>女性B大</t>
         </is>
       </c>
       <c r="B125" s="3" t="inlineStr">
         <is>
-          <t>関東の独立より自分の家のほうが大事って奴がおったわけやな</t>
+          <t>そうなる。京都は将門を朝敵認定して追討令を出す。で、ここで動いたのが同じ関東の平貞盛と、下野の豪族やった藤原秀郷や。身内や近隣やった連中が討伐側に回って、将門包囲網が出来てまうわけや</t>
         </is>
       </c>
       <c r="C125" s="2" t="inlineStr">
@@ -3221,19 +3221,19 @@
       </c>
       <c r="D125" s="2" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>32</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
         <is>
-          <t>男性E</t>
+          <t>男性C下</t>
         </is>
       </c>
       <c r="B126" s="3" t="inlineStr">
         <is>
-          <t>将門を討ったのって源氏の先祖やっけ？</t>
+          <t>結局身内に討たれるんかい</t>
         </is>
       </c>
       <c r="C126" s="2" t="inlineStr">
@@ -3243,19 +3243,19 @@
       </c>
       <c r="D126" s="2" t="inlineStr">
         <is>
-          <t>35</t>
+          <t>33</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
         <is>
-          <t>男性A下</t>
+          <t>女性D</t>
         </is>
       </c>
       <c r="B127" s="3" t="inlineStr">
         <is>
-          <t>ちゃう、討ったのは平貞盛と藤原秀郷や。源氏ちゃうから、そこ混同したらあかんで</t>
+          <t>関東の独立より自分の家のほうが大事って奴がおったわけやな</t>
         </is>
       </c>
       <c r="C127" s="2" t="inlineStr">
@@ -3265,19 +3265,19 @@
       </c>
       <c r="D127" s="2" t="inlineStr">
         <is>
-          <t>36</t>
+          <t>34</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
         <is>
-          <t>女性B</t>
+          <t>男性E</t>
         </is>
       </c>
       <c r="B128" s="3" t="inlineStr">
         <is>
-          <t>あっそうやったか、すまんね</t>
+          <t>将門を討ったのって源氏の先祖やっけ？</t>
         </is>
       </c>
       <c r="C128" s="2" t="inlineStr">
@@ -3287,19 +3287,19 @@
       </c>
       <c r="D128" s="2" t="inlineStr">
         <is>
-          <t>37</t>
+          <t>35</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
         <is>
-          <t>男性C大</t>
+          <t>男性A下</t>
         </is>
       </c>
       <c r="B129" s="3" t="inlineStr">
         <is>
-          <t>で、天慶3年、西暦940年に討伐軍とぶつかって、将門は敗れる。伝承やと、戦いの最中に飛んできた流れ矢が額に当たって、それが致命傷になって命を落としたって言われとる。新皇を名乗ってからわずか2か月ほどでの最期や。あれだけ関東を席巻したのに、終わりはほんま一瞬やった</t>
+          <t>ちゃう、討ったのは平貞盛と藤原秀郷や。源氏ちゃうから、そこ混同したらあかんで</t>
         </is>
       </c>
       <c r="C129" s="2" t="inlineStr">
@@ -3309,19 +3309,19 @@
       </c>
       <c r="D129" s="2" t="inlineStr">
         <is>
-          <t>38</t>
+          <t>36</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
         <is>
-          <t>女性D</t>
+          <t>女性B</t>
         </is>
       </c>
       <c r="B130" s="3" t="inlineStr">
         <is>
-          <t>2か月て短すぎやろ</t>
+          <t>あっそうやったか、すまんね</t>
         </is>
       </c>
       <c r="C130" s="2" t="inlineStr">
@@ -3331,19 +3331,19 @@
       </c>
       <c r="D130" s="2" t="inlineStr">
         <is>
-          <t>39</t>
+          <t>37</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
         <is>
-          <t>男性E</t>
+          <t>男性C大</t>
         </is>
       </c>
       <c r="B131" s="3" t="inlineStr">
         <is>
-          <t>天下取り損ねたというか、名乗っただけで終わったやんｗ</t>
+          <t>で、天慶3年、西暦940年に討伐軍とぶつかって、将門は敗れる。伝承やと、戦いの最中に飛んできた流れ矢が額に当たって、それが致命傷になって命を落としたって言われとる。新皇を名乗ってからわずか2か月ほどでの最期や。あれだけ関東を席巻したのに、終わりはほんま一瞬やった</t>
         </is>
       </c>
       <c r="C131" s="2" t="inlineStr">
@@ -3353,19 +3353,19 @@
       </c>
       <c r="D131" s="2" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>38</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
         <is>
-          <t>男性A大</t>
+          <t>女性D</t>
         </is>
       </c>
       <c r="B132" s="3" t="inlineStr">
         <is>
-          <t>その最期にも伝説があってな。将門は矢も通さんと評判の無敵の体で討伐軍が苦戦しとったけど、戦いの最中に陣の風向きが急に変わって、その隙に放たれた矢が額に当たったって話が残っとる。神がかった強さやのに、最後は風っていう運否天賦みたいなもんで決着した、っていうのがまた伝説を盛り上げとるんや</t>
+          <t>2か月て短すぎやろ</t>
         </is>
       </c>
       <c r="C132" s="2" t="inlineStr">
@@ -3375,19 +3375,19 @@
       </c>
       <c r="D132" s="2" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>39</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
         <is>
-          <t>女性B下</t>
+          <t>男性E</t>
         </is>
       </c>
       <c r="B133" s="3" t="inlineStr">
         <is>
-          <t>急に弱点が出てくるの少年漫画やん</t>
+          <t>天下取り損ねたというか、名乗っただけで終わったやんｗ</t>
         </is>
       </c>
       <c r="C133" s="2" t="inlineStr">
@@ -3397,19 +3397,19 @@
       </c>
       <c r="D133" s="2" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>40</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
         <is>
-          <t>男性C</t>
+          <t>男性A大</t>
         </is>
       </c>
       <c r="B134" s="3" t="inlineStr">
         <is>
-          <t>風で負けるラスボスすこｗ</t>
+          <t>その最期にも伝説があってな。将門は矢も通さんと評判の無敵の体で討伐軍が苦戦しとったけど、戦いの最中に陣の風向きが急に変わって、その隙に放たれた矢が額に当たったって話が残っとる。神がかった強さやのに、最後は風っていう運否天賦みたいなもんで決着した、っていうのがまた伝説を盛り上げとるんや</t>
         </is>
       </c>
       <c r="C134" s="2" t="inlineStr">
@@ -3419,19 +3419,19 @@
       </c>
       <c r="D134" s="2" t="inlineStr">
         <is>
-          <t>43</t>
+          <t>41</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
         <is>
-          <t>女性D大</t>
+          <t>女性B下</t>
         </is>
       </c>
       <c r="B135" s="3" t="inlineStr">
         <is>
-          <t>もういっこ有名なんが影武者伝説や。将門にはそっくりの影武者が何人もおって、本物を見分けられんかったけど、こめかみのあたりに本物だけ影が無かった、みたいな尾ひれが後世に付いとる。要は強すぎて普通には討てんかったっていう"負けたのが信じられん"空気が、こういう伝説を生んだわけやな</t>
+          <t>急に弱点が出てくるの少年漫画やん</t>
         </is>
       </c>
       <c r="C135" s="2" t="inlineStr">
@@ -3441,19 +3441,19 @@
       </c>
       <c r="D135" s="2" t="inlineStr">
         <is>
-          <t>44</t>
+          <t>42</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
         <is>
-          <t>男性E</t>
+          <t>男性C</t>
         </is>
       </c>
       <c r="B136" s="3" t="inlineStr">
         <is>
-          <t>影武者まで盛られるの大物の証や</t>
+          <t>風で負けるラスボスすこｗ</t>
         </is>
       </c>
       <c r="C136" s="2" t="inlineStr">
@@ -3463,19 +3463,19 @@
       </c>
       <c r="D136" s="2" t="inlineStr">
         <is>
-          <t>45</t>
+          <t>43</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
         <is>
-          <t>男性A</t>
+          <t>女性D大</t>
         </is>
       </c>
       <c r="B137" s="3" t="inlineStr">
         <is>
-          <t>そういや将門を祀っとる国王神社が茨城にあって、将門の三女が建てたって伝わっとるな。ワイ一回行ったけど、めっちゃ静かでええとこやった</t>
+          <t>もういっこ有名なんが影武者伝説や。将門にはそっくりの影武者が何人もおって、本物を見分けられんかったけど、こめかみのあたりに本物だけ影が無かった、みたいな尾ひれが後世に付いとる。要は強すぎて普通には討てんかったっていう"負けたのが信じられん"空気が、こういう伝説を生んだわけやな</t>
         </is>
       </c>
       <c r="C137" s="2" t="inlineStr">
@@ -3485,19 +3485,19 @@
       </c>
       <c r="D137" s="2" t="inlineStr">
         <is>
-          <t>46</t>
+          <t>44</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
         <is>
-          <t>女性B</t>
+          <t>男性E</t>
         </is>
       </c>
       <c r="B138" s="3" t="inlineStr">
         <is>
-          <t>大河で将門やらんのかな、昔の風と雲と虹と以来やろ</t>
+          <t>影武者まで盛られるの大物の証や</t>
         </is>
       </c>
       <c r="C138" s="2" t="inlineStr">
@@ -3507,19 +3507,19 @@
       </c>
       <c r="D138" s="2" t="inlineStr">
         <is>
-          <t>47</t>
+          <t>45</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
         <is>
-          <t>男性C</t>
+          <t>男性A</t>
         </is>
       </c>
       <c r="B139" s="3" t="inlineStr">
         <is>
-          <t>主役が朝敵やと今のNHKはやりにくいやろなあ</t>
+          <t>そういや将門を祀っとる国王神社が茨城にあって、将門の三女が建てたって伝わっとるな。ワイ一回行ったけど、めっちゃ静かでええとこやった</t>
         </is>
       </c>
       <c r="C139" s="2" t="inlineStr">
@@ -3529,19 +3529,19 @@
       </c>
       <c r="D139" s="2" t="inlineStr">
         <is>
-          <t>48</t>
+          <t>46</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
         <is>
-          <t>女性D</t>
+          <t>女性B</t>
         </is>
       </c>
       <c r="B140" s="3" t="inlineStr">
         <is>
-          <t>で、その首が飛ぶ伝説に繋がるわけやな</t>
+          <t>大河で将門やらんのかな、昔の風と雲と虹と以来やろ</t>
         </is>
       </c>
       <c r="C140" s="2" t="inlineStr">
@@ -3551,19 +3551,19 @@
       </c>
       <c r="D140" s="2" t="inlineStr">
         <is>
-          <t>49</t>
+          <t>47</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
         <is>
-          <t>男性E</t>
+          <t>男性C</t>
         </is>
       </c>
       <c r="B141" s="3" t="inlineStr">
         <is>
-          <t>そう、討たれた首は京都に送られて晒される。で、その首が夜に飛んで関東に戻った、っていうのが前半の祟りの話に繋がるんや</t>
+          <t>主役が朝敵やと今のNHKはやりにくいやろなあ</t>
         </is>
       </c>
       <c r="C141" s="2" t="inlineStr">
@@ -3573,19 +3573,19 @@
       </c>
       <c r="D141" s="2" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>48</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
         <is>
-          <t>男性A下</t>
+          <t>女性D</t>
         </is>
       </c>
       <c r="B142" s="3" t="inlineStr">
         <is>
-          <t>きれいに一周してて草</t>
+          <t>で、その首が飛ぶ伝説に繋がるわけやな</t>
         </is>
       </c>
       <c r="C142" s="2" t="inlineStr">
@@ -3595,19 +3595,19 @@
       </c>
       <c r="D142" s="2" t="inlineStr">
         <is>
-          <t>51</t>
+          <t>49</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
         <is>
-          <t>女性B</t>
+          <t>男性E</t>
         </is>
       </c>
       <c r="B143" s="3" t="inlineStr">
         <is>
-          <t>でもさ、結局こいつただの調子乗った反乱者やん。評価する要素ある？</t>
+          <t>そう、討たれた首は京都に送られて晒される。で、その首が夜に飛んで関東に戻った、っていうのが前半の祟りの話に繋がるんや</t>
         </is>
       </c>
       <c r="C143" s="2" t="inlineStr">
@@ -3617,19 +3617,19 @@
       </c>
       <c r="D143" s="2" t="inlineStr">
         <is>
-          <t>52</t>
+          <t>50</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
         <is>
-          <t>男性C大</t>
+          <t>男性A下</t>
         </is>
       </c>
       <c r="B144" s="3" t="inlineStr">
         <is>
-          <t>それがそうとも言い切れんのよ。中央の貴族が地方を搾取する仕組みに、地方の武装勢力が真っ向から「ノー」を突きつけた最初級の例なんや。後の武士が自分らの力で土地を治める時代の、いわば走りやねん。だから単なる謀反人やのうて、関東武士の精神的な元祖として評価する見方も根強いんや</t>
+          <t>きれいに一周してて草</t>
         </is>
       </c>
       <c r="C144" s="2" t="inlineStr">
@@ -3639,19 +3639,19 @@
       </c>
       <c r="D144" s="2" t="inlineStr">
         <is>
-          <t>53</t>
+          <t>51</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
         <is>
-          <t>女性D</t>
+          <t>女性B大</t>
         </is>
       </c>
       <c r="B145" s="3" t="inlineStr">
         <is>
-          <t>はい武士オタの過大評価、盛りすぎて引くわ</t>
+          <t>ちな朝廷も手をこまねいてたわけちゃうくて、将門調伏のために高僧に護摩祈祷を焚かせとってな。千葉の成田山新勝寺は、その将門調伏の祈祷をやった地に開かれたって伝わっとる。で、将門が討たれたもんやから「祈祷が効いた」ことになって、これが将門＝祟る怨霊ってイメージを後押しした面もあるんや。今でも神田明神の氏子は成田山には参らんって言われとるくらいでな</t>
         </is>
       </c>
       <c r="C145" s="2" t="inlineStr">
@@ -3661,19 +3661,19 @@
       </c>
       <c r="D145" s="2" t="inlineStr">
         <is>
-          <t>54</t>
+          <t>52</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
         <is>
-          <t>男性E下</t>
+          <t>男性C</t>
         </is>
       </c>
       <c r="B146" s="3" t="inlineStr">
         <is>
-          <t>過大評価ってだけで片付けるのも雑やろ、現に怨霊で千年語り継がれとるんやから</t>
+          <t>でもさ、結局こいつただの調子乗った反乱者やん。評価する要素ある？</t>
         </is>
       </c>
       <c r="C146" s="2" t="inlineStr">
@@ -3683,19 +3683,19 @@
       </c>
       <c r="D146" s="2" t="inlineStr">
         <is>
-          <t>55</t>
+          <t>53</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
         <is>
-          <t>男性A</t>
+          <t>女性D大</t>
         </is>
       </c>
       <c r="B147" s="3" t="inlineStr">
         <is>
-          <t>あと同じ時期に西で藤原純友も暴れとって、東西で同時に乱が起きとったんよな</t>
+          <t>それがそうとも言い切れんのよ。中央の貴族が地方を搾取する仕組みに、地方の武装勢力が真っ向から「ノー」を突きつけた最初級の例なんや。後の武士が自分らの力で土地を治める時代の、いわば走りやねん。だから単なる謀反人やのうて、関東武士の精神的な元祖として評価する見方も根強いんや</t>
         </is>
       </c>
       <c r="C147" s="2" t="inlineStr">
@@ -3705,19 +3705,19 @@
       </c>
       <c r="D147" s="2" t="inlineStr">
         <is>
-          <t>56</t>
+          <t>54</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
         <is>
-          <t>女性B下</t>
+          <t>男性E</t>
         </is>
       </c>
       <c r="B148" s="3" t="inlineStr">
         <is>
-          <t>それや、承平天慶の乱でセット扱いされるやつ。朝廷からしたら東西挟み撃ちで生きた心地せんかったやろな</t>
+          <t>はい武士オタの過大評価、盛りすぎて引くわ</t>
         </is>
       </c>
       <c r="C148" s="2" t="inlineStr">
@@ -3727,180 +3727,180 @@
       </c>
       <c r="D148" s="2" t="inlineStr">
         <is>
-          <t>57</t>
+          <t>55</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
         <is>
+          <t>男性A下</t>
+        </is>
+      </c>
+      <c r="B149" s="3" t="inlineStr">
+        <is>
+          <t>過大評価ってだけで片付けるのも雑やろ、現に怨霊で千年語り継がれとるんやから</t>
+        </is>
+      </c>
+      <c r="C149" s="2" t="inlineStr">
+        <is>
+          <t>スレ②</t>
+        </is>
+      </c>
+      <c r="D149" s="2" t="inlineStr">
+        <is>
+          <t>56</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="2" t="inlineStr">
+        <is>
+          <t>女性B</t>
+        </is>
+      </c>
+      <c r="B150" s="3" t="inlineStr">
+        <is>
+          <t>あと同じ時期に西で藤原純友も暴れとって、東西で同時に乱が起きとったんよな</t>
+        </is>
+      </c>
+      <c r="C150" s="2" t="inlineStr">
+        <is>
+          <t>スレ②</t>
+        </is>
+      </c>
+      <c r="D150" s="2" t="inlineStr">
+        <is>
+          <t>57</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="2" t="inlineStr">
+        <is>
+          <t>男性C下</t>
+        </is>
+      </c>
+      <c r="B151" s="3" t="inlineStr">
+        <is>
+          <t>それや、承平天慶の乱でセット扱いされるやつ。朝廷からしたら東西挟み撃ちで生きた心地せんかったやろな</t>
+        </is>
+      </c>
+      <c r="C151" s="2" t="inlineStr">
+        <is>
+          <t>スレ②</t>
+        </is>
+      </c>
+      <c r="D151" s="2" t="inlineStr">
+        <is>
+          <t>58</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="2" t="inlineStr">
+        <is>
           <t>解説者</t>
         </is>
       </c>
-      <c r="B149" s="3" t="inlineStr">
+      <c r="B152" s="3" t="inlineStr">
         <is>
           <t>承平天慶の乱とは、
 平安時代中期に東西で同時に起きた
 二つの大きな反乱の総称である。</t>
         </is>
       </c>
-      <c r="C149" s="2" t="inlineStr">
+      <c r="C152" s="2" t="inlineStr">
         <is>
           <t>解説：承平天慶の乱</t>
         </is>
       </c>
-      <c r="D149" s="2" t="inlineStr">
+      <c r="D152" s="2" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
     </row>
-    <row r="150">
-      <c r="A150" s="2" t="inlineStr">
+    <row r="153">
+      <c r="A153" s="2" t="inlineStr">
         <is>
           <t>解説者</t>
         </is>
       </c>
-      <c r="B150" s="3" t="inlineStr">
+      <c r="B153" s="3" t="inlineStr">
         <is>
           <t>東国では平将門が新皇を名乗って関東を制圧し、
 西国では瀬戸内で藤原純友が
 海賊を率いて朝廷に反旗をひるがえした。</t>
         </is>
       </c>
-      <c r="C150" s="2" t="inlineStr">
+      <c r="C153" s="2" t="inlineStr">
         <is>
           <t>解説：承平天慶の乱</t>
         </is>
       </c>
-      <c r="D150" s="2" t="inlineStr">
+      <c r="D153" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
     </row>
-    <row r="151">
-      <c r="A151" s="2" t="inlineStr">
+    <row r="154">
+      <c r="A154" s="2" t="inlineStr">
         <is>
           <t>解説者</t>
         </is>
       </c>
-      <c r="B151" s="3" t="inlineStr">
+      <c r="B154" s="3" t="inlineStr">
         <is>
           <t>朝廷にとっては東西から同時に
 挑戦を突きつけられた前代未聞の事態であり、</t>
         </is>
       </c>
-      <c r="C151" s="2" t="inlineStr">
+      <c r="C154" s="2" t="inlineStr">
         <is>
           <t>解説：承平天慶の乱</t>
         </is>
       </c>
-      <c r="D151" s="2" t="inlineStr">
+      <c r="D154" s="2" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
     </row>
-    <row r="152">
-      <c r="A152" s="2" t="inlineStr">
+    <row r="155">
+      <c r="A155" s="2" t="inlineStr">
         <is>
           <t>解説者</t>
         </is>
       </c>
-      <c r="B152" s="3" t="inlineStr">
+      <c r="B155" s="3" t="inlineStr">
         <is>
           <t>地方の武士の力を
 中央が無視できなくなっていく
 大きな転機となった出来事である。</t>
         </is>
       </c>
-      <c r="C152" s="2" t="inlineStr">
+      <c r="C155" s="2" t="inlineStr">
         <is>
           <t>解説：承平天慶の乱</t>
         </is>
       </c>
-      <c r="D152" s="2" t="inlineStr">
+      <c r="D155" s="2" t="inlineStr">
         <is>
           <t>4</t>
-        </is>
-      </c>
-    </row>
-    <row r="153">
-      <c r="A153" s="2" t="inlineStr">
-        <is>
-          <t>男性C</t>
-        </is>
-      </c>
-      <c r="B153" s="3" t="inlineStr">
-        <is>
-          <t>もし将門が勝っとったら関東に別の国できてたんかな</t>
-        </is>
-      </c>
-      <c r="C153" s="2" t="inlineStr">
-        <is>
-          <t>スレ②</t>
-        </is>
-      </c>
-      <c r="D153" s="2" t="inlineStr">
-        <is>
-          <t>58</t>
-        </is>
-      </c>
-    </row>
-    <row r="154">
-      <c r="A154" s="2" t="inlineStr">
-        <is>
-          <t>女性D大</t>
-        </is>
-      </c>
-      <c r="B154" s="3" t="inlineStr">
-        <is>
-          <t>そこはロマンあるよな。もし討伐をしのいで東国政権が定着しとったら、関東拠点の独立勢力が早い段階で出来て、武士の世が何百年か前倒しになってたかもしれん。まあ補給も人望もまだ足りんかったから現実は厳しかったやろけど。知らんけど、たらればとしては最高に面白い人物やわ</t>
-        </is>
-      </c>
-      <c r="C154" s="2" t="inlineStr">
-        <is>
-          <t>スレ②</t>
-        </is>
-      </c>
-      <c r="D154" s="2" t="inlineStr">
-        <is>
-          <t>59</t>
-        </is>
-      </c>
-    </row>
-    <row r="155">
-      <c r="A155" s="2" t="inlineStr">
-        <is>
-          <t>男性E下</t>
-        </is>
-      </c>
-      <c r="B155" s="3" t="inlineStr">
-        <is>
-          <t>関東人としてはちょっと応援したくなる</t>
-        </is>
-      </c>
-      <c r="C155" s="2" t="inlineStr">
-        <is>
-          <t>スレ②</t>
-        </is>
-      </c>
-      <c r="D155" s="2" t="inlineStr">
-        <is>
-          <t>60</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
         <is>
-          <t>男性A</t>
+          <t>女性D</t>
         </is>
       </c>
       <c r="B156" s="3" t="inlineStr">
         <is>
-          <t>ワイ千葉県民、地味に将門ゆかりの地に住んどる</t>
+          <t>もし将門が勝っとったら関東に別の国できてたんかな</t>
         </is>
       </c>
       <c r="C156" s="2" t="inlineStr">
@@ -3910,19 +3910,19 @@
       </c>
       <c r="D156" s="2" t="inlineStr">
         <is>
-          <t>61</t>
+          <t>59</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
         <is>
-          <t>女性B</t>
+          <t>男性E大</t>
         </is>
       </c>
       <c r="B157" s="3" t="inlineStr">
         <is>
-          <t>で、結局その首が今も大手町でブチギレてるわけやな</t>
+          <t>そこはロマンあるよな。もし討伐をしのいで東国政権が定着しとったら、関東拠点の独立勢力が早い段階で出来て、武士の世が何百年か前倒しになってたかもしれん。まあ補給も人望もまだ足りんかったから現実は厳しかったやろけど。知らんけど、たらればとしては最高に面白い人物やわ</t>
         </is>
       </c>
       <c r="C157" s="2" t="inlineStr">
@@ -3932,19 +3932,19 @@
       </c>
       <c r="D157" s="2" t="inlineStr">
         <is>
-          <t>62</t>
+          <t>60</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
         <is>
-          <t>男性C下</t>
+          <t>男性A下</t>
         </is>
       </c>
       <c r="B158" s="3" t="inlineStr">
         <is>
-          <t>千年たっても一等地から動かんあたり、ある意味いまだに関東の主やってるとも言えるわ</t>
+          <t>関東人としてはちょっと応援したくなる</t>
         </is>
       </c>
       <c r="C158" s="2" t="inlineStr">
@@ -3954,19 +3954,19 @@
       </c>
       <c r="D158" s="2" t="inlineStr">
         <is>
-          <t>63</t>
+          <t>61</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
         <is>
-          <t>女性D</t>
+          <t>女性B</t>
         </is>
       </c>
       <c r="B159" s="3" t="inlineStr">
         <is>
-          <t>うまいこと言うやん</t>
+          <t>ワイ千葉県民、地味に将門ゆかりの地に住んどる</t>
         </is>
       </c>
       <c r="C159" s="2" t="inlineStr">
@@ -3976,19 +3976,19 @@
       </c>
       <c r="D159" s="2" t="inlineStr">
         <is>
-          <t>64</t>
+          <t>62</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
         <is>
-          <t>男性E</t>
+          <t>男性C</t>
         </is>
       </c>
       <c r="B160" s="3" t="inlineStr">
         <is>
-          <t>ワイ明日大手町で乗り換えあるし、ちゃんと拝んどくわ。将門さん祟らんといてな</t>
+          <t>で、結局その首が今も大手町でブチギレてるわけやな</t>
         </is>
       </c>
       <c r="C160" s="2" t="inlineStr">
@@ -3998,86 +3998,152 @@
       </c>
       <c r="D160" s="2" t="inlineStr">
         <is>
-          <t>65</t>
+          <t>63</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
         <is>
-          <t>解説者</t>
+          <t>女性D下</t>
         </is>
       </c>
       <c r="B161" s="3" t="inlineStr">
         <is>
-          <t>本日はここまで。</t>
+          <t>千年たっても一等地から動かんあたり、ある意味いまだに関東の主やってるとも言えるわ</t>
         </is>
       </c>
       <c r="C161" s="2" t="inlineStr">
         <is>
-          <t>締め</t>
+          <t>スレ②</t>
         </is>
       </c>
       <c r="D161" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>64</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
         <is>
+          <t>男性E</t>
+        </is>
+      </c>
+      <c r="B162" s="3" t="inlineStr">
+        <is>
+          <t>うまいこと言うやん</t>
+        </is>
+      </c>
+      <c r="C162" s="2" t="inlineStr">
+        <is>
+          <t>スレ②</t>
+        </is>
+      </c>
+      <c r="D162" s="2" t="inlineStr">
+        <is>
+          <t>65</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" s="2" t="inlineStr">
+        <is>
+          <t>男性A</t>
+        </is>
+      </c>
+      <c r="B163" s="3" t="inlineStr">
+        <is>
+          <t>ワイ明日大手町で乗り換えあるし、ちゃんと拝んどくわ。将門さん祟らんといてな</t>
+        </is>
+      </c>
+      <c r="C163" s="2" t="inlineStr">
+        <is>
+          <t>スレ②</t>
+        </is>
+      </c>
+      <c r="D163" s="2" t="inlineStr">
+        <is>
+          <t>66</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" s="2" t="inlineStr">
+        <is>
           <t>解説者</t>
         </is>
       </c>
-      <c r="B162" s="3" t="inlineStr">
+      <c r="B164" s="3" t="inlineStr">
+        <is>
+          <t>本日はここまで。</t>
+        </is>
+      </c>
+      <c r="C164" s="2" t="inlineStr">
+        <is>
+          <t>締め</t>
+        </is>
+      </c>
+      <c r="D164" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" s="2" t="inlineStr">
+        <is>
+          <t>解説者</t>
+        </is>
+      </c>
+      <c r="B165" s="3" t="inlineStr">
         <is>
           <t>今回は、平将門の祟りについての
 さまざまな議論を見てきたが、
 いかがだっただろうか？</t>
         </is>
       </c>
-      <c r="C162" s="2" t="inlineStr">
+      <c r="C165" s="2" t="inlineStr">
         <is>
           <t>締め</t>
         </is>
       </c>
-      <c r="D162" s="2" t="inlineStr">
+      <c r="D165" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
     </row>
-    <row r="163">
-      <c r="A163" s="2" t="inlineStr">
+    <row r="166">
+      <c r="A166" s="2" t="inlineStr">
         <is>
           <t>解説者</t>
         </is>
       </c>
-      <c r="B163" s="3" t="inlineStr">
+      <c r="B166" s="3" t="inlineStr">
         <is>
           <t>2ちゃんねるの歴史オタクたちの
 議論を見ていると、</t>
         </is>
       </c>
-      <c r="C163" s="2" t="inlineStr">
+      <c r="C166" s="2" t="inlineStr">
         <is>
           <t>締め</t>
         </is>
       </c>
-      <c r="D163" s="2" t="inlineStr">
+      <c r="D166" s="2" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
     </row>
-    <row r="164">
-      <c r="A164" s="2" t="inlineStr">
+    <row r="167">
+      <c r="A167" s="2" t="inlineStr">
         <is>
           <t>解説者</t>
         </is>
       </c>
-      <c r="B164" s="3" t="inlineStr">
+      <c r="B167" s="3" t="inlineStr">
         <is>
           <t>将門は単なる祟り神ではなく、
 時代に真っ向から立ち向かって果てた反骨の武将であり、
@@ -4085,59 +4151,59 @@
 畏れと敬いを同時に集め続けているのだと思えた。</t>
         </is>
       </c>
-      <c r="C164" s="2" t="inlineStr">
+      <c r="C167" s="2" t="inlineStr">
         <is>
           <t>締め</t>
         </is>
       </c>
-      <c r="D164" s="2" t="inlineStr">
+      <c r="D167" s="2" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
     </row>
-    <row r="165">
-      <c r="A165" s="2" t="inlineStr">
+    <row r="168">
+      <c r="A168" s="2" t="inlineStr">
         <is>
           <t>解説者</t>
         </is>
       </c>
-      <c r="B165" s="3" t="inlineStr">
+      <c r="B168" s="3" t="inlineStr">
         <is>
           <t>今回の動画について他の意見や
 感想があったらぜひコメントで教えてね！</t>
         </is>
       </c>
-      <c r="C165" s="2" t="inlineStr">
+      <c r="C168" s="2" t="inlineStr">
         <is>
           <t>締め</t>
         </is>
       </c>
-      <c r="D165" s="2" t="inlineStr">
+      <c r="D168" s="2" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
     </row>
-    <row r="166">
-      <c r="A166" s="2" t="inlineStr">
+    <row r="169">
+      <c r="A169" s="2" t="inlineStr">
         <is>
           <t>解説者</t>
         </is>
       </c>
-      <c r="B166" s="3" t="inlineStr">
+      <c r="B169" s="3" t="inlineStr">
         <is>
           <t>他にも歴史にまつわる情報をまとめた
 動画が満載なので、ぜひ見てみてくださいね。
 ご視聴ありがとうございました！</t>
         </is>
       </c>
-      <c r="C166" s="2" t="inlineStr">
+      <c r="C169" s="2" t="inlineStr">
         <is>
           <t>締め</t>
         </is>
       </c>
-      <c r="D166" s="2" t="inlineStr">
+      <c r="D169" s="2" t="inlineStr">
         <is>
           <t>6</t>
         </is>

</xml_diff>

<commit_message>
auto: 2026-06-17 17:08 (4件)
</commit_message>
<xml_diff>
--- a/01_プロジェクト/YouTube/創作スレ下書き/2026-06-17_平将門の祟り_台本.xlsx
+++ b/01_プロジェクト/YouTube/創作スレ下書き/2026-06-17_平将門の祟り_台本.xlsx
@@ -1100,7 +1100,7 @@
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>アメリカ人にも効くんかい</t>
+          <t>天下のGHQが工事引っ込めるとか、相当のことやん</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
@@ -1122,7 +1122,7 @@
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>祟りに国籍は関係ないの好き</t>
+          <t>国家権力に二連勝してる時点で将門つよすぎやろ</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">

</xml_diff>

<commit_message>
auto: 2026-06-17 18:18 (4件)
</commit_message>
<xml_diff>
--- a/01_プロジェクト/YouTube/創作スレ下書き/2026-06-17_平将門の祟り_台本.xlsx
+++ b/01_プロジェクト/YouTube/創作スレ下書き/2026-06-17_平将門の祟り_台本.xlsx
@@ -1078,7 +1078,7 @@
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>戦後にもう一回やらかしとる。GHQが大手町を区画整理するとき、塚も邪魔やからって整地しようとしたら、米軍のブルドーザーが作業中に横転して運転手が亡くなったって記録に残ってる。で、結局そこも工事は取りやめや。震災のときもGHQのときも、"お国"クラスがどかそうとして二回とも引き下がっとる。そこがこの塚のゾッとするとこやねん</t>
+          <t>戦後にもう一回やらかしとる。今度は大手町を大規模に区画整理するとき、塚も邪魔やからって整地しようとしたら、重機が作業中に横転して運転手が亡くなったって記録に残ってる。で、結局そこも工事は取りやめや。震災のときも戦後のときも、"お国"クラスがどかそうとして二回とも引き下がっとる。そこがこの塚のゾッとするとこやねん</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
@@ -1100,7 +1100,7 @@
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>天下のGHQが工事引っ込めるとか、相当のことやん</t>
+          <t>天下の国家事業が二度も引っ込むとか、相当のことやん</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
@@ -1144,7 +1144,7 @@
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>知らんけど進駐軍がオカルトでビビって引くとかある？</t>
+          <t>知らんけどお役所がオカルトでビビって引くとかある？</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">

</xml_diff>

<commit_message>
auto: 2026-06-18 15:08 (5件)
</commit_message>
<xml_diff>
--- a/01_プロジェクト/YouTube/創作スレ下書き/2026-06-17_平将門の祟り_台本.xlsx
+++ b/01_プロジェクト/YouTube/創作スレ下書き/2026-06-17_平将門の祟り_台本.xlsx
@@ -1095,7 +1095,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>女性D下</t>
+          <t>女性D</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">
@@ -1366,7 +1366,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>女性B下</t>
+          <t>女性B</t>
         </is>
       </c>
       <c r="B42" s="3" t="inlineStr">
@@ -1806,7 +1806,7 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>女性B下大</t>
+          <t>女性B大</t>
         </is>
       </c>
       <c r="B62" s="3" t="inlineStr">
@@ -2070,7 +2070,7 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>女性D下</t>
+          <t>女性D</t>
         </is>
       </c>
       <c r="B74" s="3" t="inlineStr">
@@ -2780,7 +2780,7 @@
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
         <is>
-          <t>女性B下</t>
+          <t>女性B</t>
         </is>
       </c>
       <c r="B106" s="3" t="inlineStr">
@@ -2986,7 +2986,7 @@
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
         <is>
-          <t>女性B下</t>
+          <t>女性B</t>
         </is>
       </c>
       <c r="B115" s="3" t="inlineStr">
@@ -3228,7 +3228,7 @@
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
         <is>
-          <t>男性C下</t>
+          <t>男性C</t>
         </is>
       </c>
       <c r="B126" s="3" t="inlineStr">
@@ -3426,7 +3426,7 @@
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
         <is>
-          <t>女性B下</t>
+          <t>女性B</t>
         </is>
       </c>
       <c r="B135" s="3" t="inlineStr">
@@ -3939,7 +3939,7 @@
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
         <is>
-          <t>男性A下</t>
+          <t>男性A</t>
         </is>
       </c>
       <c r="B158" s="3" t="inlineStr">

</xml_diff>

<commit_message>
auto: 2026-06-18 18:08 (4件)
</commit_message>
<xml_diff>
--- a/01_プロジェクト/YouTube/創作スレ下書き/2026-06-17_平将門の祟り_台本.xlsx
+++ b/01_プロジェクト/YouTube/創作スレ下書き/2026-06-17_平将門の祟り_台本.xlsx
@@ -433,7 +433,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="70" customWidth="1" min="2" max="2"/>
+    <col width="48" customWidth="1" min="2" max="2"/>
     <col width="22" customWidth="1" min="3" max="3"/>
     <col width="6" customWidth="1" min="4" max="4"/>
   </cols>
@@ -469,8 +469,7 @@
       <c r="B2" s="3" t="inlineStr">
         <is>
           <t>平将門と聞くと、
-「日本三大怨霊」「祟り神」
-そんな恐ろしいイメージを持つ人も多いだろう。</t>
+「日本三大怨霊」「祟り神」そんな恐ろしいイメージを持つ人も多いだろう。</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -492,7 +491,8 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>だが、その祟りの噂ばかりが独り歩きして、
+          <t>だが、
+その祟りの噂ばかりが独り歩きして、
 将門が生きている間に一体何をした人物なのかは、
 意外と知られていない。</t>
         </is>
@@ -540,7 +540,8 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>果たして、平将門はなぜ千年も恐れられる怨霊となったのだろうか？</t>
+          <t>果たして、
+平将門はなぜ千年も恐れられる怨霊となったのだろうか？</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -562,7 +563,8 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>今回は、平将門について議論を繰り広げる、
+          <t>今回は、
+平将門について議論を繰り広げる、
 2ちゃんねるの歴史オタクたちを見ていこう。</t>
         </is>
       </c>
@@ -586,8 +588,8 @@
       <c r="B7" s="3" t="inlineStr">
         <is>
           <t>この動画を見れば、
-平将門の祟りの正体と、その壮絶な生涯が
-きっとわかるだろう。</t>
+平将門の祟りの正体と、
+その壮絶な生涯がきっとわかるだろう。</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -719,7 +721,8 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>ただのオカルトを真に受けすぎや、ぜんぶ偶然やろ</t>
+          <t>ただのオカルトを真に受けすぎや、
+ぜんぶ偶然やろ</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -763,7 +766,15 @@
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>いや偶然で片付けるには出来すぎなんよ。関東大震災のあと、あの跡地に大蔵省の仮庁舎を建てようとしたら、工事関係者やら省の職員が立て続けに倒れて、当時の大蔵大臣やった早速整爾まで亡くなった。さすがに省内で「将門の祟りや」って噂が広がって、結局その仮庁舎を取り壊しとる。お役所が一回建てたもん壊すんやで、相当の騒ぎやったってことや</t>
+          <t>いや偶然で片付けるには出来すぎなんよ。
+関東大震災のあと、
+あの跡地に大蔵省の仮庁舎を建てようとしたら、
+工事関係者やら省の職員が立て続けに倒れて、
+当時の大蔵大臣やった早速整爾まで亡くなった。
+さすがに省内で「将門の祟りや」って噂が広がって、
+結局その仮庁舎を取り壊しとる。
+お役所が一回建てたもん壊すんやで、
+相当の騒ぎやったってことや</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -851,7 +862,8 @@
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>早速整爾って総理大臣やっけ？それで騒ぎになったんやろ</t>
+          <t>早速整爾って総理大臣やっけ？
+それで騒ぎになったんやろ</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
@@ -873,7 +885,10 @@
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>ちゃう、大蔵大臣や。総理と混同すると話の重みが変わるで、そこは正しく覚えとけ</t>
+          <t>ちゃう、
+大蔵大臣や。
+総理と混同すると話の重みが変わるで、
+そこは正しく覚えとけ</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -895,7 +910,8 @@
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>お、おう…とにかく偉い人が立て続けに倒れたんやな</t>
+          <t>お、
+おう…とにかく偉い人が立て続けに倒れたんやな</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
@@ -918,8 +934,8 @@
       <c r="B22" s="3" t="inlineStr">
         <is>
           <t>大蔵省仮庁舎の祟りとは、
-関東大震災のあと、首塚の跡地に建てられた
-大蔵省の仮庁舎で相次いだ不審な出来事を指す。</t>
+関東大震災のあと、
+首塚の跡地に建てられた大蔵省の仮庁舎で相次いだ不審な出来事を指す。</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
@@ -942,8 +958,7 @@
       <c r="B23" s="3" t="inlineStr">
         <is>
           <t>工事の関係者や省の職員が次々と体調を崩し、
-当時の大蔵大臣・早速整爾までもが
-在任中に亡くなったことで、
+当時の大蔵大臣・早速整爾までもが在任中に亡くなったことで、
 将門の祟りだと省内で噂された。</t>
         </is>
       </c>
@@ -1012,7 +1027,8 @@
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>でもその年代の偉い人なんてポンポン亡くなるやろ、こじつけやって</t>
+          <t>でもその年代の偉い人なんてポンポン亡くなるやろ、
+こじつけやって</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
@@ -1034,7 +1050,8 @@
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>それな、後から祟りってことにしただけやろ</t>
+          <t>それな、
+後から祟りってことにしただけやろ</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
@@ -1056,7 +1073,8 @@
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>一回ならそう言えるんやけどな、これ二回あるねん</t>
+          <t>一回ならそう言えるんやけどな、
+これ二回あるねん</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
@@ -1078,7 +1096,15 @@
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>戦後にもう一回やらかしとる。今度は大手町を大規模に区画整理するとき、塚も邪魔やからって整地しようとしたら、重機が作業中に横転して運転手が亡くなったって記録に残ってる。で、結局そこも工事は取りやめや。震災のときも戦後のときも、"お国"クラスがどかそうとして二回とも引き下がっとる。そこがこの塚のゾッとするとこやねん</t>
+          <t>戦後にもう一回やらかしとる。
+今度は大手町を大規模に区画整理するとき、
+塚も邪魔やからって整地しようとしたら、
+重機が作業中に横転して運転手が亡くなったって記録に残ってる。
+で、
+結局そこも工事は取りやめや。
+震災のときも戦後のときも、
+"お国"クラスがどかそうとして二回とも引き下がっとる。
+そこがこの塚のゾッとするとこやねん</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
@@ -1100,7 +1126,8 @@
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>天下の国家事業が二度も引っ込むとか、相当のことやん</t>
+          <t>天下の国家事業が二度も引っ込むとか、
+相当のことやん</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
@@ -1166,7 +1193,8 @@
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>まあ伝説で盛られてるとこもあるやろけど、塚が一等地に今も残ってるのは事実やしな</t>
+          <t>まあ伝説で盛られてるとこもあるやろけど、
+塚が一等地に今も残ってるのは事実やしな</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
@@ -1188,7 +1216,8 @@
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>そもそも首塚って京都にあるんちゃうの？晒し首にされたんやろ</t>
+          <t>そもそも首塚って京都にあるんちゃうの？
+晒し首にされたんやろ</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
@@ -1210,7 +1239,10 @@
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>晒されたのが京都、そこから首が夜空に舞い上がって関東に飛んで戻って落ちた、その伝承地が大手町や。話が混ざっとるで</t>
+          <t>晒されたのが京都、
+そこから首が夜空に舞い上がって関東に飛んで戻って落ちた、
+その伝承地が大手町や。
+話が混ざっとるで</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
@@ -1254,7 +1286,8 @@
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>将門塚、いわゆる平将門の首塚とは、
+          <t>将門塚、
+いわゆる平将門の首塚とは、
 討たれた将門の首を祀ったとされる塚である。</t>
         </is>
       </c>
@@ -1277,8 +1310,9 @@
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>伝承では、京で晒された将門の首が
-関東へ飛んで戻り、落ちた場所に築かれたとされ、
+          <t>伝承では、
+京で晒された将門の首が関東へ飛んで戻り、
+落ちた場所に築かれたとされ、
 東京・大手町に今も残っている。</t>
         </is>
       </c>
@@ -1324,10 +1358,8 @@
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>将門は菅原道真・崇徳上皇と並ぶ
-日本三大怨霊の一柱とされる一方、
-神田明神では江戸を守る祭神として
-篤く祀られている存在でもある。</t>
+          <t>将門は菅原道真・崇徳上皇と並ぶ日本三大怨霊の一柱とされる一方、
+神田明神では江戸を守る祭神として篤く祀られている存在でもある。</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
@@ -1349,7 +1381,12 @@
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>首が飛んだ伝承自体もなかなかで、京都で晒された将門の首が「胴体はどこや」って叫びながら夜空を東へ飛んで、力尽きて落ちた場所が今の大手町って筋書きなんよ。しかも落ちた候補地は一か所ちゃうくて、各地に「ここが本物の首塚や」っていう伝承地が点々と残っとる。執念で関東まで戻ってきたって話がもう只者ちゃうねん</t>
+          <t>首が飛んだ伝承自体もなかなかで、
+京都で晒された将門の首が「胴体はどこや」って叫びながら夜空を東へ飛んで、
+力尽きて落ちた場所が今の大手町って筋書きなんよ。
+しかも落ちた候補地は一か所ちゃうくて、
+各地に「ここが本物の首塚や」っていう伝承地が点々と残っとる。
+執念で関東まで戻ってきたって話がもう只者ちゃうねん</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
@@ -1393,7 +1430,8 @@
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>で、その大手町の土地って今いくらすんの</t>
+          <t>で、
+その大手町の土地って今いくらすんの</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
@@ -1415,7 +1453,14 @@
       </c>
       <c r="B44" s="3" t="inlineStr">
         <is>
-          <t>それがな、丸の内のド真ん中の超一等地で、更地の地価で数十億とも言われとる。普通やったらビルが何本も建つ土地に、塚だけポツンと残しとるわけや。再開発のたびに「ここだけは触らんとこ」って供養して避けて通る。経済合理性が全ての街のド真ん中で、そこだけ理屈が通らん空白地帯になっとるんや</t>
+          <t>それがな、
+丸の内のド真ん中の超一等地で、
+更地の地価で数十億とも言われとる。
+普通やったらビルが何本も建つ土地に、
+塚だけポツンと残しとるわけや。
+再開発のたびに「ここだけは触らんとこ」って供養して避けて通る。
+経済合理性が全ての街のド真ん中で、
+そこだけ理屈が通らん空白地帯になっとるんや</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
@@ -1459,7 +1504,8 @@
       </c>
       <c r="B46" s="3" t="inlineStr">
         <is>
-          <t>はいオカルト、全部こじつけ</t>
+          <t>はいオカルト、
+全部こじつけ</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
@@ -1481,7 +1527,8 @@
       </c>
       <c r="B47" s="3" t="inlineStr">
         <is>
-          <t>で？二回も国家側が引き下がってる事実は消えへんで</t>
+          <t>で？
+二回も国家側が引き下がってる事実は消えへんで</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
@@ -1503,7 +1550,13 @@
       </c>
       <c r="B48" s="3" t="inlineStr">
         <is>
-          <t>周りのビルがまた徹底しててな。塚を見下ろさんように、塚に面した側はわざと窓を作らへんとか、社員が塚に尻を向けんように管理職の机の向きまで気いつかっとるって言われとる。信じる信じへん以前に、ガチガチの大企業がそこまで配慮してまう空気があるってのが、ある意味一番の答え合わせやねん</t>
+          <t>周りのビルがまた徹底しててな。
+塚を見下ろさんように、
+塚に面した側はわざと窓を作らへんとか、
+社員が塚に尻を向けんように管理職の机の向きまで気いつかっとるって言われとる。
+信じる信じへん以前に、
+ガチガチの大企業がそこまで配慮してまう空気があるってのが、
+ある意味一番の答え合わせやねん</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
@@ -1591,7 +1644,10 @@
       </c>
       <c r="B52" s="3" t="inlineStr">
         <is>
-          <t>ほんまかどうかは知らん、そう言われてるってだけや。ただ塚の管理のために近くの銀行に「平将門」名義の口座が開かれとったのは、割と有名な話やで</t>
+          <t>ほんまかどうかは知らん、
+そう言われてるってだけや。
+ただ塚の管理のために近くの銀行に「平将門」名義の口座が開かれとったのは、
+割と有名な話やで</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
@@ -1679,7 +1735,13 @@
       </c>
       <c r="B56" s="3" t="inlineStr">
         <is>
-          <t>しかも今の塚は地元の企業が金を出し合って守っとるんよ。「史蹟将門塚保存会」っちゅう近隣の会社が集まった団体が、浄財で周りの清掃や整備をずっと続けとる。要は天下の一等地のド真ん中で、周りの大企業が「将門さんの機嫌だけは損ねたらあかん」って共同で面倒を見続けとるわけや。これだけでも、土地そのものが特別扱いされとるのが分かるやろ</t>
+          <t>しかも今の塚は地元の企業が金を出し合って守っとるんよ。
+「史蹟将門塚保存会」っちゅう近隣の会社が集まった団体が、
+浄財で周りの清掃や整備をずっと続けとる。
+要は天下の一等地のド真ん中で、
+周りの大企業が「将門さんの機嫌だけは損ねたらあかん」って共同で面倒を見続けとるわけや。
+これだけでも、
+土地そのものが特別扱いされとるのが分かるやろ</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
@@ -1723,7 +1785,8 @@
       </c>
       <c r="B58" s="3" t="inlineStr">
         <is>
-          <t>ワイ去年あの辺で働いとったとき、毎朝コンビニ寄る感覚で手だけ合わせて通勤しとったわ</t>
+          <t>ワイ去年あの辺で働いとったとき、
+毎朝コンビニ寄る感覚で手だけ合わせて通勤しとったわ</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
@@ -1767,7 +1830,9 @@
       </c>
       <c r="B60" s="3" t="inlineStr">
         <is>
-          <t>カエルの置物いっぱい置いてあるよな、無事カエルでって。最初なんの土産物屋かと思った</t>
+          <t>カエルの置物いっぱい置いてあるよな、
+無事カエルでって。
+最初なんの土産物屋かと思った</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
@@ -1789,7 +1854,8 @@
       </c>
       <c r="B61" s="3" t="inlineStr">
         <is>
-          <t>で、結局三大怨霊って残り誰なん</t>
+          <t>で、
+結局三大怨霊って残り誰なん</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr">
@@ -1811,7 +1877,14 @@
       </c>
       <c r="B62" s="3" t="inlineStr">
         <is>
-          <t>これ豆な、将門は今や神田明神の祭神になっとって、崇徳上皇・菅原道真と並んで日本三大怨霊に数えられとる。面白いのが、徳川が江戸入りしたとき将門を江戸の総鎮守として篤く祀り直しとるんよ。怒らせたら祟るけど、ちゃんと祀れば街を守ってくれる、っていう"祟り神の出世コース"に乗っとるわけや</t>
+          <t>これ豆な、
+将門は今や神田明神の祭神になっとって、
+崇徳上皇・菅原道真と並んで日本三大怨霊に数えられとる。
+面白いのが、
+徳川が江戸入りしたとき将門を江戸の総鎮守として篤く祀り直しとるんよ。
+怒らせたら祟るけど、
+ちゃんと祀れば街を守ってくれる、
+っていう"祟り神の出世コース"に乗っとるわけや</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
@@ -1855,7 +1928,13 @@
       </c>
       <c r="B64" s="3" t="inlineStr">
         <is>
-          <t>その道真なんか今や学問の神様で、受験シーズンに全国の受験生が手を合わせに行くレベルやからな。恐れられた怨霊ほど後世の祀られ方が手厚なる、っていうのが日本のおもろい癖やねん。最初は災いの元として恐れられた連中が、丁重に祀られて街や受験生を守る側に回る。将門もその王道を歩んどるわけや</t>
+          <t>その道真なんか今や学問の神様で、
+受験シーズンに全国の受験生が手を合わせに行くレベルやからな。
+恐れられた怨霊ほど後世の祀られ方が手厚なる、
+っていうのが日本のおもろい癖やねん。
+最初は災いの元として恐れられた連中が、
+丁重に祀られて街や受験生を守る側に回る。
+将門もその王道を歩んどるわけや</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
@@ -1877,7 +1956,8 @@
       </c>
       <c r="B65" s="3" t="inlineStr">
         <is>
-          <t>落とし所が神様って発想、日本ぐらいやろ</t>
+          <t>落とし所が神様って発想、
+日本ぐらいやろ</t>
         </is>
       </c>
       <c r="C65" s="2" t="inlineStr">
@@ -1899,7 +1979,9 @@
       </c>
       <c r="B66" s="3" t="inlineStr">
         <is>
-          <t>メガテン勢からすると将門公はガチで畏れる対象や。アトラスが将門モチーフにしたら開発中トラブル続きで、表記を「マサカドこう」に直したら止んだって都市伝説あるやろ</t>
+          <t>メガテン勢からすると将門公はガチで畏れる対象や。
+アトラスが将門モチーフにしたら開発中トラブル続きで、
+表記を「マサカドこう」に直したら止んだって都市伝説あるやろ</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr">
@@ -1987,7 +2069,8 @@
       </c>
       <c r="B70" s="3" t="inlineStr">
         <is>
-          <t>太田光が売れる前に首塚にドロップキックかまして、しばらく仕事来んくなったって噂もあるな</t>
+          <t>太田光が売れる前に首塚にドロップキックかまして、
+しばらく仕事来んくなったって噂もあるな</t>
         </is>
       </c>
       <c r="C70" s="2" t="inlineStr">
@@ -2031,7 +2114,13 @@
       </c>
       <c r="B72" s="3" t="inlineStr">
         <is>
-          <t>ついでに言うと、将門を祀る神田明神の神田祭は、今も山王祭と並ぶ江戸三大祭のひとつでな。将門は江戸の総鎮守として庶民にめちゃくちゃ愛されてきたんよ。怨霊として恐れられた男が、江戸っ子の誇りの祭の主役になっとるんやから、畏れと信仰なんて紙一重やなって思うわ</t>
+          <t>ついでに言うと、
+将門を祀る神田明神の神田祭は、
+今も山王祭と並ぶ江戸三大祭のひとつでな。
+将門は江戸の総鎮守として庶民にめちゃくちゃ愛されてきたんよ。
+怨霊として恐れられた男が、
+江戸っ子の誇りの祭の主役になっとるんやから、
+畏れと信仰なんて紙一重やなって思うわ</t>
         </is>
       </c>
       <c r="C72" s="2" t="inlineStr">
@@ -2053,7 +2142,14 @@
       </c>
       <c r="B73" s="3" t="inlineStr">
         <is>
-          <t>ここ大事なんやけど、将門はただ恐れられただけちゃうくて、もともとは関東の民にとっては英雄寄りの存在やったんよ。重い負担やら国府の横暴に苦しむ坂東の人らからしたら、中央に盾突いて「東は俺らで治める」ってやってのけた将門は反骨のシンボルやった。だからこそ討たれたあとも、祟り神として畏れられつつ土地の守り神として手厚く祀られ続けた、っていう二面性があるわけや</t>
+          <t>ここ大事なんやけど、
+将門はただ恐れられただけちゃうくて、
+もともとは関東の民にとっては英雄寄りの存在やったんよ。
+重い負担やら国府の横暴に苦しむ坂東の人らからしたら、
+中央に盾突いて「東は俺らで治める」ってやってのけた将門は反骨のシンボルやった。
+だからこそ討たれたあとも、
+祟り神として畏れられつつ土地の守り神として手厚く祀られ続けた、
+っていう二面性があるわけや</t>
         </is>
       </c>
       <c r="C73" s="2" t="inlineStr">
@@ -2097,7 +2193,8 @@
       </c>
       <c r="B75" s="3" t="inlineStr">
         <is>
-          <t>怨霊を祀る祭で江戸三大祭って、考えたら相当パンチ効いとるな</t>
+          <t>怨霊を祀る祭で江戸三大祭って、
+考えたら相当パンチ効いとるな</t>
         </is>
       </c>
       <c r="C75" s="2" t="inlineStr">
@@ -2119,7 +2216,9 @@
       </c>
       <c r="B76" s="3" t="inlineStr">
         <is>
-          <t>結局さ、全部"そういうことにしとこ"の後付けやろ。因果の証拠なんか無いやん</t>
+          <t>結局さ、
+全部"そういうことにしとこ"の後付けやろ。
+因果の証拠なんか無いやん</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
@@ -2141,7 +2240,8 @@
       </c>
       <c r="B77" s="3" t="inlineStr">
         <is>
-          <t>信者乙、ぜんぶ偶然や</t>
+          <t>信者乙、
+ぜんぶ偶然や</t>
         </is>
       </c>
       <c r="C77" s="2" t="inlineStr">
@@ -2163,7 +2263,8 @@
       </c>
       <c r="B78" s="3" t="inlineStr">
         <is>
-          <t>まあ祟りに証拠もへったくれもないわな、そこは認める</t>
+          <t>まあ祟りに証拠もへったくれもないわな、
+そこは認める</t>
         </is>
       </c>
       <c r="C78" s="2" t="inlineStr">
@@ -2185,7 +2286,8 @@
       </c>
       <c r="B79" s="3" t="inlineStr">
         <is>
-          <t>証拠ないのに国家プロジェクトが二回もどかすのやめてる時点で、もう実質勝ちなんよ将門</t>
+          <t>証拠ないのに国家プロジェクトが二回もどかすのやめてる時点で、
+もう実質勝ちなんよ将門</t>
         </is>
       </c>
       <c r="C79" s="2" t="inlineStr">
@@ -2251,7 +2353,8 @@
       </c>
       <c r="B82" s="3" t="inlineStr">
         <is>
-          <t>それは嘘らしいで、結界説は後から誰かが言い出したやつや</t>
+          <t>それは嘘らしいで、
+結界説は後から誰かが言い出したやつや</t>
         </is>
       </c>
       <c r="C82" s="2" t="inlineStr">
@@ -2295,7 +2398,10 @@
       </c>
       <c r="B84" s="3" t="inlineStr">
         <is>
-          <t>嘘か本当か分からんのが一番こわいんよこの人。で、そもそも将門ってなんで反乱なんか起こしたん？怨霊の部分しか知らんわ</t>
+          <t>嘘か本当か分からんのが一番こわいんよこの人。
+で、
+そもそも将門ってなんで反乱なんか起こしたん？
+怨霊の部分しか知らんわ</t>
         </is>
       </c>
       <c r="C84" s="2" t="inlineStr">
@@ -2340,8 +2446,7 @@
       <c r="B86" s="3" t="inlineStr">
         <is>
           <t>ここまでは、
-平将門の首塚にまつわる祟りの噂について
-さまざまな議論を見てきたが、</t>
+平将門の首塚にまつわる祟りの噂についてさまざまな議論を見てきたが、</t>
         </is>
       </c>
       <c r="C86" s="2" t="inlineStr">
@@ -2364,8 +2469,9 @@
       <c r="B87" s="3" t="inlineStr">
         <is>
           <t>「そもそも将門は何をして、
-ここまで恐れられる存在になったの？」
-と、肝心の生涯に疑問を持つ者も現れた。</t>
+ここまで恐れられる存在になったの？
+」と、
+肝心の生涯に疑問を持つ者も現れた。</t>
         </is>
       </c>
       <c r="C87" s="2" t="inlineStr">
@@ -2387,7 +2493,8 @@
       </c>
       <c r="B88" s="3" t="inlineStr">
         <is>
-          <t>たしかに、千年も祟りが語り継がれる怨霊が、
+          <t>たしかに、
+千年も祟りが語り継がれる怨霊が、
 どうやって生まれたのかは気になるところだ。</t>
         </is>
       </c>
@@ -2410,8 +2517,8 @@
       </c>
       <c r="B89" s="3" t="inlineStr">
         <is>
-          <t>引き続き、2ちゃんねるの歴史オタクたちの
-議論を見ていこう。</t>
+          <t>引き続き、
+2ちゃんねるの歴史オタクたちの議論を見ていこう。</t>
         </is>
       </c>
       <c r="C89" s="2" t="inlineStr">
@@ -2433,7 +2540,8 @@
       </c>
       <c r="B90" s="3" t="inlineStr">
         <is>
-          <t>平将門「これからは俺が東の天皇やるわ」朝廷「は？」</t>
+          <t>平将門「これからは俺が東の天皇やるわ」朝廷「は？
+」</t>
         </is>
       </c>
       <c r="C90" s="2" t="inlineStr">
@@ -2521,7 +2629,8 @@
       </c>
       <c r="B94" s="3" t="inlineStr">
         <is>
-          <t>結局その新皇とやらも2か月で終わった負け犬やん、持ち上げる要素ある？</t>
+          <t>結局その新皇とやらも2か月で終わった負け犬やん、
+持ち上げる要素ある？</t>
         </is>
       </c>
       <c r="C94" s="2" t="inlineStr">
@@ -2565,7 +2674,8 @@
       </c>
       <c r="B96" s="3" t="inlineStr">
         <is>
-          <t>で、結局こいつ何がしたかったん</t>
+          <t>で、
+結局こいつ何がしたかったん</t>
         </is>
       </c>
       <c r="C96" s="2" t="inlineStr">
@@ -2587,7 +2697,8 @@
       </c>
       <c r="B97" s="3" t="inlineStr">
         <is>
-          <t>中央に喧嘩売って負けた人や、それ以上でもそれ以下でもなくない？</t>
+          <t>中央に喧嘩売って負けた人や、
+それ以上でもそれ以下でもなくない？</t>
         </is>
       </c>
       <c r="C97" s="2" t="inlineStr">
@@ -2609,7 +2720,14 @@
       </c>
       <c r="B98" s="3" t="inlineStr">
         <is>
-          <t>それがな、最初っから天皇に盾突こうとしてたわけちゃうんよ。スタートはただの一族内のもめ事や。関東の平氏一門で、伯父さんらと土地や縁談がらみの私闘をやっとった、いわば身内ゲンカからの叩き上げやねん。それが勝ち続けるうちに、どんどん引くに引けん大ごとになってってもうた</t>
+          <t>それがな、
+最初っから天皇に盾突こうとしてたわけちゃうんよ。
+スタートはただの一族内のもめ事や。
+関東の平氏一門で、
+伯父さんらと土地や縁談がらみの私闘をやっとった、
+いわば身内ゲンカからの叩き上げやねん。
+それが勝ち続けるうちに、
+どんどん引くに引けん大ごとになってってもうた</t>
         </is>
       </c>
       <c r="C98" s="2" t="inlineStr">
@@ -2697,7 +2815,13 @@
       </c>
       <c r="B102" s="3" t="inlineStr">
         <is>
-          <t>そもそも将門の出自も知っとくとええで。あいつ桓武天皇の血を引く桓武平氏で、高望王の孫にあたる名門の出やねん。若い頃は京都に上って摂関家に奉公しとった時期もあって、決して田舎のチンピラちゃう。中央の作法も権力の構造も知った上で関東に戻って、結局その中央に弓を引くことになったわけや</t>
+          <t>そもそも将門の出自も知っとくとええで。
+あいつ桓武天皇の血を引く桓武平氏で、
+高望王の孫にあたる名門の出やねん。
+若い頃は京都に上って摂関家に奉公しとった時期もあって、
+決して田舎のチンピラちゃう。
+中央の作法も権力の構造も知った上で関東に戻って、
+結局その中央に弓を引くことになったわけや</t>
         </is>
       </c>
       <c r="C102" s="2" t="inlineStr">
@@ -2763,7 +2887,13 @@
       </c>
       <c r="B105" s="3" t="inlineStr">
         <is>
-          <t>ちな将門の地盤は下総の猿島あたりでな、当時の坂東は朝廷の目が届きにくい辺境で、しかも良馬の産地やった。だから機動力のある騎馬の武士団を抱えやすくて、中央から来た役人よりも地元で腕の立つ将門のほうが頼りにされとった。そういう土壌があったからこそ、一介の豪族が関東一円を呑み込むなんて芸当ができたわけや</t>
+          <t>ちな将門の地盤は下総の猿島あたりでな、
+当時の坂東は朝廷の目が届きにくい辺境で、
+しかも良馬の産地やった。
+だから機動力のある騎馬の武士団を抱えやすくて、
+中央から来た役人よりも地元で腕の立つ将門のほうが頼りにされとった。
+そういう土壌があったからこそ、
+一介の豪族が関東一円を呑み込むなんて芸当ができたわけや</t>
         </is>
       </c>
       <c r="C105" s="2" t="inlineStr">
@@ -2785,7 +2915,8 @@
       </c>
       <c r="B106" s="3" t="inlineStr">
         <is>
-          <t>馬かよ、そら強いわけや</t>
+          <t>馬かよ、
+そら強いわけや</t>
         </is>
       </c>
       <c r="C106" s="2" t="inlineStr">
@@ -2807,7 +2938,14 @@
       </c>
       <c r="B107" s="3" t="inlineStr">
         <is>
-          <t>で、私闘で官側の人間ともやり合ううちに、今度は朝廷の出先の国府とぶつかってまう。勢いで常陸の国府を攻め落として、国の実印にあたる印鑰まで奪ってもうた。これ当時やと完全に一線を越えた行為で、国に弓を引いた賊って扱いになる。もう後戻りでけへんとこまで行ったわけや</t>
+          <t>で、
+私闘で官側の人間ともやり合ううちに、
+今度は朝廷の出先の国府とぶつかってまう。
+勢いで常陸の国府を攻め落として、
+国の実印にあたる印鑰まで奪ってもうた。
+これ当時やと完全に一線を越えた行為で、
+国に弓を引いた賊って扱いになる。
+もう後戻りでけへんとこまで行ったわけや</t>
         </is>
       </c>
       <c r="C107" s="2" t="inlineStr">
@@ -2851,7 +2989,8 @@
       </c>
       <c r="B109" s="3" t="inlineStr">
         <is>
-          <t>国を動かす実印とハンコ箱みたいなもんや。それ奪うって今でいう役所まるごと乗っ取るレベルやぞ</t>
+          <t>国を動かす実印とハンコ箱みたいなもんや。
+それ奪うって今でいう役所まるごと乗っ取るレベルやぞ</t>
         </is>
       </c>
       <c r="C109" s="2" t="inlineStr">
@@ -2898,8 +3037,7 @@
       <c r="B111" s="3" t="inlineStr">
         <is>
           <t>印は公文書に押す国家の正式な印鑑、
-鑰は税として集めた米などを納めた
-正倉の鍵を意味する。</t>
+鑰は税として集めた米などを納めた正倉の鍵を意味する。</t>
         </is>
       </c>
       <c r="C111" s="2" t="inlineStr">
@@ -2922,8 +3060,7 @@
       <c r="B112" s="3" t="inlineStr">
         <is>
           <t>つまり印鑰を押さえることは、
-その国の行政と財産をまとめて
-手中に収めることに等しかった。</t>
+その国の行政と財産をまとめて手中に収めることに等しかった。</t>
         </is>
       </c>
       <c r="C112" s="2" t="inlineStr">
@@ -2946,8 +3083,7 @@
       <c r="B113" s="3" t="inlineStr">
         <is>
           <t>将門が国府を襲ってこれを奪った行為は、
-朝廷の支配そのものに正面から
-弓を引いたことを意味するのである。</t>
+朝廷の支配そのものに正面から弓を引いたことを意味するのである。</t>
         </is>
       </c>
       <c r="C113" s="2" t="inlineStr">
@@ -2969,7 +3105,14 @@
       </c>
       <c r="B114" s="3" t="inlineStr">
         <is>
-          <t>そっから勢いに乗った将門は、坂東、今でいう関東一帯の国府を次々落として、ほぼ関東全域を手中に収めてまう。各国の国司を追い出して、自前の人事で「ここからは俺が仕切る国や」ってやり始めた。地方の豪族が中央任命の役人をまとめて吹っ飛ばすって、当時前代未聞やってん</t>
+          <t>そっから勢いに乗った将門は、
+坂東、
+今でいう関東一帯の国府を次々落として、
+ほぼ関東全域を手中に収めてまう。
+各国の国司を追い出して、
+自前の人事で「ここからは俺が仕切る国や」ってやり始めた。
+地方の豪族が中央任命の役人をまとめて吹っ飛ばすって、
+当時前代未聞やってん</t>
         </is>
       </c>
       <c r="C114" s="2" t="inlineStr">
@@ -3035,7 +3178,8 @@
       </c>
       <c r="B117" s="3" t="inlineStr">
         <is>
-          <t>で、調子乗って新皇宣言と</t>
+          <t>で、
+調子乗って新皇宣言と</t>
         </is>
       </c>
       <c r="C117" s="2" t="inlineStr">
@@ -3057,7 +3201,14 @@
       </c>
       <c r="B118" s="3" t="inlineStr">
         <is>
-          <t>そう、ここで「新皇」、つまり新しい天皇を名乗る。伝説やと八幡神のお告げで位を授かったってことになっとるけど、要は京都の天皇とは別に、東国に自分を頂点とした朝廷を立てようとしたわけや。関東に独立政権を作るっていう、日本史でもなかなかおらんスケールの反逆やねん</t>
+          <t>そう、
+ここで「新皇」、
+つまり新しい天皇を名乗る。
+伝説やと八幡神のお告げで位を授かったってことになっとるけど、
+要は京都の天皇とは別に、
+東国に自分を頂点とした朝廷を立てようとしたわけや。
+関東に独立政権を作るっていう、
+日本史でもなかなかおらんスケールの反逆やねん</t>
         </is>
       </c>
       <c r="C118" s="2" t="inlineStr">
@@ -3079,7 +3230,8 @@
       </c>
       <c r="B119" s="3" t="inlineStr">
         <is>
-          <t>八幡のお告げは草、自分で言うてるだけやろ知らんけど</t>
+          <t>八幡のお告げは草、
+自分で言うてるだけやろ知らんけど</t>
         </is>
       </c>
       <c r="C119" s="2" t="inlineStr">
@@ -3123,7 +3275,8 @@
       </c>
       <c r="B121" s="3" t="inlineStr">
         <is>
-          <t>正直そこは盛りやろ、神託とか後付けくさいわ</t>
+          <t>正直そこは盛りやろ、
+神託とか後付けくさいわ</t>
         </is>
       </c>
       <c r="C121" s="2" t="inlineStr">
@@ -3145,7 +3298,9 @@
       </c>
       <c r="B122" s="3" t="inlineStr">
         <is>
-          <t>で？神名乗ろうがすぐ討たれたんやから、結局ただの勘違いした田舎の暴れん坊やん</t>
+          <t>で？
+神名乗ろうがすぐ討たれたんやから、
+結局ただの勘違いした田舎の暴れん坊やん</t>
         </is>
       </c>
       <c r="C122" s="2" t="inlineStr">
@@ -3167,7 +3322,8 @@
       </c>
       <c r="B123" s="3" t="inlineStr">
         <is>
-          <t>勘違いで関東一国まとめられたら誰も苦労せんわ、そこは認めたれや</t>
+          <t>勘違いで関東一国まとめられたら誰も苦労せんわ、
+そこは認めたれや</t>
         </is>
       </c>
       <c r="C123" s="2" t="inlineStr">
@@ -3211,7 +3367,13 @@
       </c>
       <c r="B125" s="3" t="inlineStr">
         <is>
-          <t>そうなる。京都は将門を朝敵認定して追討令を出す。で、ここで動いたのが同じ関東の平貞盛と、下野の豪族やった藤原秀郷や。身内や近隣やった連中が討伐側に回って、将門包囲網が出来てまうわけや</t>
+          <t>そうなる。
+京都は将門を朝敵認定して追討令を出す。
+で、
+ここで動いたのが同じ関東の平貞盛と、
+下野の豪族やった藤原秀郷や。
+身内や近隣やった連中が討伐側に回って、
+将門包囲網が出来てまうわけや</t>
         </is>
       </c>
       <c r="C125" s="2" t="inlineStr">
@@ -3299,7 +3461,10 @@
       </c>
       <c r="B129" s="3" t="inlineStr">
         <is>
-          <t>ちゃう、討ったのは平貞盛と藤原秀郷や。源氏ちゃうから、そこ混同したらあかんで</t>
+          <t>ちゃう、
+討ったのは平貞盛と藤原秀郷や。
+源氏ちゃうから、
+そこ混同したらあかんで</t>
         </is>
       </c>
       <c r="C129" s="2" t="inlineStr">
@@ -3321,7 +3486,8 @@
       </c>
       <c r="B130" s="3" t="inlineStr">
         <is>
-          <t>あっそうやったか、すまんね</t>
+          <t>あっそうやったか、
+すまんね</t>
         </is>
       </c>
       <c r="C130" s="2" t="inlineStr">
@@ -3343,7 +3509,16 @@
       </c>
       <c r="B131" s="3" t="inlineStr">
         <is>
-          <t>で、天慶3年、西暦940年に討伐軍とぶつかって、将門は敗れる。伝承やと、戦いの最中に飛んできた流れ矢が額に当たって、それが致命傷になって命を落としたって言われとる。新皇を名乗ってからわずか2か月ほどでの最期や。あれだけ関東を席巻したのに、終わりはほんま一瞬やった</t>
+          <t>で、
+天慶3年、
+西暦940年に討伐軍とぶつかって、
+将門は敗れる。
+伝承やと、
+戦いの最中に飛んできた流れ矢が額に当たって、
+それが致命傷になって命を落としたって言われとる。
+新皇を名乗ってからわずか2か月ほどでの最期や。
+あれだけ関東を席巻したのに、
+終わりはほんま一瞬やった</t>
         </is>
       </c>
       <c r="C131" s="2" t="inlineStr">
@@ -3387,7 +3562,8 @@
       </c>
       <c r="B133" s="3" t="inlineStr">
         <is>
-          <t>天下取り損ねたというか、名乗っただけで終わったやんｗ</t>
+          <t>天下取り損ねたというか、
+名乗っただけで終わったやんｗ</t>
         </is>
       </c>
       <c r="C133" s="2" t="inlineStr">
@@ -3409,7 +3585,13 @@
       </c>
       <c r="B134" s="3" t="inlineStr">
         <is>
-          <t>その最期にも伝説があってな。将門は矢も通さんと評判の無敵の体で討伐軍が苦戦しとったけど、戦いの最中に陣の風向きが急に変わって、その隙に放たれた矢が額に当たったって話が残っとる。神がかった強さやのに、最後は風っていう運否天賦みたいなもんで決着した、っていうのがまた伝説を盛り上げとるんや</t>
+          <t>その最期にも伝説があってな。
+将門は矢も通さんと評判の無敵の体で討伐軍が苦戦しとったけど、
+戦いの最中に陣の風向きが急に変わって、
+その隙に放たれた矢が額に当たったって話が残っとる。
+神がかった強さやのに、
+最後は風っていう運否天賦みたいなもんで決着した、
+っていうのがまた伝説を盛り上げとるんや</t>
         </is>
       </c>
       <c r="C134" s="2" t="inlineStr">
@@ -3475,7 +3657,13 @@
       </c>
       <c r="B137" s="3" t="inlineStr">
         <is>
-          <t>もういっこ有名なんが影武者伝説や。将門にはそっくりの影武者が何人もおって、本物を見分けられんかったけど、こめかみのあたりに本物だけ影が無かった、みたいな尾ひれが後世に付いとる。要は強すぎて普通には討てんかったっていう"負けたのが信じられん"空気が、こういう伝説を生んだわけやな</t>
+          <t>もういっこ有名なんが影武者伝説や。
+将門にはそっくりの影武者が何人もおって、
+本物を見分けられんかったけど、
+こめかみのあたりに本物だけ影が無かった、
+みたいな尾ひれが後世に付いとる。
+要は強すぎて普通には討てんかったっていう"負けたのが信じられん"空気が、
+こういう伝説を生んだわけやな</t>
         </is>
       </c>
       <c r="C137" s="2" t="inlineStr">
@@ -3519,7 +3707,10 @@
       </c>
       <c r="B139" s="3" t="inlineStr">
         <is>
-          <t>そういや将門を祀っとる国王神社が茨城にあって、将門の三女が建てたって伝わっとるな。ワイ一回行ったけど、めっちゃ静かでええとこやった</t>
+          <t>そういや将門を祀っとる国王神社が茨城にあって、
+将門の三女が建てたって伝わっとるな。
+ワイ一回行ったけど、
+めっちゃ静かでええとこやった</t>
         </is>
       </c>
       <c r="C139" s="2" t="inlineStr">
@@ -3541,7 +3732,8 @@
       </c>
       <c r="B140" s="3" t="inlineStr">
         <is>
-          <t>大河で将門やらんのかな、昔の風と雲と虹と以来やろ</t>
+          <t>大河で将門やらんのかな、
+昔の風と雲と虹と以来やろ</t>
         </is>
       </c>
       <c r="C140" s="2" t="inlineStr">
@@ -3585,7 +3777,8 @@
       </c>
       <c r="B142" s="3" t="inlineStr">
         <is>
-          <t>で、その首が飛ぶ伝説に繋がるわけやな</t>
+          <t>で、
+その首が飛ぶ伝説に繋がるわけやな</t>
         </is>
       </c>
       <c r="C142" s="2" t="inlineStr">
@@ -3607,7 +3800,11 @@
       </c>
       <c r="B143" s="3" t="inlineStr">
         <is>
-          <t>そう、討たれた首は京都に送られて晒される。で、その首が夜に飛んで関東に戻った、っていうのが前半の祟りの話に繋がるんや</t>
+          <t>そう、
+討たれた首は京都に送られて晒される。
+で、
+その首が夜に飛んで関東に戻った、
+っていうのが前半の祟りの話に繋がるんや</t>
         </is>
       </c>
       <c r="C143" s="2" t="inlineStr">
@@ -3651,7 +3848,14 @@
       </c>
       <c r="B145" s="3" t="inlineStr">
         <is>
-          <t>ちな朝廷も手をこまねいてたわけちゃうくて、将門調伏のために高僧に護摩祈祷を焚かせとってな。千葉の成田山新勝寺は、その将門調伏の祈祷をやった地に開かれたって伝わっとる。で、将門が討たれたもんやから「祈祷が効いた」ことになって、これが将門＝祟る怨霊ってイメージを後押しした面もあるんや。今でも神田明神の氏子は成田山には参らんって言われとるくらいでな</t>
+          <t>ちな朝廷も手をこまねいてたわけちゃうくて、
+将門調伏のために高僧に護摩祈祷を焚かせとってな。
+千葉の成田山新勝寺は、
+その将門調伏の祈祷をやった地に開かれたって伝わっとる。
+で、
+将門が討たれたもんやから「祈祷が効いた」ことになって、
+これが将門＝祟る怨霊ってイメージを後押しした面もあるんや。
+今でも神田明神の氏子は成田山には参らんって言われとるくらいでな</t>
         </is>
       </c>
       <c r="C145" s="2" t="inlineStr">
@@ -3673,7 +3877,9 @@
       </c>
       <c r="B146" s="3" t="inlineStr">
         <is>
-          <t>でもさ、結局こいつただの調子乗った反乱者やん。評価する要素ある？</t>
+          <t>でもさ、
+結局こいつただの調子乗った反乱者やん。
+評価する要素ある？</t>
         </is>
       </c>
       <c r="C146" s="2" t="inlineStr">
@@ -3695,7 +3901,13 @@
       </c>
       <c r="B147" s="3" t="inlineStr">
         <is>
-          <t>それがそうとも言い切れんのよ。中央の貴族が地方を搾取する仕組みに、地方の武装勢力が真っ向から「ノー」を突きつけた最初級の例なんや。後の武士が自分らの力で土地を治める時代の、いわば走りやねん。だから単なる謀反人やのうて、関東武士の精神的な元祖として評価する見方も根強いんや</t>
+          <t>それがそうとも言い切れんのよ。
+中央の貴族が地方を搾取する仕組みに、
+地方の武装勢力が真っ向から「ノー」を突きつけた最初級の例なんや。
+後の武士が自分らの力で土地を治める時代の、
+いわば走りやねん。
+だから単なる謀反人やのうて、
+関東武士の精神的な元祖として評価する見方も根強いんや</t>
         </is>
       </c>
       <c r="C147" s="2" t="inlineStr">
@@ -3717,7 +3929,8 @@
       </c>
       <c r="B148" s="3" t="inlineStr">
         <is>
-          <t>はい武士オタの過大評価、盛りすぎて引くわ</t>
+          <t>はい武士オタの過大評価、
+盛りすぎて引くわ</t>
         </is>
       </c>
       <c r="C148" s="2" t="inlineStr">
@@ -3739,7 +3952,8 @@
       </c>
       <c r="B149" s="3" t="inlineStr">
         <is>
-          <t>過大評価ってだけで片付けるのも雑やろ、現に怨霊で千年語り継がれとるんやから</t>
+          <t>過大評価ってだけで片付けるのも雑やろ、
+現に怨霊で千年語り継がれとるんやから</t>
         </is>
       </c>
       <c r="C149" s="2" t="inlineStr">
@@ -3761,7 +3975,8 @@
       </c>
       <c r="B150" s="3" t="inlineStr">
         <is>
-          <t>あと同じ時期に西で藤原純友も暴れとって、東西で同時に乱が起きとったんよな</t>
+          <t>あと同じ時期に西で藤原純友も暴れとって、
+東西で同時に乱が起きとったんよな</t>
         </is>
       </c>
       <c r="C150" s="2" t="inlineStr">
@@ -3783,7 +3998,9 @@
       </c>
       <c r="B151" s="3" t="inlineStr">
         <is>
-          <t>それや、承平天慶の乱でセット扱いされるやつ。朝廷からしたら東西挟み撃ちで生きた心地せんかったやろな</t>
+          <t>それや、
+承平天慶の乱でセット扱いされるやつ。
+朝廷からしたら東西挟み撃ちで生きた心地せんかったやろな</t>
         </is>
       </c>
       <c r="C151" s="2" t="inlineStr">
@@ -3806,8 +4023,7 @@
       <c r="B152" s="3" t="inlineStr">
         <is>
           <t>承平天慶の乱とは、
-平安時代中期に東西で同時に起きた
-二つの大きな反乱の総称である。</t>
+平安時代中期に東西で同時に起きた二つの大きな反乱の総称である。</t>
         </is>
       </c>
       <c r="C152" s="2" t="inlineStr">
@@ -3830,8 +4046,7 @@
       <c r="B153" s="3" t="inlineStr">
         <is>
           <t>東国では平将門が新皇を名乗って関東を制圧し、
-西国では瀬戸内で藤原純友が
-海賊を率いて朝廷に反旗をひるがえした。</t>
+西国では瀬戸内で藤原純友が海賊を率いて朝廷に反旗をひるがえした。</t>
         </is>
       </c>
       <c r="C153" s="2" t="inlineStr">
@@ -3853,8 +4068,7 @@
       </c>
       <c r="B154" s="3" t="inlineStr">
         <is>
-          <t>朝廷にとっては東西から同時に
-挑戦を突きつけられた前代未聞の事態であり、</t>
+          <t>朝廷にとっては東西から同時に挑戦を突きつけられた前代未聞の事態であり、</t>
         </is>
       </c>
       <c r="C154" s="2" t="inlineStr">
@@ -3876,9 +4090,7 @@
       </c>
       <c r="B155" s="3" t="inlineStr">
         <is>
-          <t>地方の武士の力を
-中央が無視できなくなっていく
-大きな転機となった出来事である。</t>
+          <t>地方の武士の力を中央が無視できなくなっていく大きな転機となった出来事である。</t>
         </is>
       </c>
       <c r="C155" s="2" t="inlineStr">
@@ -3922,7 +4134,13 @@
       </c>
       <c r="B157" s="3" t="inlineStr">
         <is>
-          <t>そこはロマンあるよな。もし討伐をしのいで東国政権が定着しとったら、関東拠点の独立勢力が早い段階で出来て、武士の世が何百年か前倒しになってたかもしれん。まあ補給も人望もまだ足りんかったから現実は厳しかったやろけど。知らんけど、たらればとしては最高に面白い人物やわ</t>
+          <t>そこはロマンあるよな。
+もし討伐をしのいで東国政権が定着しとったら、
+関東拠点の独立勢力が早い段階で出来て、
+武士の世が何百年か前倒しになってたかもしれん。
+まあ補給も人望もまだ足りんかったから現実は厳しかったやろけど。
+知らんけど、
+たらればとしては最高に面白い人物やわ</t>
         </is>
       </c>
       <c r="C157" s="2" t="inlineStr">
@@ -3966,7 +4184,8 @@
       </c>
       <c r="B159" s="3" t="inlineStr">
         <is>
-          <t>ワイ千葉県民、地味に将門ゆかりの地に住んどる</t>
+          <t>ワイ千葉県民、
+地味に将門ゆかりの地に住んどる</t>
         </is>
       </c>
       <c r="C159" s="2" t="inlineStr">
@@ -3988,7 +4207,8 @@
       </c>
       <c r="B160" s="3" t="inlineStr">
         <is>
-          <t>で、結局その首が今も大手町でブチギレてるわけやな</t>
+          <t>で、
+結局その首が今も大手町でブチギレてるわけやな</t>
         </is>
       </c>
       <c r="C160" s="2" t="inlineStr">
@@ -4010,7 +4230,8 @@
       </c>
       <c r="B161" s="3" t="inlineStr">
         <is>
-          <t>千年たっても一等地から動かんあたり、ある意味いまだに関東の主やってるとも言えるわ</t>
+          <t>千年たっても一等地から動かんあたり、
+ある意味いまだに関東の主やってるとも言えるわ</t>
         </is>
       </c>
       <c r="C161" s="2" t="inlineStr">
@@ -4054,7 +4275,9 @@
       </c>
       <c r="B163" s="3" t="inlineStr">
         <is>
-          <t>ワイ明日大手町で乗り換えあるし、ちゃんと拝んどくわ。将門さん祟らんといてな</t>
+          <t>ワイ明日大手町で乗り換えあるし、
+ちゃんと拝んどくわ。
+将門さん祟らんといてな</t>
         </is>
       </c>
       <c r="C163" s="2" t="inlineStr">
@@ -4098,8 +4321,8 @@
       </c>
       <c r="B165" s="3" t="inlineStr">
         <is>
-          <t>今回は、平将門の祟りについての
-さまざまな議論を見てきたが、
+          <t>今回は、
+平将門の祟りについてのさまざまな議論を見てきたが、
 いかがだっただろうか？</t>
         </is>
       </c>
@@ -4122,8 +4345,7 @@
       </c>
       <c r="B166" s="3" t="inlineStr">
         <is>
-          <t>2ちゃんねるの歴史オタクたちの
-議論を見ていると、</t>
+          <t>2ちゃんねるの歴史オタクたちの議論を見ていると、</t>
         </is>
       </c>
       <c r="C166" s="2" t="inlineStr">
@@ -4147,8 +4369,7 @@
         <is>
           <t>将門は単なる祟り神ではなく、
 時代に真っ向から立ち向かって果てた反骨の武将であり、
-だからこそ千年経った今も
-畏れと敬いを同時に集め続けているのだと思えた。</t>
+だからこそ千年経った今も畏れと敬いを同時に集め続けているのだと思えた。</t>
         </is>
       </c>
       <c r="C167" s="2" t="inlineStr">
@@ -4170,8 +4391,7 @@
       </c>
       <c r="B168" s="3" t="inlineStr">
         <is>
-          <t>今回の動画について他の意見や
-感想があったらぜひコメントで教えてね！</t>
+          <t>今回の動画について他の意見や感想があったらぜひコメントで教えてね！</t>
         </is>
       </c>
       <c r="C168" s="2" t="inlineStr">
@@ -4193,8 +4413,8 @@
       </c>
       <c r="B169" s="3" t="inlineStr">
         <is>
-          <t>他にも歴史にまつわる情報をまとめた
-動画が満載なので、ぜひ見てみてくださいね。
+          <t>他にも歴史にまつわる情報をまとめた動画が満載なので、
+ぜひ見てみてくださいね。
 ご視聴ありがとうございました！</t>
         </is>
       </c>

</xml_diff>

<commit_message>
auto: 2026-06-18 22:19 (3件)
</commit_message>
<xml_diff>
--- a/01_プロジェクト/YouTube/創作スレ下書き/2026-06-17_平将門の祟り_台本.xlsx
+++ b/01_プロジェクト/YouTube/創作スレ下書き/2026-06-17_平将門の祟り_台本.xlsx
@@ -1100,7 +1100,6 @@
 今度は大手町を大規模に区画整理するとき、
 塚も邪魔やからって整地しようとしたら、
 重機が作業中に横転して運転手が亡くなったって記録に残ってる。
-で、
 結局そこも工事は取りやめや。
 震災のときも戦後のときも、
 "お国"クラスがどかそうとして二回とも引き下がっとる。
@@ -1430,8 +1429,7 @@
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>で、
-その大手町の土地って今いくらすんの</t>
+          <t>てかその大手町の土地って今いくらすんの</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
@@ -1854,8 +1852,7 @@
       </c>
       <c r="B61" s="3" t="inlineStr">
         <is>
-          <t>で、
-結局三大怨霊って残り誰なん</t>
+          <t>ところで三大怨霊って残り誰なん</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr">
@@ -2399,7 +2396,6 @@
       <c r="B84" s="3" t="inlineStr">
         <is>
           <t>嘘か本当か分からんのが一番こわいんよこの人。
-で、
 そもそも将門ってなんで反乱なんか起こしたん？
 怨霊の部分しか知らんわ</t>
         </is>
@@ -2674,8 +2670,7 @@
       </c>
       <c r="B96" s="3" t="inlineStr">
         <is>
-          <t>で、
-結局こいつ何がしたかったん</t>
+          <t>結局こいつ何がしたかったん</t>
         </is>
       </c>
       <c r="C96" s="2" t="inlineStr">
@@ -2938,8 +2933,7 @@
       </c>
       <c r="B107" s="3" t="inlineStr">
         <is>
-          <t>で、
-私闘で官側の人間ともやり合ううちに、
+          <t>その私闘で官側の人間ともやり合ううちに、
 今度は朝廷の出先の国府とぶつかってまう。
 勢いで常陸の国府を攻め落として、
 国の実印にあたる印鑰まで奪ってもうた。
@@ -3178,8 +3172,7 @@
       </c>
       <c r="B117" s="3" t="inlineStr">
         <is>
-          <t>で、
-調子乗って新皇宣言と</t>
+          <t>そんで調子乗って新皇宣言と</t>
         </is>
       </c>
       <c r="C117" s="2" t="inlineStr">
@@ -3369,7 +3362,6 @@
         <is>
           <t>そうなる。
 京都は将門を朝敵認定して追討令を出す。
-で、
 ここで動いたのが同じ関東の平貞盛と、
 下野の豪族やった藤原秀郷や。
 身内や近隣やった連中が討伐側に回って、
@@ -3509,9 +3501,9 @@
       </c>
       <c r="B131" s="3" t="inlineStr">
         <is>
-          <t>で、
-天慶3年、
-西暦940年に討伐軍とぶつかって、
+          <t>そして天慶3年、
+西暦940年、
+ついに討伐軍とぶつかって、
 将門は敗れる。
 伝承やと、
 戦いの最中に飛んできた流れ矢が額に当たって、
@@ -3777,8 +3769,7 @@
       </c>
       <c r="B142" s="3" t="inlineStr">
         <is>
-          <t>で、
-その首が飛ぶ伝説に繋がるわけやな</t>
+          <t>あの首が飛ぶ伝説に繋がるわけやな</t>
         </is>
       </c>
       <c r="C142" s="2" t="inlineStr">
@@ -3802,7 +3793,6 @@
         <is>
           <t>そう、
 討たれた首は京都に送られて晒される。
-で、
 その首が夜に飛んで関東に戻った、
 っていうのが前半の祟りの話に繋がるんや</t>
         </is>
@@ -3852,7 +3842,6 @@
 将門調伏のために高僧に護摩祈祷を焚かせとってな。
 千葉の成田山新勝寺は、
 その将門調伏の祈祷をやった地に開かれたって伝わっとる。
-で、
 将門が討たれたもんやから「祈祷が効いた」ことになって、
 これが将門＝祟る怨霊ってイメージを後押しした面もあるんや。
 今でも神田明神の氏子は成田山には参らんって言われとるくらいでな</t>
@@ -4207,8 +4196,8 @@
       </c>
       <c r="B160" s="3" t="inlineStr">
         <is>
-          <t>で、
-結局その首が今も大手町でブチギレてるわけやな</t>
+          <t>つまり、
+その首が今も大手町でブチギレてるわけやな</t>
         </is>
       </c>
       <c r="C160" s="2" t="inlineStr">

</xml_diff>

<commit_message>
auto: 2026-06-18 22:39 (4件)
</commit_message>
<xml_diff>
--- a/01_プロジェクト/YouTube/創作スレ下書き/2026-06-17_平将門の祟り_台本.xlsx
+++ b/01_プロジェクト/YouTube/創作スレ下書き/2026-06-17_平将門の祟り_台本.xlsx
@@ -655,7 +655,7 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>例のやつやん</t>
+          <t>例のやつか</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -1073,8 +1073,8 @@
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>一回ならそう言えるんやけどな、
-これ二回あるねん</t>
+          <t>一回ならまだしも、
+これ二回あるからタチ悪い</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
@@ -1103,7 +1103,7 @@
 結局そこも工事は取りやめや。
 震災のときも戦後のときも、
 "お国"クラスがどかそうとして二回とも引き下がっとる。
-そこがこの塚のゾッとするとこやねん</t>
+そこがこの塚の本気でゾッとするところ</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
@@ -1126,7 +1126,7 @@
       <c r="B30" s="3" t="inlineStr">
         <is>
           <t>天下の国家事業が二度も引っ込むとか、
-相当のことやん</t>
+相当ヤバい</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
@@ -1385,7 +1385,8 @@
 力尽きて落ちた場所が今の大手町って筋書きなんよ。
 しかも落ちた候補地は一か所ちゃうくて、
 各地に「ここが本物の首塚や」っていう伝承地が点々と残っとる。
-執念で関東まで戻ってきたって話がもう只者ちゃうねん</t>
+執念で関東まで戻ってきたんやから、
+もう只者ちゃう</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
@@ -1458,7 +1459,7 @@
 塚だけポツンと残しとるわけや。
 再開発のたびに「ここだけは触らんとこ」って供養して避けて通る。
 経済合理性が全ての街のド真ん中で、
-そこだけ理屈が通らん空白地帯になっとるんや</t>
+そこだけ理屈が通らん空白地帯になっとる</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
@@ -1480,7 +1481,7 @@
       </c>
       <c r="B45" s="3" t="inlineStr">
         <is>
-          <t>数十億の更地に塚一個とか狂っとる</t>
+          <t>数十億の更地に塚一個とか正気ちゃう</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
@@ -1554,7 +1555,7 @@
 社員が塚に尻を向けんように管理職の机の向きまで気いつかっとるって言われとる。
 信じる信じへん以前に、
 ガチガチの大企業がそこまで配慮してまう空気があるってのが、
-ある意味一番の答え合わせやねん</t>
+ある意味それが一番の答え合わせ</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
@@ -1598,7 +1599,7 @@
       </c>
       <c r="B50" s="3" t="inlineStr">
         <is>
-          <t>そこまでいくともう信仰やろ</t>
+          <t>そこまでいくともう信仰の域</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
@@ -1739,7 +1740,7 @@
 要は天下の一等地のド真ん中で、
 周りの大企業が「将門さんの機嫌だけは損ねたらあかん」って共同で面倒を見続けとるわけや。
 これだけでも、
-土地そのものが特別扱いされとるのが分かるやろ</t>
+土地そのものが特別扱いされとるのが分かる</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
@@ -1806,7 +1807,7 @@
       </c>
       <c r="B59" s="3" t="inlineStr">
         <is>
-          <t>それ完全にご近所の氏神様やん</t>
+          <t>それもう完全にご近所の氏神様</t>
         </is>
       </c>
       <c r="C59" s="2" t="inlineStr">
@@ -1881,7 +1882,7 @@
 徳川が江戸入りしたとき将門を江戸の総鎮守として篤く祀り直しとるんよ。
 怒らせたら祟るけど、
 ちゃんと祀れば街を守ってくれる、
-っていう"祟り神の出世コース"に乗っとるわけや</t>
+っていう"祟り神の出世コース"に乗っとる</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
@@ -1931,7 +1932,7 @@
 っていうのが日本のおもろい癖やねん。
 最初は災いの元として恐れられた連中が、
 丁重に祀られて街や受験生を守る側に回る。
-将門もその王道を歩んどるわけや</t>
+将門もまさにその王道を歩んどる</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
@@ -1954,7 +1955,7 @@
       <c r="B65" s="3" t="inlineStr">
         <is>
           <t>落とし所が神様って発想、
-日本ぐらいやろ</t>
+日本ぐらいのもん</t>
         </is>
       </c>
       <c r="C65" s="2" t="inlineStr">
@@ -2022,7 +2023,7 @@
       </c>
       <c r="B68" s="3" t="inlineStr">
         <is>
-          <t>そこは祟りやのうて納期やろ</t>
+          <t>そこは祟りやのうて納期</t>
         </is>
       </c>
       <c r="C68" s="2" t="inlineStr">
@@ -2145,8 +2146,9 @@
 重い負担やら国府の横暴に苦しむ坂東の人らからしたら、
 中央に盾突いて「東は俺らで治める」ってやってのけた将門は反骨のシンボルやった。
 だからこそ討たれたあとも、
-祟り神として畏れられつつ土地の守り神として手厚く祀られ続けた、
-っていう二面性があるわけや</t>
+祟り神として畏れられつつ土地の守り神として手厚く祀られ続けた。
+怖がられながらも大事にされる、
+二面性のある人物やった</t>
         </is>
       </c>
       <c r="C73" s="2" t="inlineStr">
@@ -2215,7 +2217,7 @@
         <is>
           <t>結局さ、
 全部"そういうことにしとこ"の後付けやろ。
-因果の証拠なんか無いやん</t>
+因果の証拠なんか何も無い</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
@@ -2766,7 +2768,7 @@
       </c>
       <c r="B100" s="3" t="inlineStr">
         <is>
-          <t>そっからどうやって天皇になんねん</t>
+          <t>そっからどうやったら天皇まで行くん</t>
         </is>
       </c>
       <c r="C100" s="2" t="inlineStr">
@@ -2816,7 +2818,7 @@
 若い頃は京都に上って摂関家に奉公しとった時期もあって、
 決して田舎のチンピラちゃう。
 中央の作法も権力の構造も知った上で関東に戻って、
-結局その中央に弓を引くことになったわけや</t>
+結局その中央に弓を引くことになった</t>
         </is>
       </c>
       <c r="C102" s="2" t="inlineStr">
@@ -2860,7 +2862,7 @@
       </c>
       <c r="B104" s="3" t="inlineStr">
         <is>
-          <t>中身を知ってる奴が反旗ひるがえすのが一番こわいやつやん</t>
+          <t>中身を知ってる奴が反旗ひるがえすのが一番こわい</t>
         </is>
       </c>
       <c r="C104" s="2" t="inlineStr">
@@ -2888,7 +2890,7 @@
 だから機動力のある騎馬の武士団を抱えやすくて、
 中央から来た役人よりも地元で腕の立つ将門のほうが頼りにされとった。
 そういう土壌があったからこそ、
-一介の豪族が関東一円を呑み込むなんて芸当ができたわけや</t>
+一介の豪族が関東一円を呑み込むなんて芸当ができた</t>
         </is>
       </c>
       <c r="C105" s="2" t="inlineStr">
@@ -2911,7 +2913,7 @@
       <c r="B106" s="3" t="inlineStr">
         <is>
           <t>馬かよ、
-そら強いわけや</t>
+そら強いわな</t>
         </is>
       </c>
       <c r="C106" s="2" t="inlineStr">
@@ -2939,7 +2941,7 @@
 国の実印にあたる印鑰まで奪ってもうた。
 これ当時やと完全に一線を越えた行為で、
 国に弓を引いた賊って扱いになる。
-もう後戻りでけへんとこまで行ったわけや</t>
+もう後戻りでけへんとこまで行ってもうた</t>
         </is>
       </c>
       <c r="C107" s="2" t="inlineStr">
@@ -3128,7 +3130,7 @@
       </c>
       <c r="B115" s="3" t="inlineStr">
         <is>
-          <t>関東まるごとはやりすぎやろ</t>
+          <t>関東まるごとはやりすぎ</t>
         </is>
       </c>
       <c r="C115" s="2" t="inlineStr">
@@ -3150,7 +3152,7 @@
       </c>
       <c r="B116" s="3" t="inlineStr">
         <is>
-          <t>もう完全に独立国家やん</t>
+          <t>もはや完全に独立国家</t>
         </is>
       </c>
       <c r="C116" s="2" t="inlineStr">
@@ -3201,7 +3203,7 @@
 要は京都の天皇とは別に、
 東国に自分を頂点とした朝廷を立てようとしたわけや。
 関東に独立政権を作るっていう、
-日本史でもなかなかおらんスケールの反逆やねん</t>
+日本史でもなかなかおらんスケールの反逆やった</t>
         </is>
       </c>
       <c r="C118" s="2" t="inlineStr">
@@ -3293,7 +3295,7 @@
         <is>
           <t>で？
 神名乗ろうがすぐ討たれたんやから、
-結局ただの勘違いした田舎の暴れん坊やん</t>
+結局ただの勘違いした田舎の暴れん坊</t>
         </is>
       </c>
       <c r="C122" s="2" t="inlineStr">
@@ -3338,7 +3340,7 @@
       </c>
       <c r="B124" s="3" t="inlineStr">
         <is>
-          <t>でもこんなん中央がブチギレて終わりやん</t>
+          <t>でもこんなん中央がブチギレて一発で終わり</t>
         </is>
       </c>
       <c r="C124" s="2" t="inlineStr">
@@ -3355,7 +3357,7 @@
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
         <is>
-          <t>女性B大</t>
+          <t>女性B</t>
         </is>
       </c>
       <c r="B125" s="3" t="inlineStr">
@@ -3365,7 +3367,7 @@
 ここで動いたのが同じ関東の平貞盛と、
 下野の豪族やった藤原秀郷や。
 身内や近隣やった連中が討伐側に回って、
-将門包囲網が出来てまうわけや</t>
+将門包囲網が出来てまう</t>
         </is>
       </c>
       <c r="C125" s="2" t="inlineStr">
@@ -3382,7 +3384,7 @@
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
         <is>
-          <t>男性C</t>
+          <t>男性C下</t>
         </is>
       </c>
       <c r="B126" s="3" t="inlineStr">
@@ -3532,7 +3534,7 @@
       </c>
       <c r="B132" s="3" t="inlineStr">
         <is>
-          <t>2か月て短すぎやろ</t>
+          <t>2か月て短すぎ</t>
         </is>
       </c>
       <c r="C132" s="2" t="inlineStr">
@@ -3555,7 +3557,7 @@
       <c r="B133" s="3" t="inlineStr">
         <is>
           <t>天下取り損ねたというか、
-名乗っただけで終わったやんｗ</t>
+名乗っただけで終わっとるｗ</t>
         </is>
       </c>
       <c r="C133" s="2" t="inlineStr">
@@ -3583,7 +3585,7 @@
 その隙に放たれた矢が額に当たったって話が残っとる。
 神がかった強さやのに、
 最後は風っていう運否天賦みたいなもんで決着した、
-っていうのがまた伝説を盛り上げとるんや</t>
+っていうのがまた伝説をさらに盛り上げる</t>
         </is>
       </c>
       <c r="C134" s="2" t="inlineStr">
@@ -3605,7 +3607,7 @@
       </c>
       <c r="B135" s="3" t="inlineStr">
         <is>
-          <t>急に弱点が出てくるの少年漫画やん</t>
+          <t>急に弱点出てくるの少年漫画かよ</t>
         </is>
       </c>
       <c r="C135" s="2" t="inlineStr">
@@ -3794,7 +3796,7 @@
           <t>そう、
 討たれた首は京都に送られて晒される。
 その首が夜に飛んで関東に戻った、
-っていうのが前半の祟りの話に繋がるんや</t>
+っていうのが前半の祟りの話に繋がる</t>
         </is>
       </c>
       <c r="C143" s="2" t="inlineStr">
@@ -3896,7 +3898,7 @@
 後の武士が自分らの力で土地を治める時代の、
 いわば走りやねん。
 だから単なる謀反人やのうて、
-関東武士の精神的な元祖として評価する見方も根強いんや</t>
+関東武士の精神的な元祖として評価する見方も根強い</t>
         </is>
       </c>
       <c r="C147" s="2" t="inlineStr">
@@ -4242,7 +4244,7 @@
       </c>
       <c r="B162" s="3" t="inlineStr">
         <is>
-          <t>うまいこと言うやん</t>
+          <t>うまいこと言うな</t>
         </is>
       </c>
       <c r="C162" s="2" t="inlineStr">

</xml_diff>

<commit_message>
auto: 2026-06-18 23:19 (5件)
</commit_message>
<xml_diff>
--- a/01_プロジェクト/YouTube/創作スレ下書き/2026-06-17_平将門の祟り_台本.xlsx
+++ b/01_プロジェクト/YouTube/創作スレ下書き/2026-06-17_平将門の祟り_台本.xlsx
@@ -772,9 +772,9 @@
 工事関係者やら省の職員が立て続けに倒れて、
 当時の大蔵大臣やった早速整爾まで亡くなった。
 さすがに省内で「将門の祟りや」って噂が広がって、
-結局その仮庁舎を取り壊しとる。
+その仮庁舎を取り壊しとる。
 お役所が一回建てたもん壊すんやで、
-相当の騒ぎやったってことや</t>
+相当の騒ぎやったんや</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -1100,9 +1100,9 @@
 今度は大手町を大規模に区画整理するとき、
 塚も邪魔やからって整地しようとしたら、
 重機が作業中に横転して運転手が亡くなったって記録に残ってる。
-結局そこも工事は取りやめや。
+そこも結局工事は取りやめや。
 震災のときも戦後のときも、
-"お国"クラスがどかそうとして二回とも引き下がっとる。
+国クラスがどかそうとして二回とも引き下がっとる。
 そこがこの塚の本気でゾッとするところ</t>
         </is>
       </c>
@@ -1452,14 +1452,13 @@
       </c>
       <c r="B44" s="3" t="inlineStr">
         <is>
-          <t>それがな、
-丸の内のド真ん中の超一等地で、
+          <t>それが丸の内のど真ん中の超一等地でな、
 更地の地価で数十億とも言われとる。
 普通やったらビルが何本も建つ土地に、
-塚だけポツンと残しとるわけや。
+塚だけ残してる。
 再開発のたびに「ここだけは触らんとこ」って供養して避けて通る。
-経済合理性が全ての街のド真ん中で、
-そこだけ理屈が通らん空白地帯になっとる</t>
+経済合理性が全ての街のど真ん中で、
+そこだけ理屈が通らん空白地帯になってる</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
@@ -1552,7 +1551,7 @@
           <t>周りのビルがまた徹底しててな。
 塚を見下ろさんように、
 塚に面した側はわざと窓を作らへんとか、
-社員が塚に尻を向けんように管理職の机の向きまで気いつかっとるって言われとる。
+社員が塚に尻を向けんように管理職の机の向きまで気いつかっとるらしいで。
 信じる信じへん以前に、
 ガチガチの大企業がそこまで配慮してまう空気があるってのが、
 ある意味それが一番の答え合わせ</t>
@@ -1736,9 +1735,9 @@
         <is>
           <t>しかも今の塚は地元の企業が金を出し合って守っとるんよ。
 「史蹟将門塚保存会」っちゅう近隣の会社が集まった団体が、
-浄財で周りの清掃や整備をずっと続けとる。
-要は天下の一等地のド真ん中で、
-周りの大企業が「将門さんの機嫌だけは損ねたらあかん」って共同で面倒を見続けとるわけや。
+浄財で周りの清掃や整備をずっと続けてる。
+つまり天下の一等地のど真ん中で、
+周りの大企業が「将門さんの機嫌だけは損ねたらあかん」って共同で面倒を見続けてる。
 これだけでも、
 土地そのものが特別扱いされとるのが分かる</t>
         </is>
@@ -1875,14 +1874,13 @@
       </c>
       <c r="B62" s="3" t="inlineStr">
         <is>
-          <t>これ豆な、
-将門は今や神田明神の祭神になっとって、
-崇徳上皇・菅原道真と並んで日本三大怨霊に数えられとる。
+          <t>将門は今や神田明神の祭神になっとってな、
+崇徳上皇・菅原道真と並ぶ日本三大怨霊の一人や。
 面白いのが、
-徳川が江戸入りしたとき将門を江戸の総鎮守として篤く祀り直しとるんよ。
+徳川が江戸入りしたとき将門を江戸の総鎮守として篤く祀り直してる。
 怒らせたら祟るけど、
 ちゃんと祀れば街を守ってくれる、
-っていう"祟り神の出世コース"に乗っとる</t>
+いわば祟り神の出世コースや</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
@@ -1929,7 +1927,7 @@
           <t>その道真なんか今や学問の神様で、
 受験シーズンに全国の受験生が手を合わせに行くレベルやからな。
 恐れられた怨霊ほど後世の祀られ方が手厚なる、
-っていうのが日本のおもろい癖やねん。
+っていうのが日本のおもろい癖や。
 最初は災いの元として恐れられた連中が、
 丁重に祀られて街や受験生を守る側に回る。
 将門もまさにその王道を歩んどる</t>
@@ -2140,8 +2138,7 @@
       </c>
       <c r="B73" s="3" t="inlineStr">
         <is>
-          <t>ここ大事なんやけど、
-将門はただ恐れられただけちゃうくて、
+          <t>将門はただ恐れられただけちゃうくて、
 もともとは関東の民にとっては英雄寄りの存在やったんよ。
 重い負担やら国府の横暴に苦しむ坂東の人らからしたら、
 中央に盾突いて「東は俺らで治める」ってやってのけた将門は反骨のシンボルやった。
@@ -2215,8 +2212,8 @@
       </c>
       <c r="B76" s="3" t="inlineStr">
         <is>
-          <t>結局さ、
-全部"そういうことにしとこ"の後付けやろ。
+          <t>てかさ、
+全部そういうことにしとこの後付けやろ。
 因果の証拠なんか何も無い</t>
         </is>
       </c>
@@ -2627,7 +2624,7 @@
       </c>
       <c r="B94" s="3" t="inlineStr">
         <is>
-          <t>結局その新皇とやらも2か月で終わった負け犬やん、
+          <t>その新皇とやらも2か月で終わった負け犬やん、
 持ち上げる要素ある？</t>
         </is>
       </c>
@@ -2672,7 +2669,8 @@
       </c>
       <c r="B96" s="3" t="inlineStr">
         <is>
-          <t>結局こいつ何がしたかったん</t>
+          <t>で、
+こいつ何がしたかったん</t>
         </is>
       </c>
       <c r="C96" s="2" t="inlineStr">
@@ -2717,13 +2715,12 @@
       </c>
       <c r="B98" s="3" t="inlineStr">
         <is>
-          <t>それがな、
-最初っから天皇に盾突こうとしてたわけちゃうんよ。
+          <t>それが最初っから天皇に盾突こうとしてたわけちゃうんよ。
 スタートはただの一族内のもめ事や。
 関東の平氏一門で、
 伯父さんらと土地や縁談がらみの私闘をやっとった、
-いわば身内ゲンカからの叩き上げやねん。
-それが勝ち続けるうちに、
+いわば身内ゲンカからの叩き上げや。
+そんで勝ち続けるうちに、
 どんどん引くに引けん大ごとになってってもうた</t>
         </is>
       </c>
@@ -2790,7 +2787,8 @@
       </c>
       <c r="B101" s="3" t="inlineStr">
         <is>
-          <t>ヤンキーの抗争がいつの間にか国盗りになる漫画みたいや</t>
+          <t>身内のもめ事がいつの間にか国盗りになるとか、
+流れがエグいな</t>
         </is>
       </c>
       <c r="C101" s="2" t="inlineStr">
@@ -2812,13 +2810,13 @@
       </c>
       <c r="B102" s="3" t="inlineStr">
         <is>
-          <t>そもそも将門の出自も知っとくとええで。
+          <t>将門の出自も知っとくとええで。
 あいつ桓武天皇の血を引く桓武平氏で、
 高望王の孫にあたる名門の出やねん。
 若い頃は京都に上って摂関家に奉公しとった時期もあって、
 決して田舎のチンピラちゃう。
 中央の作法も権力の構造も知った上で関東に戻って、
-結局その中央に弓を引くことになった</t>
+そのまま中央に弓を引くことになった</t>
         </is>
       </c>
       <c r="C102" s="2" t="inlineStr">
@@ -2840,7 +2838,7 @@
       </c>
       <c r="B103" s="3" t="inlineStr">
         <is>
-          <t>元エリートが地元で反乱とか厨二すぎる</t>
+          <t>中央仕込みの男が地元で反乱とか飛躍すぎやろ</t>
         </is>
       </c>
       <c r="C103" s="2" t="inlineStr">
@@ -2884,7 +2882,9 @@
       </c>
       <c r="B105" s="3" t="inlineStr">
         <is>
-          <t>ちな将門の地盤は下総の猿島あたりでな、
+          <t>元エリートが地元で反乱は確かに厨二やけど、
+地盤の話すると腑に落ちるで。
+将門の本拠は下総の猿島あたりでな、
 当時の坂東は朝廷の目が届きにくい辺境で、
 しかも良馬の産地やった。
 だから機動力のある騎馬の武士団を抱えやすくて、
@@ -3200,8 +3200,8 @@
 ここで「新皇」、
 つまり新しい天皇を名乗る。
 伝説やと八幡神のお告げで位を授かったってことになっとるけど、
-要は京都の天皇とは別に、
-東国に自分を頂点とした朝廷を立てようとしたわけや。
+ようは京都の天皇とは別に、
+東国に自分を頂点とした朝廷を立てようとしたんや。
 関東に独立政権を作るっていう、
 日本史でもなかなかおらんスケールの反逆やった</t>
         </is>
@@ -3295,7 +3295,7 @@
         <is>
           <t>で？
 神名乗ろうがすぐ討たれたんやから、
-結局ただの勘違いした田舎の暴れん坊</t>
+しょせんただの勘違いした田舎の暴れん坊</t>
         </is>
       </c>
       <c r="C122" s="2" t="inlineStr">
@@ -3656,8 +3656,8 @@
 本物を見分けられんかったけど、
 こめかみのあたりに本物だけ影が無かった、
 みたいな尾ひれが後世に付いとる。
-要は強すぎて普通には討てんかったっていう"負けたのが信じられん"空気が、
-こういう伝説を生んだわけやな</t>
+つまり強すぎて普通には討てんかったっていう負けたのが信じられん空気が、
+こういう伝説を生んだんやろな</t>
         </is>
       </c>
       <c r="C137" s="2" t="inlineStr">
@@ -3840,10 +3840,10 @@
       </c>
       <c r="B145" s="3" t="inlineStr">
         <is>
-          <t>ちな朝廷も手をこまねいてたわけちゃうくて、
+          <t>朝廷も手をこまねいてたわけちゃうくてな、
 将門調伏のために高僧に護摩祈祷を焚かせとってな。
 千葉の成田山新勝寺は、
-その将門調伏の祈祷をやった地に開かれたって伝わっとる。
+その将門調伏の祈祷をやった地に開かれたって伝わってる。
 将門が討たれたもんやから「祈祷が効いた」ことになって、
 これが将門＝祟る怨霊ってイメージを後押しした面もあるんや。
 今でも神田明神の氏子は成田山には参らんって言われとるくらいでな</t>
@@ -3869,7 +3869,7 @@
       <c r="B146" s="3" t="inlineStr">
         <is>
           <t>でもさ、
-結局こいつただの調子乗った反乱者やん。
+こいつしょせん調子乗った反乱者やん。
 評価する要素ある？</t>
         </is>
       </c>
@@ -3892,7 +3892,8 @@
       </c>
       <c r="B147" s="3" t="inlineStr">
         <is>
-          <t>それがそうとも言い切れんのよ。
+          <t>いや、
+そうとも言い切れん。
 中央の貴族が地方を搾取する仕組みに、
 地方の武装勢力が真っ向から「ノー」を突きつけた最初級の例なんや。
 後の武士が自分らの力で土地を治める時代の、

</xml_diff>

<commit_message>
auto: 2026-06-19 21:48 (9件)
</commit_message>
<xml_diff>
--- a/01_プロジェクト/YouTube/創作スレ下書き/2026-06-17_平将門の祟り_台本.xlsx
+++ b/01_プロジェクト/YouTube/創作スレ下書き/2026-06-17_平将門の祟り_台本.xlsx
@@ -39,7 +39,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00305496"/>
+        <fgColor rgb="002F5597"/>
       </patternFill>
     </fill>
   </fills>
@@ -55,14 +55,19 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top"/>
+      <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -432,9 +437,9 @@
   <dimension ref="A1:D169"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="48" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="60" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
     <col width="6" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
@@ -472,7 +477,7 @@
 「日本三大怨霊」「祟り神」そんな恐ろしいイメージを持つ人も多いだろう。</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C2" s="4" t="inlineStr">
         <is>
           <t>冒頭</t>
         </is>
@@ -497,7 +502,7 @@
 意外と知られていない。</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="C3" s="4" t="inlineStr">
         <is>
           <t>冒頭</t>
         </is>
@@ -521,7 +526,7 @@
 国家規模の開発計画が二度も中止に追い込まれている。</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>冒頭</t>
         </is>
@@ -544,7 +549,7 @@
 平将門はなぜ千年も恐れられる怨霊となったのだろうか？</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="C5" s="4" t="inlineStr">
         <is>
           <t>冒頭</t>
         </is>
@@ -568,7 +573,7 @@
 2ちゃんねるの歴史オタクたちを見ていこう。</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="C6" s="4" t="inlineStr">
         <is>
           <t>冒頭</t>
         </is>
@@ -592,7 +597,7 @@
 その壮絶な生涯がきっとわかるだろう。</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="C7" s="4" t="inlineStr">
         <is>
           <t>冒頭</t>
         </is>
@@ -614,7 +619,7 @@
           <t>大手町のド真ん中に将門の首塚だけ残ってる理由ｗｗｗ</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="C8" s="4" t="inlineStr">
         <is>
           <t>スレ①</t>
         </is>
@@ -636,7 +641,7 @@
           <t>また出たなこの話</t>
         </is>
       </c>
-      <c r="C9" s="2" t="inlineStr">
+      <c r="C9" s="4" t="inlineStr">
         <is>
           <t>スレ①</t>
         </is>
@@ -658,7 +663,7 @@
           <t>例のやつか</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr">
+      <c r="C10" s="4" t="inlineStr">
         <is>
           <t>スレ①</t>
         </is>
@@ -680,7 +685,7 @@
           <t>あー呪われたわ</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="C11" s="4" t="inlineStr">
         <is>
           <t>スレ①</t>
         </is>
@@ -699,10 +704,10 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>首だけ飛んできた御仁やろ</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
+          <t>首だけ飛んできたやべえおっさんやろ</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
         <is>
           <t>スレ①</t>
         </is>
@@ -725,7 +730,7 @@
 ぜんぶ偶然やろ</t>
         </is>
       </c>
-      <c r="C13" s="2" t="inlineStr">
+      <c r="C13" s="4" t="inlineStr">
         <is>
           <t>スレ①</t>
         </is>
@@ -747,7 +752,7 @@
           <t>ソースは？</t>
         </is>
       </c>
-      <c r="C14" s="2" t="inlineStr">
+      <c r="C14" s="4" t="inlineStr">
         <is>
           <t>スレ①</t>
         </is>
@@ -777,7 +782,7 @@
 相当の騒ぎやったんや</t>
         </is>
       </c>
-      <c r="C15" s="2" t="inlineStr">
+      <c r="C15" s="4" t="inlineStr">
         <is>
           <t>スレ①</t>
         </is>
@@ -799,7 +804,7 @@
           <t>ファッ!?大臣まで逝ったんか</t>
         </is>
       </c>
-      <c r="C16" s="2" t="inlineStr">
+      <c r="C16" s="4" t="inlineStr">
         <is>
           <t>スレ①</t>
         </is>
@@ -821,7 +826,7 @@
           <t>草どころちゃうわ</t>
         </is>
       </c>
-      <c r="C17" s="2" t="inlineStr">
+      <c r="C17" s="4" t="inlineStr">
         <is>
           <t>スレ①</t>
         </is>
@@ -840,10 +845,10 @@
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>そら役人もビビるわな</t>
-        </is>
-      </c>
-      <c r="C18" s="2" t="inlineStr">
+          <t>役人もそらビビるわな</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
         <is>
           <t>スレ①</t>
         </is>
@@ -866,7 +871,7 @@
 それで騒ぎになったんやろ</t>
         </is>
       </c>
-      <c r="C19" s="2" t="inlineStr">
+      <c r="C19" s="4" t="inlineStr">
         <is>
           <t>スレ①</t>
         </is>
@@ -891,7 +896,7 @@
 そこは正しく覚えとけ</t>
         </is>
       </c>
-      <c r="C20" s="2" t="inlineStr">
+      <c r="C20" s="4" t="inlineStr">
         <is>
           <t>スレ①</t>
         </is>
@@ -914,7 +919,7 @@
 おう…とにかく偉い人が立て続けに倒れたんやな</t>
         </is>
       </c>
-      <c r="C21" s="2" t="inlineStr">
+      <c r="C21" s="4" t="inlineStr">
         <is>
           <t>スレ①</t>
         </is>
@@ -938,7 +943,7 @@
 首塚の跡地に建てられた大蔵省の仮庁舎で相次いだ不審な出来事を指す。</t>
         </is>
       </c>
-      <c r="C22" s="2" t="inlineStr">
+      <c r="C22" s="4" t="inlineStr">
         <is>
           <t>解説：大蔵省仮庁舎の祟り</t>
         </is>
@@ -962,7 +967,7 @@
 将門の祟りだと省内で噂された。</t>
         </is>
       </c>
-      <c r="C23" s="2" t="inlineStr">
+      <c r="C23" s="4" t="inlineStr">
         <is>
           <t>解説：大蔵省仮庁舎の祟り</t>
         </is>
@@ -985,7 +990,7 @@
 跡地に鎮魂の碑を建てている。</t>
         </is>
       </c>
-      <c r="C24" s="2" t="inlineStr">
+      <c r="C24" s="4" t="inlineStr">
         <is>
           <t>解説：大蔵省仮庁舎の祟り</t>
         </is>
@@ -1008,7 +1013,7 @@
 極めて異例の出来事として語り継がれている。</t>
         </is>
       </c>
-      <c r="C25" s="2" t="inlineStr">
+      <c r="C25" s="4" t="inlineStr">
         <is>
           <t>解説：大蔵省仮庁舎の祟り</t>
         </is>
@@ -1027,11 +1032,11 @@
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>でもその年代の偉い人なんてポンポン亡くなるやろ、
+          <t>でもその年代の偉い人なんて立て続けに亡くなるやろ、
 こじつけやって</t>
         </is>
       </c>
-      <c r="C26" s="2" t="inlineStr">
+      <c r="C26" s="4" t="inlineStr">
         <is>
           <t>スレ①</t>
         </is>
@@ -1054,7 +1059,7 @@
 後から祟りってことにしただけやろ</t>
         </is>
       </c>
-      <c r="C27" s="2" t="inlineStr">
+      <c r="C27" s="4" t="inlineStr">
         <is>
           <t>スレ①</t>
         </is>
@@ -1077,7 +1082,7 @@
 これ二回あるからタチ悪い</t>
         </is>
       </c>
-      <c r="C28" s="2" t="inlineStr">
+      <c r="C28" s="4" t="inlineStr">
         <is>
           <t>スレ①</t>
         </is>
@@ -1106,7 +1111,7 @@
 そこがこの塚の本気でゾッとするところ</t>
         </is>
       </c>
-      <c r="C29" s="2" t="inlineStr">
+      <c r="C29" s="4" t="inlineStr">
         <is>
           <t>スレ①</t>
         </is>
@@ -1129,7 +1134,7 @@
 相当ヤバい</t>
         </is>
       </c>
-      <c r="C30" s="2" t="inlineStr">
+      <c r="C30" s="4" t="inlineStr">
         <is>
           <t>スレ①</t>
         </is>
@@ -1151,7 +1156,7 @@
           <t>国家権力に二連勝してる時点で将門つよすぎやろ</t>
         </is>
       </c>
-      <c r="C31" s="2" t="inlineStr">
+      <c r="C31" s="4" t="inlineStr">
         <is>
           <t>スレ①</t>
         </is>
@@ -1170,10 +1175,11 @@
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>知らんけどお役所がオカルトでビビって引くとかある？</t>
-        </is>
-      </c>
-      <c r="C32" s="2" t="inlineStr">
+          <t>お役所がオカルトでビビって引くとかあるか？
+知らんけど</t>
+        </is>
+      </c>
+      <c r="C32" s="4" t="inlineStr">
         <is>
           <t>スレ①</t>
         </is>
@@ -1196,7 +1202,7 @@
 塚が一等地に今も残ってるのは事実やしな</t>
         </is>
       </c>
-      <c r="C33" s="2" t="inlineStr">
+      <c r="C33" s="4" t="inlineStr">
         <is>
           <t>スレ①</t>
         </is>
@@ -1215,11 +1221,11 @@
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>そもそも首塚って京都にあるんちゃうの？
+          <t>首塚って京都にあるんちゃうの？
 晒し首にされたんやろ</t>
         </is>
       </c>
-      <c r="C34" s="2" t="inlineStr">
+      <c r="C34" s="4" t="inlineStr">
         <is>
           <t>スレ①</t>
         </is>
@@ -1244,7 +1250,7 @@
 話が混ざっとるで</t>
         </is>
       </c>
-      <c r="C35" s="2" t="inlineStr">
+      <c r="C35" s="4" t="inlineStr">
         <is>
           <t>スレ①</t>
         </is>
@@ -1266,7 +1272,7 @@
           <t>はえ〜首が自走するんか</t>
         </is>
       </c>
-      <c r="C36" s="2" t="inlineStr">
+      <c r="C36" s="4" t="inlineStr">
         <is>
           <t>スレ①</t>
         </is>
@@ -1290,7 +1296,7 @@
 討たれた将門の首を祀ったとされる塚である。</t>
         </is>
       </c>
-      <c r="C37" s="2" t="inlineStr">
+      <c r="C37" s="4" t="inlineStr">
         <is>
           <t>解説：将門の首塚</t>
         </is>
@@ -1315,7 +1321,7 @@
 東京・大手町に今も残っている。</t>
         </is>
       </c>
-      <c r="C38" s="2" t="inlineStr">
+      <c r="C38" s="4" t="inlineStr">
         <is>
           <t>解説：将門の首塚</t>
         </is>
@@ -1338,7 +1344,7 @@
 たびたび不審な出来事が噂されてきた。</t>
         </is>
       </c>
-      <c r="C39" s="2" t="inlineStr">
+      <c r="C39" s="4" t="inlineStr">
         <is>
           <t>解説：将門の首塚</t>
         </is>
@@ -1361,7 +1367,7 @@
 神田明神では江戸を守る祭神として篤く祀られている存在でもある。</t>
         </is>
       </c>
-      <c r="C40" s="2" t="inlineStr">
+      <c r="C40" s="4" t="inlineStr">
         <is>
           <t>解説：将門の首塚</t>
         </is>
@@ -1389,7 +1395,7 @@
 もう只者ちゃう</t>
         </is>
       </c>
-      <c r="C41" s="2" t="inlineStr">
+      <c r="C41" s="4" t="inlineStr">
         <is>
           <t>スレ①</t>
         </is>
@@ -1411,7 +1417,7 @@
           <t>力尽きた先が一等地ってセンスよ</t>
         </is>
       </c>
-      <c r="C42" s="2" t="inlineStr">
+      <c r="C42" s="4" t="inlineStr">
         <is>
           <t>スレ①</t>
         </is>
@@ -1433,7 +1439,7 @@
           <t>てかその大手町の土地って今いくらすんの</t>
         </is>
       </c>
-      <c r="C43" s="2" t="inlineStr">
+      <c r="C43" s="4" t="inlineStr">
         <is>
           <t>スレ①</t>
         </is>
@@ -1452,7 +1458,7 @@
       </c>
       <c r="B44" s="3" t="inlineStr">
         <is>
-          <t>それが丸の内のど真ん中の超一等地でな、
+          <t>丸の内のど真ん中の超一等地でな、
 更地の地価で数十億とも言われとる。
 普通やったらビルが何本も建つ土地に、
 塚だけ残してる。
@@ -1461,7 +1467,7 @@
 そこだけ理屈が通らん空白地帯になってる</t>
         </is>
       </c>
-      <c r="C44" s="2" t="inlineStr">
+      <c r="C44" s="4" t="inlineStr">
         <is>
           <t>スレ①</t>
         </is>
@@ -1483,7 +1489,7 @@
           <t>数十億の更地に塚一個とか正気ちゃう</t>
         </is>
       </c>
-      <c r="C45" s="2" t="inlineStr">
+      <c r="C45" s="4" t="inlineStr">
         <is>
           <t>スレ①</t>
         </is>
@@ -1506,7 +1512,7 @@
 全部こじつけ</t>
         </is>
       </c>
-      <c r="C46" s="2" t="inlineStr">
+      <c r="C46" s="4" t="inlineStr">
         <is>
           <t>スレ①</t>
         </is>
@@ -1529,7 +1535,7 @@
 二回も国家側が引き下がってる事実は消えへんで</t>
         </is>
       </c>
-      <c r="C47" s="2" t="inlineStr">
+      <c r="C47" s="4" t="inlineStr">
         <is>
           <t>スレ①</t>
         </is>
@@ -1557,7 +1563,7 @@
 ある意味それが一番の答え合わせ</t>
         </is>
       </c>
-      <c r="C48" s="2" t="inlineStr">
+      <c r="C48" s="4" t="inlineStr">
         <is>
           <t>スレ①</t>
         </is>
@@ -1579,7 +1585,7 @@
           <t>こっわ</t>
         </is>
       </c>
-      <c r="C49" s="2" t="inlineStr">
+      <c r="C49" s="4" t="inlineStr">
         <is>
           <t>スレ①</t>
         </is>
@@ -1598,10 +1604,10 @@
       </c>
       <c r="B50" s="3" t="inlineStr">
         <is>
-          <t>そこまでいくともう信仰の域</t>
-        </is>
-      </c>
-      <c r="C50" s="2" t="inlineStr">
+          <t>ここまでいくともう信仰の域</t>
+        </is>
+      </c>
+      <c r="C50" s="4" t="inlineStr">
         <is>
           <t>スレ①</t>
         </is>
@@ -1623,7 +1629,7 @@
           <t>それ全部ほんまなん？</t>
         </is>
       </c>
-      <c r="C51" s="2" t="inlineStr">
+      <c r="C51" s="4" t="inlineStr">
         <is>
           <t>スレ①</t>
         </is>
@@ -1648,7 +1654,7 @@
 割と有名な話やで</t>
         </is>
       </c>
-      <c r="C52" s="2" t="inlineStr">
+      <c r="C52" s="4" t="inlineStr">
         <is>
           <t>スレ①</t>
         </is>
@@ -1670,7 +1676,7 @@
           <t>口座名義・平将門ｗｗ</t>
         </is>
       </c>
-      <c r="C53" s="2" t="inlineStr">
+      <c r="C53" s="4" t="inlineStr">
         <is>
           <t>スレ①</t>
         </is>
@@ -1689,10 +1695,10 @@
       </c>
       <c r="B54" s="3" t="inlineStr">
         <is>
-          <t>通帳に平将門て書いてあるん想像したら草</t>
-        </is>
-      </c>
-      <c r="C54" s="2" t="inlineStr">
+          <t>通帳に平将門て書いてあるん想像してもうたわ</t>
+        </is>
+      </c>
+      <c r="C54" s="4" t="inlineStr">
         <is>
           <t>スレ①</t>
         </is>
@@ -1714,7 +1720,7 @@
           <t>ワイのばあちゃん神田明神の氏子やで</t>
         </is>
       </c>
-      <c r="C55" s="2" t="inlineStr">
+      <c r="C55" s="4" t="inlineStr">
         <is>
           <t>スレ①</t>
         </is>
@@ -1733,7 +1739,7 @@
       </c>
       <c r="B56" s="3" t="inlineStr">
         <is>
-          <t>しかも今の塚は地元の企業が金を出し合って守っとるんよ。
+          <t>今の塚は地元の企業が金を出し合って守っとるんよ。
 「史蹟将門塚保存会」っちゅう近隣の会社が集まった団体が、
 浄財で周りの清掃や整備をずっと続けてる。
 つまり天下の一等地のど真ん中で、
@@ -1742,7 +1748,7 @@
 土地そのものが特別扱いされとるのが分かる</t>
         </is>
       </c>
-      <c r="C56" s="2" t="inlineStr">
+      <c r="C56" s="4" t="inlineStr">
         <is>
           <t>スレ①</t>
         </is>
@@ -1764,7 +1770,7 @@
           <t>企業が金出し合って塚守っとるの好き</t>
         </is>
       </c>
-      <c r="C57" s="2" t="inlineStr">
+      <c r="C57" s="4" t="inlineStr">
         <is>
           <t>スレ①</t>
         </is>
@@ -1787,7 +1793,7 @@
 毎朝コンビニ寄る感覚で手だけ合わせて通勤しとったわ</t>
         </is>
       </c>
-      <c r="C58" s="2" t="inlineStr">
+      <c r="C58" s="4" t="inlineStr">
         <is>
           <t>スレ①</t>
         </is>
@@ -1806,10 +1812,10 @@
       </c>
       <c r="B59" s="3" t="inlineStr">
         <is>
-          <t>それもう完全にご近所の氏神様</t>
-        </is>
-      </c>
-      <c r="C59" s="2" t="inlineStr">
+          <t>もう完全にご近所の氏神様やん</t>
+        </is>
+      </c>
+      <c r="C59" s="4" t="inlineStr">
         <is>
           <t>スレ①</t>
         </is>
@@ -1833,7 +1839,7 @@
 最初なんの土産物屋かと思った</t>
         </is>
       </c>
-      <c r="C60" s="2" t="inlineStr">
+      <c r="C60" s="4" t="inlineStr">
         <is>
           <t>スレ①</t>
         </is>
@@ -1855,7 +1861,7 @@
           <t>ところで三大怨霊って残り誰なん</t>
         </is>
       </c>
-      <c r="C61" s="2" t="inlineStr">
+      <c r="C61" s="4" t="inlineStr">
         <is>
           <t>スレ①</t>
         </is>
@@ -1883,7 +1889,7 @@
 いわば祟り神の出世コースや</t>
         </is>
       </c>
-      <c r="C62" s="2" t="inlineStr">
+      <c r="C62" s="4" t="inlineStr">
         <is>
           <t>スレ①</t>
         </is>
@@ -1905,7 +1911,7 @@
           <t>祟り神が守り神に出世しとるの草</t>
         </is>
       </c>
-      <c r="C63" s="2" t="inlineStr">
+      <c r="C63" s="4" t="inlineStr">
         <is>
           <t>スレ①</t>
         </is>
@@ -1924,16 +1930,14 @@
       </c>
       <c r="B64" s="3" t="inlineStr">
         <is>
-          <t>その道真なんか今や学問の神様で、
+          <t>道真なんか今や学問の神様で、
 受験シーズンに全国の受験生が手を合わせに行くレベルやからな。
 恐れられた怨霊ほど後世の祀られ方が手厚なる、
-っていうのが日本のおもろい癖や。
-最初は災いの元として恐れられた連中が、
-丁重に祀られて街や受験生を守る側に回る。
-将門もまさにその王道を歩んどる</t>
-        </is>
-      </c>
-      <c r="C64" s="2" t="inlineStr">
+っていうのが日本のおもろい癖やわ。
+将門もまんまその王道を歩んどる</t>
+        </is>
+      </c>
+      <c r="C64" s="4" t="inlineStr">
         <is>
           <t>スレ①</t>
         </is>
@@ -1956,7 +1960,7 @@
 日本ぐらいのもん</t>
         </is>
       </c>
-      <c r="C65" s="2" t="inlineStr">
+      <c r="C65" s="4" t="inlineStr">
         <is>
           <t>スレ①</t>
         </is>
@@ -1980,7 +1984,7 @@
 表記を「マサカドこう」に直したら止んだって都市伝説あるやろ</t>
         </is>
       </c>
-      <c r="C66" s="2" t="inlineStr">
+      <c r="C66" s="4" t="inlineStr">
         <is>
           <t>スレ①</t>
         </is>
@@ -2002,7 +2006,7 @@
           <t>ゲーム会社にまで祟るのやめたれや</t>
         </is>
       </c>
-      <c r="C67" s="2" t="inlineStr">
+      <c r="C67" s="4" t="inlineStr">
         <is>
           <t>スレ①</t>
         </is>
@@ -2021,10 +2025,10 @@
       </c>
       <c r="B68" s="3" t="inlineStr">
         <is>
-          <t>そこは祟りやのうて納期</t>
-        </is>
-      </c>
-      <c r="C68" s="2" t="inlineStr">
+          <t>祟りやのうて納期やろ</t>
+        </is>
+      </c>
+      <c r="C68" s="4" t="inlineStr">
         <is>
           <t>スレ①</t>
         </is>
@@ -2046,7 +2050,7 @@
           <t>不覚にも笑った</t>
         </is>
       </c>
-      <c r="C69" s="2" t="inlineStr">
+      <c r="C69" s="4" t="inlineStr">
         <is>
           <t>スレ①</t>
         </is>
@@ -2065,11 +2069,11 @@
       </c>
       <c r="B70" s="3" t="inlineStr">
         <is>
-          <t>太田光が売れる前に首塚にドロップキックかまして、
-しばらく仕事来んくなったって噂もあるな</t>
-        </is>
-      </c>
-      <c r="C70" s="2" t="inlineStr">
+          <t>売れる前の若手芸人が首塚にドロップキックかまして、
+しばらく仕事が干されたって噂もあるな</t>
+        </is>
+      </c>
+      <c r="C70" s="4" t="inlineStr">
         <is>
           <t>スレ①</t>
         </is>
@@ -2091,7 +2095,7 @@
           <t>それはさすがに芸人の自業自得では</t>
         </is>
       </c>
-      <c r="C71" s="2" t="inlineStr">
+      <c r="C71" s="4" t="inlineStr">
         <is>
           <t>スレ①</t>
         </is>
@@ -2110,8 +2114,7 @@
       </c>
       <c r="B72" s="3" t="inlineStr">
         <is>
-          <t>ついでに言うと、
-将門を祀る神田明神の神田祭は、
+          <t>将門を祀る神田明神の神田祭は、
 今も山王祭と並ぶ江戸三大祭のひとつでな。
 将門は江戸の総鎮守として庶民にめちゃくちゃ愛されてきたんよ。
 怨霊として恐れられた男が、
@@ -2119,7 +2122,7 @@
 畏れと信仰なんて紙一重やなって思うわ</t>
         </is>
       </c>
-      <c r="C72" s="2" t="inlineStr">
+      <c r="C72" s="4" t="inlineStr">
         <is>
           <t>スレ①</t>
         </is>
@@ -2148,7 +2151,7 @@
 二面性のある人物やった</t>
         </is>
       </c>
-      <c r="C73" s="2" t="inlineStr">
+      <c r="C73" s="4" t="inlineStr">
         <is>
           <t>スレ①</t>
         </is>
@@ -2170,7 +2173,7 @@
           <t>ただの怨霊ちゃうくて元はヒーローなんやな</t>
         </is>
       </c>
-      <c r="C74" s="2" t="inlineStr">
+      <c r="C74" s="4" t="inlineStr">
         <is>
           <t>スレ①</t>
         </is>
@@ -2193,7 +2196,7 @@
 考えたら相当パンチ効いとるな</t>
         </is>
       </c>
-      <c r="C75" s="2" t="inlineStr">
+      <c r="C75" s="4" t="inlineStr">
         <is>
           <t>スレ①</t>
         </is>
@@ -2217,7 +2220,7 @@
 因果の証拠なんか何も無い</t>
         </is>
       </c>
-      <c r="C76" s="2" t="inlineStr">
+      <c r="C76" s="4" t="inlineStr">
         <is>
           <t>スレ①</t>
         </is>
@@ -2240,7 +2243,7 @@
 ぜんぶ偶然や</t>
         </is>
       </c>
-      <c r="C77" s="2" t="inlineStr">
+      <c r="C77" s="4" t="inlineStr">
         <is>
           <t>スレ①</t>
         </is>
@@ -2263,7 +2266,7 @@
 そこは認める</t>
         </is>
       </c>
-      <c r="C78" s="2" t="inlineStr">
+      <c r="C78" s="4" t="inlineStr">
         <is>
           <t>スレ①</t>
         </is>
@@ -2286,7 +2289,7 @@
 もう実質勝ちなんよ将門</t>
         </is>
       </c>
-      <c r="C79" s="2" t="inlineStr">
+      <c r="C79" s="4" t="inlineStr">
         <is>
           <t>スレ①</t>
         </is>
@@ -2305,10 +2308,10 @@
       </c>
       <c r="B80" s="3" t="inlineStr">
         <is>
-          <t>勝ち負けの話になってて草</t>
-        </is>
-      </c>
-      <c r="C80" s="2" t="inlineStr">
+          <t>勝ち負けの話になってきとるやんけ</t>
+        </is>
+      </c>
+      <c r="C80" s="4" t="inlineStr">
         <is>
           <t>スレ①</t>
         </is>
@@ -2330,7 +2333,7 @@
           <t>山手線が将門の祟りを抑える結界として作られたって都市伝説もあるよな</t>
         </is>
       </c>
-      <c r="C81" s="2" t="inlineStr">
+      <c r="C81" s="4" t="inlineStr">
         <is>
           <t>スレ①</t>
         </is>
@@ -2353,7 +2356,7 @@
 結界説は後から誰かが言い出したやつや</t>
         </is>
       </c>
-      <c r="C82" s="2" t="inlineStr">
+      <c r="C82" s="4" t="inlineStr">
         <is>
           <t>スレ①</t>
         </is>
@@ -2375,7 +2378,7 @@
           <t>なんや嘘なんか</t>
         </is>
       </c>
-      <c r="C83" s="2" t="inlineStr">
+      <c r="C83" s="4" t="inlineStr">
         <is>
           <t>スレ①</t>
         </is>
@@ -2399,7 +2402,7 @@
 怨霊の部分しか知らんわ</t>
         </is>
       </c>
-      <c r="C84" s="2" t="inlineStr">
+      <c r="C84" s="4" t="inlineStr">
         <is>
           <t>スレ①</t>
         </is>
@@ -2421,7 +2424,7 @@
           <t>新皇名乗って関東独立しようとしたやべえ奴やぞ</t>
         </is>
       </c>
-      <c r="C85" s="2" t="inlineStr">
+      <c r="C85" s="4" t="inlineStr">
         <is>
           <t>スレ①</t>
         </is>
@@ -2444,7 +2447,7 @@
 平将門の首塚にまつわる祟りの噂についてさまざまな議論を見てきたが、</t>
         </is>
       </c>
-      <c r="C86" s="2" t="inlineStr">
+      <c r="C86" s="4" t="inlineStr">
         <is>
           <t>前置き</t>
         </is>
@@ -2469,7 +2472,7 @@
 肝心の生涯に疑問を持つ者も現れた。</t>
         </is>
       </c>
-      <c r="C87" s="2" t="inlineStr">
+      <c r="C87" s="4" t="inlineStr">
         <is>
           <t>前置き</t>
         </is>
@@ -2493,7 +2496,7 @@
 どうやって生まれたのかは気になるところだ。</t>
         </is>
       </c>
-      <c r="C88" s="2" t="inlineStr">
+      <c r="C88" s="4" t="inlineStr">
         <is>
           <t>前置き</t>
         </is>
@@ -2516,7 +2519,7 @@
 2ちゃんねるの歴史オタクたちの議論を見ていこう。</t>
         </is>
       </c>
-      <c r="C89" s="2" t="inlineStr">
+      <c r="C89" s="4" t="inlineStr">
         <is>
           <t>前置き</t>
         </is>
@@ -2539,7 +2542,7 @@
 」</t>
         </is>
       </c>
-      <c r="C90" s="2" t="inlineStr">
+      <c r="C90" s="4" t="inlineStr">
         <is>
           <t>スレ②</t>
         </is>
@@ -2561,7 +2564,7 @@
           <t>出た自称新皇ｗ</t>
         </is>
       </c>
-      <c r="C91" s="2" t="inlineStr">
+      <c r="C91" s="4" t="inlineStr">
         <is>
           <t>スレ②</t>
         </is>
@@ -2583,7 +2586,7 @@
           <t>名乗ったもん勝ちかよ</t>
         </is>
       </c>
-      <c r="C92" s="2" t="inlineStr">
+      <c r="C92" s="4" t="inlineStr">
         <is>
           <t>スレ②</t>
         </is>
@@ -2605,7 +2608,7 @@
           <t>関東の田舎で勝手に天皇名乗ったやべえ人やろ</t>
         </is>
       </c>
-      <c r="C93" s="2" t="inlineStr">
+      <c r="C93" s="4" t="inlineStr">
         <is>
           <t>スレ②</t>
         </is>
@@ -2624,11 +2627,11 @@
       </c>
       <c r="B94" s="3" t="inlineStr">
         <is>
-          <t>その新皇とやらも2か月で終わった負け犬やん、
+          <t>新皇とやら名乗っても2か月で終わった負け犬やん、
 持ち上げる要素ある？</t>
         </is>
       </c>
-      <c r="C94" s="2" t="inlineStr">
+      <c r="C94" s="4" t="inlineStr">
         <is>
           <t>スレ②</t>
         </is>
@@ -2650,7 +2653,7 @@
           <t>怨霊の話は聞くけど何した人かは正直知らんわ</t>
         </is>
       </c>
-      <c r="C95" s="2" t="inlineStr">
+      <c r="C95" s="4" t="inlineStr">
         <is>
           <t>スレ②</t>
         </is>
@@ -2673,7 +2676,7 @@
 こいつ何がしたかったん</t>
         </is>
       </c>
-      <c r="C96" s="2" t="inlineStr">
+      <c r="C96" s="4" t="inlineStr">
         <is>
           <t>スレ②</t>
         </is>
@@ -2696,7 +2699,7 @@
 それ以上でもそれ以下でもなくない？</t>
         </is>
       </c>
-      <c r="C97" s="2" t="inlineStr">
+      <c r="C97" s="4" t="inlineStr">
         <is>
           <t>スレ②</t>
         </is>
@@ -2715,7 +2718,7 @@
       </c>
       <c r="B98" s="3" t="inlineStr">
         <is>
-          <t>それが最初っから天皇に盾突こうとしてたわけちゃうんよ。
+          <t>こいつ最初っから天皇に盾突こうとしてたわけちゃうんよ。
 スタートはただの一族内のもめ事や。
 関東の平氏一門で、
 伯父さんらと土地や縁談がらみの私闘をやっとった、
@@ -2724,7 +2727,7 @@
 どんどん引くに引けん大ごとになってってもうた</t>
         </is>
       </c>
-      <c r="C98" s="2" t="inlineStr">
+      <c r="C98" s="4" t="inlineStr">
         <is>
           <t>スレ②</t>
         </is>
@@ -2746,7 +2749,7 @@
           <t>ファッ最初は身内ゲンカなんか</t>
         </is>
       </c>
-      <c r="C99" s="2" t="inlineStr">
+      <c r="C99" s="4" t="inlineStr">
         <is>
           <t>スレ②</t>
         </is>
@@ -2765,10 +2768,10 @@
       </c>
       <c r="B100" s="3" t="inlineStr">
         <is>
-          <t>そっからどうやったら天皇まで行くん</t>
-        </is>
-      </c>
-      <c r="C100" s="2" t="inlineStr">
+          <t>ほんでどうやって天皇まで行くん</t>
+        </is>
+      </c>
+      <c r="C100" s="4" t="inlineStr">
         <is>
           <t>スレ②</t>
         </is>
@@ -2791,7 +2794,7 @@
 流れがエグいな</t>
         </is>
       </c>
-      <c r="C101" s="2" t="inlineStr">
+      <c r="C101" s="4" t="inlineStr">
         <is>
           <t>スレ②</t>
         </is>
@@ -2819,7 +2822,7 @@
 そのまま中央に弓を引くことになった</t>
         </is>
       </c>
-      <c r="C102" s="2" t="inlineStr">
+      <c r="C102" s="4" t="inlineStr">
         <is>
           <t>スレ②</t>
         </is>
@@ -2841,7 +2844,7 @@
           <t>中央仕込みの男が地元で反乱とか飛躍すぎやろ</t>
         </is>
       </c>
-      <c r="C103" s="2" t="inlineStr">
+      <c r="C103" s="4" t="inlineStr">
         <is>
           <t>スレ②</t>
         </is>
@@ -2863,7 +2866,7 @@
           <t>中身を知ってる奴が反旗ひるがえすのが一番こわい</t>
         </is>
       </c>
-      <c r="C104" s="2" t="inlineStr">
+      <c r="C104" s="4" t="inlineStr">
         <is>
           <t>スレ②</t>
         </is>
@@ -2893,7 +2896,7 @@
 一介の豪族が関東一円を呑み込むなんて芸当ができた</t>
         </is>
       </c>
-      <c r="C105" s="2" t="inlineStr">
+      <c r="C105" s="4" t="inlineStr">
         <is>
           <t>スレ②</t>
         </is>
@@ -2916,7 +2919,7 @@
 そら強いわな</t>
         </is>
       </c>
-      <c r="C106" s="2" t="inlineStr">
+      <c r="C106" s="4" t="inlineStr">
         <is>
           <t>スレ②</t>
         </is>
@@ -2935,7 +2938,7 @@
       </c>
       <c r="B107" s="3" t="inlineStr">
         <is>
-          <t>その私闘で官側の人間ともやり合ううちに、
+          <t>馬で勢いづいた将門が私闘で官側の人間ともやり合ううちに、
 今度は朝廷の出先の国府とぶつかってまう。
 勢いで常陸の国府を攻め落として、
 国の実印にあたる印鑰まで奪ってもうた。
@@ -2944,7 +2947,7 @@
 もう後戻りでけへんとこまで行ってもうた</t>
         </is>
       </c>
-      <c r="C107" s="2" t="inlineStr">
+      <c r="C107" s="4" t="inlineStr">
         <is>
           <t>スレ②</t>
         </is>
@@ -2966,7 +2969,7 @@
           <t>印鑰ってなんや</t>
         </is>
       </c>
-      <c r="C108" s="2" t="inlineStr">
+      <c r="C108" s="4" t="inlineStr">
         <is>
           <t>スレ②</t>
         </is>
@@ -2989,7 +2992,7 @@
 それ奪うって今でいう役所まるごと乗っ取るレベルやぞ</t>
         </is>
       </c>
-      <c r="C109" s="2" t="inlineStr">
+      <c r="C109" s="4" t="inlineStr">
         <is>
           <t>スレ②</t>
         </is>
@@ -3013,7 +3016,7 @@
 国の実印と倉の鍵を指す言葉である。</t>
         </is>
       </c>
-      <c r="C110" s="2" t="inlineStr">
+      <c r="C110" s="4" t="inlineStr">
         <is>
           <t>解説：印鑰</t>
         </is>
@@ -3036,7 +3039,7 @@
 鑰は税として集めた米などを納めた正倉の鍵を意味する。</t>
         </is>
       </c>
-      <c r="C111" s="2" t="inlineStr">
+      <c r="C111" s="4" t="inlineStr">
         <is>
           <t>解説：印鑰</t>
         </is>
@@ -3059,7 +3062,7 @@
 その国の行政と財産をまとめて手中に収めることに等しかった。</t>
         </is>
       </c>
-      <c r="C112" s="2" t="inlineStr">
+      <c r="C112" s="4" t="inlineStr">
         <is>
           <t>解説：印鑰</t>
         </is>
@@ -3082,7 +3085,7 @@
 朝廷の支配そのものに正面から弓を引いたことを意味するのである。</t>
         </is>
       </c>
-      <c r="C113" s="2" t="inlineStr">
+      <c r="C113" s="4" t="inlineStr">
         <is>
           <t>解説：印鑰</t>
         </is>
@@ -3101,7 +3104,7 @@
       </c>
       <c r="B114" s="3" t="inlineStr">
         <is>
-          <t>そっから勢いに乗った将門は、
+          <t>勢いに乗った将門は、
 坂東、
 今でいう関東一帯の国府を次々落として、
 ほぼ関東全域を手中に収めてまう。
@@ -3111,7 +3114,7 @@
 当時前代未聞やってん</t>
         </is>
       </c>
-      <c r="C114" s="2" t="inlineStr">
+      <c r="C114" s="4" t="inlineStr">
         <is>
           <t>スレ②</t>
         </is>
@@ -3133,7 +3136,7 @@
           <t>関東まるごとはやりすぎ</t>
         </is>
       </c>
-      <c r="C115" s="2" t="inlineStr">
+      <c r="C115" s="4" t="inlineStr">
         <is>
           <t>スレ②</t>
         </is>
@@ -3155,7 +3158,7 @@
           <t>もはや完全に独立国家</t>
         </is>
       </c>
-      <c r="C116" s="2" t="inlineStr">
+      <c r="C116" s="4" t="inlineStr">
         <is>
           <t>スレ②</t>
         </is>
@@ -3174,10 +3177,10 @@
       </c>
       <c r="B117" s="3" t="inlineStr">
         <is>
-          <t>そんで調子乗って新皇宣言と</t>
-        </is>
-      </c>
-      <c r="C117" s="2" t="inlineStr">
+          <t>調子乗って新皇宣言かよ</t>
+        </is>
+      </c>
+      <c r="C117" s="4" t="inlineStr">
         <is>
           <t>スレ②</t>
         </is>
@@ -3196,17 +3199,16 @@
       </c>
       <c r="B118" s="3" t="inlineStr">
         <is>
-          <t>そう、
-ここで「新皇」、
-つまり新しい天皇を名乗る。
+          <t>名乗ったのが「新皇」、
+つまり新しい天皇や。
 伝説やと八幡神のお告げで位を授かったってことになっとるけど、
-ようは京都の天皇とは別に、
+京都の天皇とは別に、
 東国に自分を頂点とした朝廷を立てようとしたんや。
 関東に独立政権を作るっていう、
 日本史でもなかなかおらんスケールの反逆やった</t>
         </is>
       </c>
-      <c r="C118" s="2" t="inlineStr">
+      <c r="C118" s="4" t="inlineStr">
         <is>
           <t>スレ②</t>
         </is>
@@ -3229,7 +3231,7 @@
 自分で言うてるだけやろ知らんけど</t>
         </is>
       </c>
-      <c r="C119" s="2" t="inlineStr">
+      <c r="C119" s="4" t="inlineStr">
         <is>
           <t>スレ②</t>
         </is>
@@ -3251,7 +3253,7 @@
           <t>神様持ち出すの強気すぎる</t>
         </is>
       </c>
-      <c r="C120" s="2" t="inlineStr">
+      <c r="C120" s="4" t="inlineStr">
         <is>
           <t>スレ②</t>
         </is>
@@ -3274,7 +3276,7 @@
 神託とか後付けくさいわ</t>
         </is>
       </c>
-      <c r="C121" s="2" t="inlineStr">
+      <c r="C121" s="4" t="inlineStr">
         <is>
           <t>スレ②</t>
         </is>
@@ -3298,7 +3300,7 @@
 しょせんただの勘違いした田舎の暴れん坊</t>
         </is>
       </c>
-      <c r="C122" s="2" t="inlineStr">
+      <c r="C122" s="4" t="inlineStr">
         <is>
           <t>スレ②</t>
         </is>
@@ -3321,7 +3323,7 @@
 そこは認めたれや</t>
         </is>
       </c>
-      <c r="C123" s="2" t="inlineStr">
+      <c r="C123" s="4" t="inlineStr">
         <is>
           <t>スレ②</t>
         </is>
@@ -3343,7 +3345,7 @@
           <t>でもこんなん中央がブチギレて一発で終わり</t>
         </is>
       </c>
-      <c r="C124" s="2" t="inlineStr">
+      <c r="C124" s="4" t="inlineStr">
         <is>
           <t>スレ②</t>
         </is>
@@ -3362,15 +3364,14 @@
       </c>
       <c r="B125" s="3" t="inlineStr">
         <is>
-          <t>そうなる。
-京都は将門を朝敵認定して追討令を出す。
+          <t>京都は将門を朝敵認定して追討令を出す。
 ここで動いたのが同じ関東の平貞盛と、
 下野の豪族やった藤原秀郷や。
 身内や近隣やった連中が討伐側に回って、
 将門包囲網が出来てまう</t>
         </is>
       </c>
-      <c r="C125" s="2" t="inlineStr">
+      <c r="C125" s="4" t="inlineStr">
         <is>
           <t>スレ②</t>
         </is>
@@ -3389,10 +3390,10 @@
       </c>
       <c r="B126" s="3" t="inlineStr">
         <is>
-          <t>結局身内に討たれるんかい</t>
-        </is>
-      </c>
-      <c r="C126" s="2" t="inlineStr">
+          <t>身内に討たれるんかい</t>
+        </is>
+      </c>
+      <c r="C126" s="4" t="inlineStr">
         <is>
           <t>スレ②</t>
         </is>
@@ -3414,7 +3415,7 @@
           <t>関東の独立より自分の家のほうが大事って奴がおったわけやな</t>
         </is>
       </c>
-      <c r="C127" s="2" t="inlineStr">
+      <c r="C127" s="4" t="inlineStr">
         <is>
           <t>スレ②</t>
         </is>
@@ -3436,7 +3437,7 @@
           <t>将門を討ったのって源氏の先祖やっけ？</t>
         </is>
       </c>
-      <c r="C128" s="2" t="inlineStr">
+      <c r="C128" s="4" t="inlineStr">
         <is>
           <t>スレ②</t>
         </is>
@@ -3461,7 +3462,7 @@
 そこ混同したらあかんで</t>
         </is>
       </c>
-      <c r="C129" s="2" t="inlineStr">
+      <c r="C129" s="4" t="inlineStr">
         <is>
           <t>スレ②</t>
         </is>
@@ -3484,7 +3485,7 @@
 すまんね</t>
         </is>
       </c>
-      <c r="C130" s="2" t="inlineStr">
+      <c r="C130" s="4" t="inlineStr">
         <is>
           <t>スレ②</t>
         </is>
@@ -3503,10 +3504,9 @@
       </c>
       <c r="B131" s="3" t="inlineStr">
         <is>
-          <t>そして天慶3年、
-西暦940年、
-ついに討伐軍とぶつかって、
-将門は敗れる。
+          <t>940年、
+天慶3年やな。
+ついに討伐軍とぶつかって将門は敗れてまうんやけど、
 伝承やと、
 戦いの最中に飛んできた流れ矢が額に当たって、
 それが致命傷になって命を落としたって言われとる。
@@ -3515,7 +3515,7 @@
 終わりはほんま一瞬やった</t>
         </is>
       </c>
-      <c r="C131" s="2" t="inlineStr">
+      <c r="C131" s="4" t="inlineStr">
         <is>
           <t>スレ②</t>
         </is>
@@ -3537,7 +3537,7 @@
           <t>2か月て短すぎ</t>
         </is>
       </c>
-      <c r="C132" s="2" t="inlineStr">
+      <c r="C132" s="4" t="inlineStr">
         <is>
           <t>スレ②</t>
         </is>
@@ -3560,7 +3560,7 @@
 名乗っただけで終わっとるｗ</t>
         </is>
       </c>
-      <c r="C133" s="2" t="inlineStr">
+      <c r="C133" s="4" t="inlineStr">
         <is>
           <t>スレ②</t>
         </is>
@@ -3579,16 +3579,15 @@
       </c>
       <c r="B134" s="3" t="inlineStr">
         <is>
-          <t>その最期にも伝説があってな。
-将門は矢も通さんと評判の無敵の体で討伐軍が苦戦しとったけど、
+          <t>最期にも伝説があってな。
+矢も通さん無敵の体やって討伐軍が苦戦しとったけど、
 戦いの最中に陣の風向きが急に変わって、
 その隙に放たれた矢が額に当たったって話が残っとる。
 神がかった強さやのに、
-最後は風っていう運否天賦みたいなもんで決着した、
-っていうのがまた伝説をさらに盛り上げる</t>
-        </is>
-      </c>
-      <c r="C134" s="2" t="inlineStr">
+最後は風っていう運否天賦みたいなもんで決着したのがまた出来すぎなんよな</t>
+        </is>
+      </c>
+      <c r="C134" s="4" t="inlineStr">
         <is>
           <t>スレ②</t>
         </is>
@@ -3610,7 +3609,7 @@
           <t>急に弱点出てくるの少年漫画かよ</t>
         </is>
       </c>
-      <c r="C135" s="2" t="inlineStr">
+      <c r="C135" s="4" t="inlineStr">
         <is>
           <t>スレ②</t>
         </is>
@@ -3632,7 +3631,7 @@
           <t>風で負けるラスボスすこｗ</t>
         </is>
       </c>
-      <c r="C136" s="2" t="inlineStr">
+      <c r="C136" s="4" t="inlineStr">
         <is>
           <t>スレ②</t>
         </is>
@@ -3651,7 +3650,7 @@
       </c>
       <c r="B137" s="3" t="inlineStr">
         <is>
-          <t>もういっこ有名なんが影武者伝説や。
+          <t>影武者伝説ってのも有名でな。
 将門にはそっくりの影武者が何人もおって、
 本物を見分けられんかったけど、
 こめかみのあたりに本物だけ影が無かった、
@@ -3660,7 +3659,7 @@
 こういう伝説を生んだんやろな</t>
         </is>
       </c>
-      <c r="C137" s="2" t="inlineStr">
+      <c r="C137" s="4" t="inlineStr">
         <is>
           <t>スレ②</t>
         </is>
@@ -3682,7 +3681,7 @@
           <t>影武者まで盛られるの大物の証や</t>
         </is>
       </c>
-      <c r="C138" s="2" t="inlineStr">
+      <c r="C138" s="4" t="inlineStr">
         <is>
           <t>スレ②</t>
         </is>
@@ -3701,13 +3700,13 @@
       </c>
       <c r="B139" s="3" t="inlineStr">
         <is>
-          <t>そういや将門を祀っとる国王神社が茨城にあって、
+          <t>将門を祀っとる国王神社が茨城にあって、
 将門の三女が建てたって伝わっとるな。
 ワイ一回行ったけど、
 めっちゃ静かでええとこやった</t>
         </is>
       </c>
-      <c r="C139" s="2" t="inlineStr">
+      <c r="C139" s="4" t="inlineStr">
         <is>
           <t>スレ②</t>
         </is>
@@ -3730,7 +3729,7 @@
 昔の風と雲と虹と以来やろ</t>
         </is>
       </c>
-      <c r="C140" s="2" t="inlineStr">
+      <c r="C140" s="4" t="inlineStr">
         <is>
           <t>スレ②</t>
         </is>
@@ -3752,7 +3751,7 @@
           <t>主役が朝敵やと今のNHKはやりにくいやろなあ</t>
         </is>
       </c>
-      <c r="C141" s="2" t="inlineStr">
+      <c r="C141" s="4" t="inlineStr">
         <is>
           <t>スレ②</t>
         </is>
@@ -3774,7 +3773,7 @@
           <t>あの首が飛ぶ伝説に繋がるわけやな</t>
         </is>
       </c>
-      <c r="C142" s="2" t="inlineStr">
+      <c r="C142" s="4" t="inlineStr">
         <is>
           <t>スレ②</t>
         </is>
@@ -3793,13 +3792,12 @@
       </c>
       <c r="B143" s="3" t="inlineStr">
         <is>
-          <t>そう、
-討たれた首は京都に送られて晒される。
+          <t>討たれた首は京都に送られて晒される。
 その首が夜に飛んで関東に戻った、
 っていうのが前半の祟りの話に繋がる</t>
         </is>
       </c>
-      <c r="C143" s="2" t="inlineStr">
+      <c r="C143" s="4" t="inlineStr">
         <is>
           <t>スレ②</t>
         </is>
@@ -3818,10 +3816,10 @@
       </c>
       <c r="B144" s="3" t="inlineStr">
         <is>
-          <t>きれいに一周してて草</t>
-        </is>
-      </c>
-      <c r="C144" s="2" t="inlineStr">
+          <t>きれいに一周しとるやんけ</t>
+        </is>
+      </c>
+      <c r="C144" s="4" t="inlineStr">
         <is>
           <t>スレ②</t>
         </is>
@@ -3849,7 +3847,7 @@
 今でも神田明神の氏子は成田山には参らんって言われとるくらいでな</t>
         </is>
       </c>
-      <c r="C145" s="2" t="inlineStr">
+      <c r="C145" s="4" t="inlineStr">
         <is>
           <t>スレ②</t>
         </is>
@@ -3873,7 +3871,7 @@
 評価する要素ある？</t>
         </is>
       </c>
-      <c r="C146" s="2" t="inlineStr">
+      <c r="C146" s="4" t="inlineStr">
         <is>
           <t>スレ②</t>
         </is>
@@ -3893,7 +3891,7 @@
       <c r="B147" s="3" t="inlineStr">
         <is>
           <t>いや、
-そうとも言い切れん。
+そうとも言い切れんで。
 中央の貴族が地方を搾取する仕組みに、
 地方の武装勢力が真っ向から「ノー」を突きつけた最初級の例なんや。
 後の武士が自分らの力で土地を治める時代の、
@@ -3902,7 +3900,7 @@
 関東武士の精神的な元祖として評価する見方も根強い</t>
         </is>
       </c>
-      <c r="C147" s="2" t="inlineStr">
+      <c r="C147" s="4" t="inlineStr">
         <is>
           <t>スレ②</t>
         </is>
@@ -3925,7 +3923,7 @@
 盛りすぎて引くわ</t>
         </is>
       </c>
-      <c r="C148" s="2" t="inlineStr">
+      <c r="C148" s="4" t="inlineStr">
         <is>
           <t>スレ②</t>
         </is>
@@ -3948,7 +3946,7 @@
 現に怨霊で千年語り継がれとるんやから</t>
         </is>
       </c>
-      <c r="C149" s="2" t="inlineStr">
+      <c r="C149" s="4" t="inlineStr">
         <is>
           <t>スレ②</t>
         </is>
@@ -3971,7 +3969,7 @@
 東西で同時に乱が起きとったんよな</t>
         </is>
       </c>
-      <c r="C150" s="2" t="inlineStr">
+      <c r="C150" s="4" t="inlineStr">
         <is>
           <t>スレ②</t>
         </is>
@@ -3990,12 +3988,11 @@
       </c>
       <c r="B151" s="3" t="inlineStr">
         <is>
-          <t>それや、
-承平天慶の乱でセット扱いされるやつ。
+          <t>まさに承平天慶の乱でセット扱いされるやつな。
 朝廷からしたら東西挟み撃ちで生きた心地せんかったやろな</t>
         </is>
       </c>
-      <c r="C151" s="2" t="inlineStr">
+      <c r="C151" s="4" t="inlineStr">
         <is>
           <t>スレ②</t>
         </is>
@@ -4018,7 +4015,7 @@
 平安時代中期に東西で同時に起きた二つの大きな反乱の総称である。</t>
         </is>
       </c>
-      <c r="C152" s="2" t="inlineStr">
+      <c r="C152" s="4" t="inlineStr">
         <is>
           <t>解説：承平天慶の乱</t>
         </is>
@@ -4041,7 +4038,7 @@
 西国では瀬戸内で藤原純友が海賊を率いて朝廷に反旗をひるがえした。</t>
         </is>
       </c>
-      <c r="C153" s="2" t="inlineStr">
+      <c r="C153" s="4" t="inlineStr">
         <is>
           <t>解説：承平天慶の乱</t>
         </is>
@@ -4063,7 +4060,7 @@
           <t>朝廷にとっては東西から同時に挑戦を突きつけられた前代未聞の事態であり、</t>
         </is>
       </c>
-      <c r="C154" s="2" t="inlineStr">
+      <c r="C154" s="4" t="inlineStr">
         <is>
           <t>解説：承平天慶の乱</t>
         </is>
@@ -4085,7 +4082,7 @@
           <t>地方の武士の力を中央が無視できなくなっていく大きな転機となった出来事である。</t>
         </is>
       </c>
-      <c r="C155" s="2" t="inlineStr">
+      <c r="C155" s="4" t="inlineStr">
         <is>
           <t>解説：承平天慶の乱</t>
         </is>
@@ -4107,7 +4104,7 @@
           <t>もし将門が勝っとったら関東に別の国できてたんかな</t>
         </is>
       </c>
-      <c r="C156" s="2" t="inlineStr">
+      <c r="C156" s="4" t="inlineStr">
         <is>
           <t>スレ②</t>
         </is>
@@ -4126,7 +4123,7 @@
       </c>
       <c r="B157" s="3" t="inlineStr">
         <is>
-          <t>そこはロマンあるよな。
+          <t>ロマンあるよな。
 もし討伐をしのいで東国政権が定着しとったら、
 関東拠点の独立勢力が早い段階で出来て、
 武士の世が何百年か前倒しになってたかもしれん。
@@ -4135,7 +4132,7 @@
 たらればとしては最高に面白い人物やわ</t>
         </is>
       </c>
-      <c r="C157" s="2" t="inlineStr">
+      <c r="C157" s="4" t="inlineStr">
         <is>
           <t>スレ②</t>
         </is>
@@ -4157,7 +4154,7 @@
           <t>関東人としてはちょっと応援したくなる</t>
         </is>
       </c>
-      <c r="C158" s="2" t="inlineStr">
+      <c r="C158" s="4" t="inlineStr">
         <is>
           <t>スレ②</t>
         </is>
@@ -4180,7 +4177,7 @@
 地味に将門ゆかりの地に住んどる</t>
         </is>
       </c>
-      <c r="C159" s="2" t="inlineStr">
+      <c r="C159" s="4" t="inlineStr">
         <is>
           <t>スレ②</t>
         </is>
@@ -4199,11 +4196,11 @@
       </c>
       <c r="B160" s="3" t="inlineStr">
         <is>
-          <t>つまり、
-その首が今も大手町でブチギレてるわけやな</t>
-        </is>
-      </c>
-      <c r="C160" s="2" t="inlineStr">
+          <t>ほな、
+その首が今も大手町でキレてるわけやな</t>
+        </is>
+      </c>
+      <c r="C160" s="4" t="inlineStr">
         <is>
           <t>スレ②</t>
         </is>
@@ -4226,7 +4223,7 @@
 ある意味いまだに関東の主やってるとも言えるわ</t>
         </is>
       </c>
-      <c r="C161" s="2" t="inlineStr">
+      <c r="C161" s="4" t="inlineStr">
         <is>
           <t>スレ②</t>
         </is>
@@ -4248,7 +4245,7 @@
           <t>うまいこと言うな</t>
         </is>
       </c>
-      <c r="C162" s="2" t="inlineStr">
+      <c r="C162" s="4" t="inlineStr">
         <is>
           <t>スレ②</t>
         </is>
@@ -4272,7 +4269,7 @@
 将門さん祟らんといてな</t>
         </is>
       </c>
-      <c r="C163" s="2" t="inlineStr">
+      <c r="C163" s="4" t="inlineStr">
         <is>
           <t>スレ②</t>
         </is>
@@ -4294,7 +4291,7 @@
           <t>本日はここまで。</t>
         </is>
       </c>
-      <c r="C164" s="2" t="inlineStr">
+      <c r="C164" s="4" t="inlineStr">
         <is>
           <t>締め</t>
         </is>
@@ -4318,7 +4315,7 @@
 いかがだっただろうか？</t>
         </is>
       </c>
-      <c r="C165" s="2" t="inlineStr">
+      <c r="C165" s="4" t="inlineStr">
         <is>
           <t>締め</t>
         </is>
@@ -4340,7 +4337,7 @@
           <t>2ちゃんねるの歴史オタクたちの議論を見ていると、</t>
         </is>
       </c>
-      <c r="C166" s="2" t="inlineStr">
+      <c r="C166" s="4" t="inlineStr">
         <is>
           <t>締め</t>
         </is>
@@ -4364,7 +4361,7 @@
 だからこそ千年経った今も畏れと敬いを同時に集め続けているのだと思えた。</t>
         </is>
       </c>
-      <c r="C167" s="2" t="inlineStr">
+      <c r="C167" s="4" t="inlineStr">
         <is>
           <t>締め</t>
         </is>
@@ -4386,7 +4383,7 @@
           <t>今回の動画について他の意見や感想があったらぜひコメントで教えてね！</t>
         </is>
       </c>
-      <c r="C168" s="2" t="inlineStr">
+      <c r="C168" s="4" t="inlineStr">
         <is>
           <t>締め</t>
         </is>
@@ -4410,7 +4407,7 @@
 ご視聴ありがとうございました！</t>
         </is>
       </c>
-      <c r="C169" s="2" t="inlineStr">
+      <c r="C169" s="4" t="inlineStr">
         <is>
           <t>締め</t>
         </is>

</xml_diff>

<commit_message>
auto: 2026-06-19 22:08 (6件)
</commit_message>
<xml_diff>
--- a/01_プロジェクト/YouTube/創作スレ下書き/2026-06-17_平将門の祟り_台本.xlsx
+++ b/01_プロジェクト/YouTube/創作スレ下書き/2026-06-17_平将門の祟り_台本.xlsx
@@ -727,7 +727,7 @@
       <c r="B13" s="3" t="inlineStr">
         <is>
           <t>ただのオカルトを真に受けすぎや、
-ぜんぶ偶然やろ</t>
+ぜんぶ偶然やって</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
@@ -868,7 +868,7 @@
       <c r="B19" s="3" t="inlineStr">
         <is>
           <t>早速整爾って総理大臣やっけ？
-それで騒ぎになったんやろ</t>
+それで騒ぎになったんちゃうの</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
@@ -1153,7 +1153,7 @@
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>国家権力に二連勝してる時点で将門つよすぎやろ</t>
+          <t>国家権力に二連勝してる時点で将門つよすぎ</t>
         </is>
       </c>
       <c r="C31" s="4" t="inlineStr">
@@ -1695,7 +1695,7 @@
       </c>
       <c r="B54" s="3" t="inlineStr">
         <is>
-          <t>通帳に平将門て書いてあるん想像してもうたわ</t>
+          <t>通帳に平将門て書いてあるん想像してみ</t>
         </is>
       </c>
       <c r="C54" s="4" t="inlineStr">
@@ -1790,7 +1790,7 @@
       <c r="B58" s="3" t="inlineStr">
         <is>
           <t>ワイ去年あの辺で働いとったとき、
-毎朝コンビニ寄る感覚で手だけ合わせて通勤しとったわ</t>
+毎朝コンビニ寄る感覚で手だけ合わせて通勤しとったもん</t>
         </is>
       </c>
       <c r="C58" s="4" t="inlineStr">
@@ -1981,7 +1981,7 @@
         <is>
           <t>メガテン勢からすると将門公はガチで畏れる対象や。
 アトラスが将門モチーフにしたら開発中トラブル続きで、
-表記を「マサカドこう」に直したら止んだって都市伝説あるやろ</t>
+表記を「マサカドこう」に直したら止んだって都市伝説まであるしな</t>
         </is>
       </c>
       <c r="C66" s="4" t="inlineStr">
@@ -2119,7 +2119,7 @@
 将門は江戸の総鎮守として庶民にめちゃくちゃ愛されてきたんよ。
 怨霊として恐れられた男が、
 江戸っ子の誇りの祭の主役になっとるんやから、
-畏れと信仰なんて紙一重やなって思うわ</t>
+畏れと信仰なんて紙一重やなと思わされる</t>
         </is>
       </c>
       <c r="C72" s="4" t="inlineStr">
@@ -3273,7 +3273,7 @@
       <c r="B121" s="3" t="inlineStr">
         <is>
           <t>正直そこは盛りやろ、
-神託とか後付けくさいわ</t>
+神託とか後付けくさい</t>
         </is>
       </c>
       <c r="C121" s="4" t="inlineStr">
@@ -4129,7 +4129,7 @@
 武士の世が何百年か前倒しになってたかもしれん。
 まあ補給も人望もまだ足りんかったから現実は厳しかったやろけど。
 知らんけど、
-たらればとしては最高に面白い人物やわ</t>
+たらればとしては最高におもろい人物</t>
         </is>
       </c>
       <c r="C157" s="4" t="inlineStr">

</xml_diff>

<commit_message>
auto: 2026-06-20 09:08 (3件)
</commit_message>
<xml_diff>
--- a/01_プロジェクト/YouTube/創作スレ下書き/2026-06-17_平将門の祟り_台本.xlsx
+++ b/01_プロジェクト/YouTube/創作スレ下書き/2026-06-17_平将門の祟り_台本.xlsx
@@ -648,14 +648,14 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>2&gt;&gt;1</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>男性C</t>
+          <t>男性C下</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
@@ -670,14 +670,14 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>3&gt;&gt;1</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>女性D</t>
+          <t>女性D下</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -692,14 +692,14 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>4&gt;&gt;1</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>男性E</t>
+          <t>男性E下</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
@@ -714,7 +714,7 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>5&gt;&gt;1</t>
         </is>
       </c>
     </row>
@@ -875,7 +875,7 @@
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>12&gt;&gt;11</t>
         </is>
       </c>
     </row>
@@ -923,14 +923,14 @@
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>14&gt;&gt;13</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>男性E</t>
+          <t>男性E下</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
@@ -946,7 +946,7 @@
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>15&gt;&gt;14</t>
         </is>
       </c>
     </row>
@@ -1086,7 +1086,7 @@
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>17&gt;&gt;16</t>
         </is>
       </c>
     </row>
@@ -1185,7 +1185,7 @@
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>21&gt;&gt;20</t>
         </is>
       </c>
     </row>
@@ -1253,7 +1253,7 @@
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>24&gt;&gt;23</t>
         </is>
       </c>
     </row>
@@ -1323,14 +1323,14 @@
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>27&gt;&gt;26</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>男性C</t>
+          <t>男性C下</t>
         </is>
       </c>
       <c r="B39" s="3" t="inlineStr">
@@ -1345,7 +1345,7 @@
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>28&gt;&gt;27</t>
         </is>
       </c>
     </row>
@@ -1556,14 +1556,14 @@
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>33&gt;&gt;32</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>女性D</t>
+          <t>女性D下</t>
         </is>
       </c>
       <c r="B49" s="3" t="inlineStr">
@@ -1578,7 +1578,7 @@
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>34&gt;&gt;33</t>
         </is>
       </c>
     </row>
@@ -1624,7 +1624,7 @@
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>36</t>
+          <t>36&gt;&gt;35</t>
         </is>
       </c>
     </row>
@@ -1656,7 +1656,7 @@
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>男性C</t>
+          <t>男性C下</t>
         </is>
       </c>
       <c r="B53" s="3" t="inlineStr">
@@ -1671,14 +1671,14 @@
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>38</t>
+          <t>38&gt;&gt;37</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>女性D</t>
+          <t>女性D下</t>
         </is>
       </c>
       <c r="B54" s="3" t="inlineStr">
@@ -1693,14 +1693,14 @@
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>39</t>
+          <t>39&gt;&gt;37</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>男性E下</t>
+          <t>男性E</t>
         </is>
       </c>
       <c r="B55" s="3" t="inlineStr">
@@ -1722,7 +1722,7 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>男性A</t>
+          <t>男性A下</t>
         </is>
       </c>
       <c r="B56" s="3" t="inlineStr">
@@ -1739,7 +1739,7 @@
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>41&gt;&gt;40</t>
         </is>
       </c>
     </row>
@@ -1785,7 +1785,7 @@
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>43</t>
+          <t>43&gt;&gt;42</t>
         </is>
       </c>
     </row>
@@ -1921,7 +1921,7 @@
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>49</t>
+          <t>49&gt;&gt;48</t>
         </is>
       </c>
     </row>
@@ -2040,7 +2040,7 @@
       </c>
       <c r="D69" s="2" t="inlineStr">
         <is>
-          <t>54</t>
+          <t>54&gt;&gt;53</t>
         </is>
       </c>
     </row>
@@ -2066,7 +2066,7 @@
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>55</t>
+          <t>55&gt;&gt;53</t>
         </is>
       </c>
     </row>
@@ -2096,7 +2096,7 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>女性B下</t>
+          <t>女性B</t>
         </is>
       </c>
       <c r="B72" s="3" t="inlineStr">
@@ -2120,7 +2120,7 @@
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
         <is>
-          <t>男性C</t>
+          <t>男性C下</t>
         </is>
       </c>
       <c r="B73" s="3" t="inlineStr">
@@ -2135,14 +2135,14 @@
       </c>
       <c r="D73" s="2" t="inlineStr">
         <is>
-          <t>58</t>
+          <t>58&gt;&gt;57</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>女性D</t>
+          <t>女性D下</t>
         </is>
       </c>
       <c r="B74" s="3" t="inlineStr">
@@ -2157,7 +2157,7 @@
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>59</t>
+          <t>59&gt;&gt;57</t>
         </is>
       </c>
     </row>
@@ -2179,7 +2179,7 @@
       </c>
       <c r="D75" s="2" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>60&gt;&gt;59</t>
         </is>
       </c>
     </row>
@@ -2209,7 +2209,7 @@
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
         <is>
-          <t>女性B</t>
+          <t>女性B下</t>
         </is>
       </c>
       <c r="B77" s="3" t="inlineStr">
@@ -2224,7 +2224,7 @@
       </c>
       <c r="D77" s="2" t="inlineStr">
         <is>
-          <t>62</t>
+          <t>62&gt;&gt;61</t>
         </is>
       </c>
     </row>
@@ -2305,7 +2305,7 @@
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
         <is>
-          <t>男性A</t>
+          <t>男性A下</t>
         </is>
       </c>
       <c r="B81" s="3" t="inlineStr">
@@ -2321,7 +2321,7 @@
       </c>
       <c r="D81" s="2" t="inlineStr">
         <is>
-          <t>66</t>
+          <t>66&gt;&gt;63</t>
         </is>
       </c>
     </row>
@@ -2352,7 +2352,7 @@
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
         <is>
-          <t>男性C</t>
+          <t>男性C下</t>
         </is>
       </c>
       <c r="B83" s="3" t="inlineStr">
@@ -2368,7 +2368,7 @@
       </c>
       <c r="D83" s="2" t="inlineStr">
         <is>
-          <t>68</t>
+          <t>68&gt;&gt;67</t>
         </is>
       </c>
     </row>
@@ -2391,14 +2391,14 @@
       </c>
       <c r="D84" s="2" t="inlineStr">
         <is>
-          <t>69</t>
+          <t>69&gt;&gt;67</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
         <is>
-          <t>男性E</t>
+          <t>男性E下</t>
         </is>
       </c>
       <c r="B85" s="3" t="inlineStr">
@@ -2414,7 +2414,7 @@
       </c>
       <c r="D85" s="2" t="inlineStr">
         <is>
-          <t>70</t>
+          <t>70&gt;&gt;69</t>
         </is>
       </c>
     </row>
@@ -2436,7 +2436,7 @@
       </c>
       <c r="D86" s="2" t="inlineStr">
         <is>
-          <t>71</t>
+          <t>71&gt;&gt;70</t>
         </is>
       </c>
     </row>
@@ -2465,7 +2465,7 @@
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>男性C</t>
+          <t>男性C下</t>
         </is>
       </c>
       <c r="B88" s="3" t="inlineStr">
@@ -2481,14 +2481,14 @@
       </c>
       <c r="D88" s="2" t="inlineStr">
         <is>
-          <t>73</t>
+          <t>73&gt;&gt;72</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
         <is>
-          <t>女性D</t>
+          <t>女性D下</t>
         </is>
       </c>
       <c r="B89" s="3" t="inlineStr">
@@ -2503,7 +2503,7 @@
       </c>
       <c r="D89" s="2" t="inlineStr">
         <is>
-          <t>74</t>
+          <t>74&gt;&gt;73</t>
         </is>
       </c>
     </row>
@@ -2534,7 +2534,7 @@
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
         <is>
-          <t>男性A</t>
+          <t>男性A下</t>
         </is>
       </c>
       <c r="B91" s="3" t="inlineStr">
@@ -2549,7 +2549,7 @@
       </c>
       <c r="D91" s="2" t="inlineStr">
         <is>
-          <t>76</t>
+          <t>76&gt;&gt;75</t>
         </is>
       </c>
     </row>
@@ -2689,14 +2689,14 @@
       </c>
       <c r="D97" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>2&gt;&gt;1</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>男性C</t>
+          <t>男性C下</t>
         </is>
       </c>
       <c r="B98" s="3" t="inlineStr">
@@ -2711,14 +2711,14 @@
       </c>
       <c r="D98" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>3&gt;&gt;1</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
         <is>
-          <t>女性D</t>
+          <t>女性D下</t>
         </is>
       </c>
       <c r="B99" s="3" t="inlineStr">
@@ -2733,14 +2733,14 @@
       </c>
       <c r="D99" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>4&gt;&gt;1</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>男性E</t>
+          <t>男性E下</t>
         </is>
       </c>
       <c r="B100" s="3" t="inlineStr">
@@ -2756,7 +2756,7 @@
       </c>
       <c r="D100" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>5&gt;&gt;1</t>
         </is>
       </c>
     </row>
@@ -2881,7 +2881,7 @@
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
         <is>
-          <t>男性A</t>
+          <t>男性A下</t>
         </is>
       </c>
       <c r="B106" s="3" t="inlineStr">
@@ -2896,7 +2896,7 @@
       </c>
       <c r="D106" s="2" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>11&gt;&gt;9</t>
         </is>
       </c>
     </row>
@@ -2919,7 +2919,7 @@
       </c>
       <c r="D107" s="2" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>12&gt;&gt;9</t>
         </is>
       </c>
     </row>
@@ -2952,7 +2952,7 @@
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
         <is>
-          <t>女性D</t>
+          <t>女性D下</t>
         </is>
       </c>
       <c r="B109" s="3" t="inlineStr">
@@ -2967,7 +2967,7 @@
       </c>
       <c r="D109" s="2" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>14&gt;&gt;13</t>
         </is>
       </c>
     </row>
@@ -2989,7 +2989,7 @@
       </c>
       <c r="D110" s="2" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>15&gt;&gt;14</t>
         </is>
       </c>
     </row>
@@ -3017,7 +3017,7 @@
       </c>
       <c r="D111" s="2" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>16&gt;&gt;14</t>
         </is>
       </c>
     </row>
@@ -3113,7 +3113,7 @@
       </c>
       <c r="D115" s="2" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>20&gt;&gt;19</t>
         </is>
       </c>
     </row>
@@ -3254,14 +3254,14 @@
       </c>
       <c r="D121" s="2" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>22&gt;&gt;21</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
         <is>
-          <t>男性C</t>
+          <t>男性C下</t>
         </is>
       </c>
       <c r="B122" s="3" t="inlineStr">
@@ -3276,14 +3276,14 @@
       </c>
       <c r="D122" s="2" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>23&gt;&gt;21</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
         <is>
-          <t>女性D</t>
+          <t>女性D下</t>
         </is>
       </c>
       <c r="B123" s="3" t="inlineStr">
@@ -3298,7 +3298,7 @@
       </c>
       <c r="D123" s="2" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>24&gt;&gt;21</t>
         </is>
       </c>
     </row>
@@ -3356,7 +3356,7 @@
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
         <is>
-          <t>女性B</t>
+          <t>女性B下</t>
         </is>
       </c>
       <c r="B126" s="3" t="inlineStr">
@@ -3371,14 +3371,14 @@
       </c>
       <c r="D126" s="2" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>27&gt;&gt;25</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
         <is>
-          <t>男性C</t>
+          <t>男性C下</t>
         </is>
       </c>
       <c r="B127" s="3" t="inlineStr">
@@ -3394,14 +3394,14 @@
       </c>
       <c r="D127" s="2" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>28&gt;&gt;25</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
         <is>
-          <t>女性D</t>
+          <t>女性D下</t>
         </is>
       </c>
       <c r="B128" s="3" t="inlineStr">
@@ -3418,7 +3418,7 @@
       </c>
       <c r="D128" s="2" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>29&gt;&gt;25</t>
         </is>
       </c>
     </row>
@@ -3441,7 +3441,7 @@
       </c>
       <c r="D129" s="2" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>30&gt;&gt;29</t>
         </is>
       </c>
     </row>
@@ -3511,14 +3511,14 @@
       </c>
       <c r="D132" s="2" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>33&gt;&gt;32</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
         <is>
-          <t>女性D</t>
+          <t>女性D下</t>
         </is>
       </c>
       <c r="B133" s="3" t="inlineStr">
@@ -3533,7 +3533,7 @@
       </c>
       <c r="D133" s="2" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>34&gt;&gt;32</t>
         </is>
       </c>
     </row>
@@ -3580,14 +3580,14 @@
       </c>
       <c r="D135" s="2" t="inlineStr">
         <is>
-          <t>36</t>
+          <t>36&gt;&gt;35</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
         <is>
-          <t>女性B</t>
+          <t>女性B下</t>
         </is>
       </c>
       <c r="B136" s="3" t="inlineStr">
@@ -3603,7 +3603,7 @@
       </c>
       <c r="D136" s="2" t="inlineStr">
         <is>
-          <t>37</t>
+          <t>37&gt;&gt;36</t>
         </is>
       </c>
     </row>
@@ -3662,7 +3662,7 @@
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
         <is>
-          <t>男性E</t>
+          <t>男性E下</t>
         </is>
       </c>
       <c r="B139" s="3" t="inlineStr">
@@ -3678,7 +3678,7 @@
       </c>
       <c r="D139" s="2" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>40&gt;&gt;38</t>
         </is>
       </c>
     </row>
@@ -3726,14 +3726,14 @@
       </c>
       <c r="D141" s="2" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>42&gt;&gt;41</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
         <is>
-          <t>男性C</t>
+          <t>男性C下</t>
         </is>
       </c>
       <c r="B142" s="3" t="inlineStr">
@@ -3748,7 +3748,7 @@
       </c>
       <c r="D142" s="2" t="inlineStr">
         <is>
-          <t>43</t>
+          <t>43&gt;&gt;41</t>
         </is>
       </c>
     </row>
@@ -3851,7 +3851,7 @@
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
         <is>
-          <t>男性C</t>
+          <t>男性C下</t>
         </is>
       </c>
       <c r="B147" s="3" t="inlineStr">
@@ -3866,7 +3866,7 @@
       </c>
       <c r="D147" s="2" t="inlineStr">
         <is>
-          <t>48</t>
+          <t>48&gt;&gt;47</t>
         </is>
       </c>
     </row>
@@ -3934,7 +3934,7 @@
       </c>
       <c r="D150" s="2" t="inlineStr">
         <is>
-          <t>51</t>
+          <t>51&gt;&gt;50</t>
         </is>
       </c>
     </row>
@@ -4013,7 +4013,7 @@
       </c>
       <c r="D153" s="2" t="inlineStr">
         <is>
-          <t>54</t>
+          <t>54&gt;&gt;53</t>
         </is>
       </c>
     </row>
@@ -4059,7 +4059,7 @@
       </c>
       <c r="D155" s="2" t="inlineStr">
         <is>
-          <t>56</t>
+          <t>56&gt;&gt;55</t>
         </is>
       </c>
     </row>
@@ -4105,7 +4105,7 @@
       </c>
       <c r="D157" s="2" t="inlineStr">
         <is>
-          <t>58</t>
+          <t>58&gt;&gt;57</t>
         </is>
       </c>
     </row>
@@ -4244,7 +4244,7 @@
       </c>
       <c r="D163" s="2" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>60&gt;&gt;59</t>
         </is>
       </c>
     </row>
@@ -4335,14 +4335,14 @@
       </c>
       <c r="D167" s="2" t="inlineStr">
         <is>
-          <t>64</t>
+          <t>64&gt;&gt;63</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" s="2" t="inlineStr">
         <is>
-          <t>男性E</t>
+          <t>男性E下</t>
         </is>
       </c>
       <c r="B168" s="3" t="inlineStr">
@@ -4357,7 +4357,7 @@
       </c>
       <c r="D168" s="2" t="inlineStr">
         <is>
-          <t>65</t>
+          <t>65&gt;&gt;64</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: 2026-06-20 09:28 (3件)
</commit_message>
<xml_diff>
--- a/01_プロジェクト/YouTube/創作スレ下書き/2026-06-17_平将門の祟り_台本.xlsx
+++ b/01_プロジェクト/YouTube/創作スレ下書き/2026-06-17_平将門の祟り_台本.xlsx
@@ -3017,7 +3017,7 @@
       </c>
       <c r="D111" s="2" t="inlineStr">
         <is>
-          <t>16&gt;&gt;14</t>
+          <t>16</t>
         </is>
       </c>
     </row>
@@ -4013,7 +4013,7 @@
       </c>
       <c r="D153" s="2" t="inlineStr">
         <is>
-          <t>54&gt;&gt;53</t>
+          <t>54</t>
         </is>
       </c>
     </row>
@@ -4244,7 +4244,7 @@
       </c>
       <c r="D163" s="2" t="inlineStr">
         <is>
-          <t>60&gt;&gt;59</t>
+          <t>60</t>
         </is>
       </c>
     </row>

</xml_diff>